<commit_message>
Mandala con más ritmo, línea de montaje y publicación por Metricool
- mandala.html: anillos en contrarrotación con más pasos por bucle y una ola
  que sale del centro cada 6 s; el bucle de 48 s sigue cerrando sin salto
- render_mandala.py: --segundos (vista previa) y --crf
- montar.py: de una obra del catálogo a video.mp4 + miniatura.jpg +
  metadatos.json listos para subir, reanudable paso a paso
- catálogo: OBRA-012 y OBRA-034 cambian de nombre (repetían la duración)
- publicacion-automatizada.md: Make descartado (5 MB por archivo en el
  plan Free); se publica con Metricool tomando el video de Drive

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -1845,12 +1845,12 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Music for Anxiety · Zen Temple · 528 Hz · Ten Minutes · 10 Minutes</t>
+          <t>Music for Anxiety · Zen Temple · 528 Hz · A Brief Pause · 10 Minutes</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Música para momentos de ansiedad · Templo zen · 528 Hz · Diez minutos · 10 minutos</t>
+          <t>Música para momentos de ansiedad · Templo zen · 528 Hz · Pausa breve · 10 minutos</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Ten Minutes · 10 Minutes
+          <t>A Brief Pause · 10 Minutes
 To accompany a pause when your mind won't stop.
 Ambience: zen temple.
 Composed around a root of 528 Hz, in just intonation, shin mode.
@@ -1877,7 +1877,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Diez minutos · 10 minutos
+          <t>Pausa breve · 10 minutos
 Para acompañar un momento de pausa cuando la cabeza no para.
 Ambiente: templo zen.
 Compuesta con raíz en 528 Hz, en entonación justa, modo shin.
@@ -1918,19 +1918,19 @@
         </is>
       </c>
       <c r="P13" s="2" t="n">
-        <v>207307</v>
+        <v>43734</v>
       </c>
       <c r="Q13" s="2" t="n">
         <v>10</v>
       </c>
       <c r="R13" s="3" t="inlineStr">
         <is>
-          <t>python3 03-composicion/compositor.py --minutos 10 --raiz 528 --modo shin --semilla 207307 --caracter sin-cuenco</t>
+          <t>python3 03-composicion/compositor.py --minutos 10 --raiz 528 --modo shin --semilla 43734 --caracter sin-cuenco</t>
         </is>
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 640 audio/OBRA-012_capa.wav --semilla 207307 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-012_528_shin.wav audio/OBRA-012_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-012_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 640 audio/OBRA-012_capa.wav --semilla 43734 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-012_528_shin.wav audio/OBRA-012_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-012_capa.wav</t>
         </is>
       </c>
       <c r="T13" s="4" t="inlineStr">
@@ -4243,12 +4243,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Focus Music · Ocean and Birds · 528 Hz · Three Hours · 3 Hours</t>
+          <t>Focus Music · Ocean and Birds · 528 Hz · Deep Work · 3 Hours</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Música para concentrarse · Mar y pájaros · 528 Hz · Tres horas · 3 horas</t>
+          <t>Música para concentrarse · Mar y pájaros · 528 Hz · Trabajo profundo · 3 horas</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -4263,7 +4263,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Three Hours · 3 Hours
+          <t>Deep Work · 3 Hours
 To accompany work or study.
 Ambience: ocean and birds.
 Composed around a root of 264 Hz, the low octave of 528 Hz, in just intonation, yo mode.
@@ -4275,7 +4275,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Tres horas · 3 horas
+          <t>Trabajo profundo · 3 horas
 Para acompañar el trabajo o el estudio.
 Ambiente: mar y pájaros.
 Compuesta con raíz en 264 Hz, la octava grave de 528 Hz, en entonación justa, modo yo.
@@ -4316,19 +4316,19 @@
         </is>
       </c>
       <c r="P35" s="2" t="n">
-        <v>935486</v>
+        <v>249239</v>
       </c>
       <c r="Q35" s="2" t="n">
         <v>180</v>
       </c>
       <c r="R35" s="3" t="inlineStr">
         <is>
-          <t>python3 03-composicion/compositor.py --minutos 180 --raiz 528 --modo yo --semilla 935486 --caracter sin-cuenco --registro grave</t>
+          <t>python3 03-composicion/compositor.py --minutos 180 --raiz 528 --modo yo --semilla 249239 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
       <c r="S35" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 10840 audio/OBRA-034_capa.wav --semilla 935486 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-034_528_yo.wav audio/OBRA-034_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-034_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 10840 audio/OBRA-034_capa.wav --semilla 249239 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-034_528_yo.wav audio/OBRA-034_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-034_capa.wav</t>
         </is>
       </c>
       <c r="T35" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Descripciones sin marcador de capítulos, etiquetas en inglés, mandala a CRF 28
- La descripción terminaba en "Chapters: 00:00 [fill in after editing]": ahora
  cierra con la invitación a suscribirse y los hashtags
- Etiquetas en inglés por intención y ambiente, con la palabra clave en
  español al final
- render_mandala.py: CRF 28 con -tune animation por defecto; el video pesa
  la mitad con la misma imagen (SSIM 0,988 frente a CRF 24)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -672,8 +672,9 @@
 Composed around a root of 216 Hz, the low octave of 432 Hz, in just intonation, shin mode.
 Breathing cycle: from 4.5 down to 3.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -684,8 +685,9 @@
 Compuesta con raíz en 216 Hz, la octava grave de 432 Hz, en entonación justa, modo shin.
 Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -700,7 +702,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>432 hz, música 432 hz, música para dormir, sleep music, dormir, shin, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, singing bowls, just intonation</t>
+          <t>sleep music, 432 hz, 432 hz music, deep sleep, insomnia, ocean waves, sea sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para dormir</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr"/>
@@ -781,8 +783,9 @@
 Composed around a root of 264 Hz, the low octave of 528 Hz, in just intonation, kumoi mode.
 Breathing cycle: from 4.5 down to 3.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -793,8 +796,9 @@
 Compuesta con raíz en 264 Hz, la octava grave de 528 Hz, en entonación justa, modo kumoi.
 Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -809,7 +813,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>528 hz, música 528 hz, música para dormir, sleep music, dormir, kumoi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, singing bowls, just intonation</t>
+          <t>sleep music, 528 hz, 528 hz music, deep sleep, insomnia, ocean waves, sea sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para dormir</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr"/>
@@ -890,8 +894,9 @@
 Composed around a root of 198 Hz, the low octave of 396 Hz, in just intonation, kumoi mode.
 Breathing cycle: from 4.5 down to 3.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #396Hz</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -902,8 +907,9 @@
 Compuesta con raíz en 198 Hz, la octava grave de 396 Hz, en entonación justa, modo kumoi.
 Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #396Hz</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -918,7 +924,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>396 hz, música 396 hz, música para dormir, sleep music, dormir, kumoi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, singing bowls, just intonation</t>
+          <t>sleep music, 396 hz, 396 hz music, deep sleep, insomnia, ocean waves, sea sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para dormir</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr"/>
@@ -999,8 +1005,9 @@
 Composed around a root of 264 Hz, the low octave of 528 Hz, in just intonation, shin mode.
 Breathing cycle: from 4.5 down to 3.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1011,8 +1018,9 @@
 Compuesta con raíz en 264 Hz, la octava grave de 528 Hz, en entonación justa, modo shin.
 Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1027,7 +1035,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>528 hz, música 528 hz, música para dormir, sleep music, dormir, shin, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, singing bowls, just intonation</t>
+          <t>sleep music, 528 hz, 528 hz music, deep sleep, insomnia, ocean waves, sea sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para dormir</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr"/>
@@ -1108,8 +1116,9 @@
 Composed around a root of 216 Hz, the low octave of 432 Hz, in just intonation, kumoi mode.
 Breathing cycle: from 4.5 down to 3.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1120,8 +1129,9 @@
 Compuesta con raíz en 216 Hz, la octava grave de 432 Hz, en entonación justa, modo kumoi.
 Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1136,7 +1146,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>432 hz, música 432 hz, música para dormir, sleep music, dormir, kumoi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, singing bowls, just intonation</t>
+          <t>sleep music, 432 hz, 432 hz music, deep sleep, insomnia, ocean waves, sea sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para dormir</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr"/>
@@ -1217,8 +1227,9 @@
 Composed around a root of 208.5 Hz, the low octave of 417 Hz, in just intonation, kumoi mode.
 Breathing cycle: from 4.5 down to 3.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #417Hz</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1229,8 +1240,9 @@
 Compuesta con raíz en 208.5 Hz, la octava grave de 417 Hz, en entonación justa, modo kumoi.
 Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #417Hz</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -1245,7 +1257,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>417 hz, música 417 hz, música para dormir, sleep music, dormir, kumoi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, singing bowls, just intonation</t>
+          <t>sleep music, 417 hz, 417 hz music, deep sleep, insomnia, ocean waves, sea sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para dormir</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr"/>
@@ -1326,8 +1338,9 @@
 Composed around a root of 198 Hz, the low octave of 396 Hz, in just intonation, shin mode.
 Breathing cycle: from 4.5 down to 3.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #396Hz</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1338,8 +1351,9 @@
 Compuesta con raíz en 198 Hz, la octava grave de 396 Hz, en entonación justa, modo shin.
 Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #396Hz</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1354,7 +1368,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>396 hz, música 396 hz, música para dormir, sleep music, dormir, shin, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, singing bowls, just intonation</t>
+          <t>sleep music, 396 hz, 396 hz music, deep sleep, insomnia, ocean waves, sea sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para dormir</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr"/>
@@ -1435,8 +1449,9 @@
 Composed around a root of 216 Hz, the low octave of 432 Hz, in just intonation, kumoi mode.
 Breathing cycle: from 4.5 down to 3.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1447,8 +1462,9 @@
 Compuesta con raíz en 216 Hz, la octava grave de 432 Hz, en entonación justa, modo kumoi.
 Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#SleepMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1463,7 +1479,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>432 hz, música 432 hz, música para dormir, sleep music, dormir, kumoi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, singing bowls, just intonation</t>
+          <t>sleep music, 432 hz, 432 hz music, deep sleep, insomnia, ocean waves, sea sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para dormir</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr"/>
@@ -1544,8 +1560,9 @@
 Composed around a root of 396 Hz, in just intonation, kumoi mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #396Hz</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1556,8 +1573,9 @@
 Compuesta con raíz en 396 Hz, en entonación justa, modo kumoi.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #396Hz</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1572,7 +1590,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>396 hz, música 396 hz, música para momentos de ansiedad, music for anxiety, ansiedad, kumoi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music for anxiety, 396 hz, 396 hz music, anxiety relief, stress relief, calming music, ocean waves, birdsong, nature sounds, relaxing music, meditation music, ambient music, just intonation, original composition, Rin, música para momentos de ansiedad</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr"/>
@@ -1653,8 +1671,9 @@
 Composed around a root of 432 Hz, in just intonation, hirajoshi mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1665,8 +1684,9 @@
 Compuesta con raíz en 432 Hz, en entonación justa, modo hirajoshi.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1681,7 +1701,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>432 hz, música 432 hz, música para momentos de ansiedad, music for anxiety, ansiedad, hirajoshi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music for anxiety, 432 hz, 432 hz music, anxiety relief, stress relief, calming music, zen temple, temple bells, wind chimes, relaxing music, meditation music, ambient music, just intonation, original composition, Rin, música para momentos de ansiedad</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr"/>
@@ -1762,8 +1782,9 @@
 Composed around a root of 528 Hz, in just intonation, hirajoshi mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1774,8 +1795,9 @@
 Compuesta con raíz en 528 Hz, en entonación justa, modo hirajoshi.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1790,7 +1812,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>528 hz, música 528 hz, música para momentos de ansiedad, music for anxiety, ansiedad, hirajoshi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music for anxiety, 528 hz, 528 hz music, anxiety relief, stress relief, calming music, ocean waves, birdsong, nature sounds, relaxing music, meditation music, ambient music, just intonation, original composition, Rin, música para momentos de ansiedad</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr"/>
@@ -1871,8 +1893,9 @@
 Composed around a root of 528 Hz, in just intonation, shin mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1883,8 +1906,9 @@
 Compuesta con raíz en 528 Hz, en entonación justa, modo shin.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1899,7 +1923,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>528 hz, música 528 hz, música para momentos de ansiedad, music for anxiety, ansiedad, shin, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music for anxiety, 528 hz, 528 hz music, anxiety relief, stress relief, calming music, zen temple, temple bells, wind chimes, relaxing music, meditation music, ambient music, just intonation, original composition, Rin, música para momentos de ansiedad</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr"/>
@@ -1980,8 +2004,9 @@
 Composed around a root of 432 Hz, in just intonation, hirajoshi mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1992,8 +2017,9 @@
 Compuesta con raíz en 432 Hz, en entonación justa, modo hirajoshi.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -2008,7 +2034,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>432 hz, música 432 hz, música para momentos de ansiedad, music for anxiety, ansiedad, hirajoshi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music for anxiety, 432 hz, 432 hz music, anxiety relief, stress relief, calming music, ocean waves, birdsong, nature sounds, relaxing music, meditation music, ambient music, just intonation, original composition, Rin, música para momentos de ansiedad</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr"/>
@@ -2089,8 +2115,9 @@
 Composed around a root of 528 Hz, in just intonation, yo mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -2101,8 +2128,9 @@
 Compuesta con raíz en 528 Hz, en entonación justa, modo yo.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -2117,7 +2145,7 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>528 hz, música 528 hz, música para momentos de ansiedad, music for anxiety, ansiedad, yo, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music for anxiety, 528 hz, 528 hz music, anxiety relief, stress relief, calming music, zen temple, temple bells, wind chimes, relaxing music, meditation music, ambient music, just intonation, original composition, Rin, música para momentos de ansiedad</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr"/>
@@ -2198,8 +2226,9 @@
 Composed around a root of 639 Hz, in just intonation, yo mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #639Hz</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2210,8 +2239,9 @@
 Compuesta con raíz en 639 Hz, en entonación justa, modo yo.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #639Hz</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -2226,7 +2256,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>639 hz, música 639 hz, música para momentos de ansiedad, music for anxiety, ansiedad, yo, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music for anxiety, 639 hz, 639 hz music, anxiety relief, stress relief, calming music, ocean waves, birdsong, nature sounds, relaxing music, meditation music, ambient music, just intonation, original composition, Rin, música para momentos de ansiedad</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr"/>
@@ -2307,8 +2337,9 @@
 Composed around a root of 417 Hz, in just intonation, kumoi mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #417Hz</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -2319,8 +2350,9 @@
 Compuesta con raíz en 417 Hz, en entonación justa, modo kumoi.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #417Hz</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -2335,7 +2367,7 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>417 hz, música 417 hz, música para momentos de ansiedad, music for anxiety, ansiedad, kumoi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music for anxiety, 417 hz, 417 hz music, anxiety relief, stress relief, calming music, rain sounds, rain on leaves, shamanic drum, relaxing music, meditation music, ambient music, just intonation, original composition, Rin, música para momentos de ansiedad</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr"/>
@@ -2416,8 +2448,9 @@
 Composed around a root of 417 Hz, in just intonation, hirajoshi mode.
 Breathing cycle: from 5.5 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #417Hz</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2428,8 +2461,9 @@
 Compuesta con raíz en 417 Hz, en entonación justa, modo hirajoshi.
 Ciclo respiratorio: de 5.5 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #417Hz</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -2444,7 +2478,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>417 hz, música 417 hz, música para meditar, meditation music, meditar, hirajoshi, música relajante, meditación, relajación, entonación justa, composición original, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>meditation music, 417 hz, 417 hz music, mindfulness, zen music, yoga music, zen temple, temple bells, wind chimes, relaxing music, calming music, ambient music, just intonation, original composition, Rin, música para meditar</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr"/>
@@ -2525,8 +2559,9 @@
 Composed around a root of 528 Hz, in just intonation, hirajoshi mode.
 Breathing cycle: from 5.5 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -2537,8 +2572,9 @@
 Compuesta con raíz en 528 Hz, en entonación justa, modo hirajoshi.
 Ciclo respiratorio: de 5.5 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -2553,7 +2589,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>528 hz, música 528 hz, música para meditar, meditation music, meditar, hirajoshi, música relajante, meditación, relajación, entonación justa, composición original, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>meditation music, 528 hz, 528 hz music, mindfulness, zen music, yoga music, zen temple, temple bells, wind chimes, relaxing music, calming music, ambient music, just intonation, original composition, Rin, música para meditar</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr"/>
@@ -2634,8 +2670,9 @@
 Composed around a root of 432 Hz, in just intonation, shin mode.
 Breathing cycle: from 5.5 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2646,8 +2683,9 @@
 Compuesta con raíz en 432 Hz, en entonación justa, modo shin.
 Ciclo respiratorio: de 5.5 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -2662,7 +2700,7 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>432 hz, música 432 hz, música para meditar, meditation music, meditar, shin, música relajante, meditación, relajación, entonación justa, composición original, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>meditation music, 432 hz, 432 hz music, mindfulness, zen music, yoga music, zen temple, temple bells, wind chimes, relaxing music, calming music, ambient music, just intonation, original composition, Rin, música para meditar</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr"/>
@@ -2743,8 +2781,9 @@
 Composed around a root of 528 Hz, in just intonation, shin mode.
 Breathing cycle: from 5.5 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -2755,8 +2794,9 @@
 Compuesta con raíz en 528 Hz, en entonación justa, modo shin.
 Ciclo respiratorio: de 5.5 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -2771,7 +2811,7 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>528 hz, música 528 hz, música para meditar, meditation music, meditar, shin, música relajante, meditación, relajación, entonación justa, composición original, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>meditation music, 528 hz, 528 hz music, mindfulness, zen music, yoga music, rain sounds, rain on leaves, shamanic drum, relaxing music, calming music, ambient music, just intonation, original composition, Rin, música para meditar</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr"/>
@@ -2852,8 +2892,9 @@
 Composed around a root of 396 Hz, in just intonation, kumoi mode.
 Breathing cycle: from 5.5 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #396Hz</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2864,8 +2905,9 @@
 Compuesta con raíz en 396 Hz, en entonación justa, modo kumoi.
 Ciclo respiratorio: de 5.5 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #396Hz</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -2880,7 +2922,7 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>396 hz, música 396 hz, música para meditar, meditation music, meditar, kumoi, música relajante, meditación, relajación, entonación justa, composición original, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>meditation music, 396 hz, 396 hz music, mindfulness, zen music, yoga music, zen temple, temple bells, wind chimes, relaxing music, calming music, ambient music, just intonation, original composition, Rin, música para meditar</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr"/>
@@ -2961,8 +3003,9 @@
 Composed around a root of 639 Hz, in just intonation, yo mode.
 Breathing cycle: from 5.5 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #639Hz</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -2973,8 +3016,9 @@
 Compuesta con raíz en 639 Hz, en entonación justa, modo yo.
 Ciclo respiratorio: de 5.5 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #639Hz</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2989,7 +3033,7 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>639 hz, música 639 hz, música para meditar, meditation music, meditar, yo, música relajante, meditación, relajación, entonación justa, composición original, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>meditation music, 639 hz, 639 hz music, mindfulness, zen music, yoga music, zen temple, temple bells, wind chimes, relaxing music, calming music, ambient music, just intonation, original composition, Rin, música para meditar</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr"/>
@@ -3070,8 +3114,9 @@
 Composed around a root of 528 Hz, in just intonation, shin mode.
 Breathing cycle: from 5.5 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -3082,8 +3127,9 @@
 Compuesta con raíz en 528 Hz, en entonación justa, modo shin.
 Ciclo respiratorio: de 5.5 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -3098,7 +3144,7 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>528 hz, música 528 hz, música para meditar, meditation music, meditar, shin, música relajante, meditación, relajación, entonación justa, composición original, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>meditation music, 528 hz, 528 hz music, mindfulness, zen music, yoga music, zen temple, temple bells, wind chimes, relaxing music, calming music, ambient music, just intonation, original composition, Rin, música para meditar</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr"/>
@@ -3179,8 +3225,9 @@
 Composed around a root of 432 Hz, in just intonation, kumoi mode.
 Breathing cycle: from 5.5 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -3191,8 +3238,9 @@
 Compuesta con raíz en 432 Hz, en entonación justa, modo kumoi.
 Ciclo respiratorio: de 5.5 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#MeditationMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -3207,7 +3255,7 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>432 hz, música 432 hz, música para meditar, meditation music, meditar, kumoi, música relajante, meditación, relajación, entonación justa, composición original, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>meditation music, 432 hz, 432 hz music, mindfulness, zen music, yoga music, rain sounds, rain on leaves, shamanic drum, relaxing music, calming music, ambient music, just intonation, original composition, Rin, música para meditar</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr"/>
@@ -3288,8 +3336,9 @@
 Composed around a root of 528 Hz, in just intonation, hirajoshi mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -3300,8 +3349,9 @@
 Compuesta con raíz en 528 Hz, en entonación justa, modo hirajoshi.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -3316,7 +3366,7 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>528 hz, música 528 hz, música para soltar tensión, music to release tension, soltar, hirajoshi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music to release tension, 528 hz, 528 hz music, stress relief, let go, healing music, ocean waves, birdsong, nature sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para soltar tensión</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr"/>
@@ -3397,8 +3447,9 @@
 Composed around a root of 432 Hz, in just intonation, kumoi mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -3409,8 +3460,9 @@
 Compuesta con raíz en 432 Hz, en entonación justa, modo kumoi.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -3425,7 +3477,7 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>432 hz, música 432 hz, música para soltar tensión, music to release tension, soltar, kumoi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music to release tension, 432 hz, 432 hz music, stress relief, let go, healing music, ocean waves, sea sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para soltar tensión</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr"/>
@@ -3506,8 +3558,9 @@
 Composed around a root of 396 Hz, in just intonation, kumoi mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #396Hz</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3518,8 +3571,9 @@
 Compuesta con raíz en 396 Hz, en entonación justa, modo kumoi.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #396Hz</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -3534,7 +3588,7 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>396 hz, música 396 hz, música para soltar tensión, music to release tension, soltar, kumoi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music to release tension, 396 hz, 396 hz music, stress relief, let go, healing music, rain sounds, rain on leaves, shamanic drum, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para soltar tensión</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr"/>
@@ -3615,8 +3669,9 @@
 Composed around a root of 417 Hz, in just intonation, hirajoshi mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #417Hz</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -3627,8 +3682,9 @@
 Compuesta con raíz en 417 Hz, en entonación justa, modo hirajoshi.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #417Hz</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -3643,7 +3699,7 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>417 hz, música 417 hz, música para soltar tensión, music to release tension, soltar, hirajoshi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music to release tension, 417 hz, 417 hz music, stress relief, let go, healing music, zen temple, temple bells, wind chimes, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para soltar tensión</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr"/>
@@ -3724,8 +3780,9 @@
 Composed around a root of 639 Hz, in just intonation, yo mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #639Hz</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3736,8 +3793,9 @@
 Compuesta con raíz en 639 Hz, en entonación justa, modo yo.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #639Hz</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3752,7 +3810,7 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>639 hz, música 639 hz, música para soltar tensión, music to release tension, soltar, yo, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music to release tension, 639 hz, 639 hz music, stress relief, let go, healing music, rainforest sounds, birdsong, nature sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para soltar tensión</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr"/>
@@ -3833,8 +3891,9 @@
 Composed around a root of 741 Hz, in just intonation, yo mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #741Hz</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -3845,8 +3904,9 @@
 Compuesta con raíz en 741 Hz, en entonación justa, modo yo.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #741Hz</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -3861,7 +3921,7 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>741 hz, música 741 hz, música para soltar tensión, music to release tension, soltar, yo, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music to release tension, 741 hz, 741 hz music, stress relief, let go, healing music, ocean waves, birdsong, nature sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para soltar tensión</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr"/>
@@ -3942,8 +4002,9 @@
 Composed around a root of 852 Hz, in just intonation, hirajoshi mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #852Hz</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -3954,8 +4015,9 @@
 Compuesta con raíz en 852 Hz, en entonación justa, modo hirajoshi.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #852Hz</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -3970,7 +4032,7 @@
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>852 hz, música 852 hz, música para soltar tensión, music to release tension, soltar, hirajoshi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music to release tension, 852 hz, 852 hz music, stress relief, let go, healing music, zen temple, temple bells, wind chimes, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para soltar tensión</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr"/>
@@ -4051,8 +4113,9 @@
 Composed around a root of 528 Hz, in just intonation, hirajoshi mode.
 Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -4063,8 +4126,9 @@
 Compuesta con raíz en 528 Hz, en entonación justa, modo hirajoshi.
 Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#RelaxingMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -4079,7 +4143,7 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>528 hz, música 528 hz, música para soltar tensión, music to release tension, soltar, hirajoshi, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>music to release tension, 528 hz, 528 hz music, stress relief, let go, healing music, ocean waves, birdsong, nature sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para soltar tensión</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr"/>
@@ -4160,8 +4224,9 @@
 Composed around a root of 319.5 Hz, the low octave of 639 Hz, in just intonation, yo mode.
 Breathing cycle: from 6.0 down to 5.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #639Hz</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -4172,8 +4237,9 @@
 Compuesta con raíz en 319.5 Hz, la octava grave de 639 Hz, en entonación justa, modo yo.
 Ciclo respiratorio: de 6.0 a 5.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #639Hz</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -4188,7 +4254,7 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>639 hz, música 639 hz, música para concentrarse, focus music, concentración, yo, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>focus music, 639 hz, 639 hz music, study music, deep focus, work music, rainforest sounds, birdsong, nature sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para concentrarse</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr"/>
@@ -4269,8 +4335,9 @@
 Composed around a root of 264 Hz, the low octave of 528 Hz, in just intonation, yo mode.
 Breathing cycle: from 6.0 down to 5.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -4281,8 +4348,9 @@
 Compuesta con raíz en 264 Hz, la octava grave de 528 Hz, en entonación justa, modo yo.
 Ciclo respiratorio: de 6.0 a 5.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -4297,7 +4365,7 @@
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>528 hz, música 528 hz, música para concentrarse, focus music, concentración, yo, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>focus music, 528 hz, 528 hz music, study music, deep focus, work music, ocean waves, birdsong, nature sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para concentrarse</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr"/>
@@ -4378,8 +4446,9 @@
 Composed around a root of 370.5 Hz, the low octave of 741 Hz, in just intonation, yo mode.
 Breathing cycle: from 6.0 down to 5.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #741Hz</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -4390,8 +4459,9 @@
 Compuesta con raíz en 370.5 Hz, la octava grave de 741 Hz, en entonación justa, modo yo.
 Ciclo respiratorio: de 6.0 a 5.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #741Hz</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -4406,7 +4476,7 @@
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>741 hz, música 741 hz, música para concentrarse, focus music, concentración, yo, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>focus music, 741 hz, 741 hz music, study music, deep focus, work music, rainforest sounds, birdsong, nature sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para concentrarse</t>
         </is>
       </c>
       <c r="K36" s="4" t="inlineStr"/>
@@ -4487,8 +4557,9 @@
 Composed around a root of 426 Hz, the low octave of 852 Hz, in just intonation, yo mode.
 Breathing cycle: from 6.0 down to 5.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #852Hz</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -4499,8 +4570,9 @@
 Compuesta con raíz en 426 Hz, la octava grave de 852 Hz, en entonación justa, modo yo.
 Ciclo respiratorio: de 6.0 a 5.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #852Hz</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -4515,7 +4587,7 @@
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>852 hz, música 852 hz, música para concentrarse, focus music, concentración, yo, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>focus music, 852 hz, 852 hz music, study music, deep focus, work music, ocean waves, birdsong, nature sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para concentrarse</t>
         </is>
       </c>
       <c r="K37" s="4" t="inlineStr"/>
@@ -4596,8 +4668,9 @@
 Composed around a root of 216 Hz, the low octave of 432 Hz, in just intonation, yo mode.
 Breathing cycle: from 6.0 down to 5.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4608,8 +4681,9 @@
 Compuesta con raíz en 216 Hz, la octava grave de 432 Hz, en entonación justa, modo yo.
 Ciclo respiratorio: de 6.0 a 5.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #432Hz</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -4624,7 +4698,7 @@
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>432 hz, música 432 hz, música para concentrarse, focus music, concentración, yo, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>focus music, 432 hz, 432 hz music, study music, deep focus, work music, rainforest sounds, birdsong, nature sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para concentrarse</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr"/>
@@ -4705,8 +4779,9 @@
 Composed around a root of 264 Hz, the low octave of 528 Hz, in just intonation, shin mode.
 Breathing cycle: from 6.0 down to 5.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -4717,8 +4792,9 @@
 Compuesta con raíz en 264 Hz, la octava grave de 528 Hz, en entonación justa, modo shin.
 Ciclo respiratorio: de 6.0 a 5.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #528Hz</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -4733,7 +4809,7 @@
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>528 hz, música 528 hz, música para concentrarse, focus music, concentración, shin, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>focus music, 528 hz, 528 hz music, study music, deep focus, work music, ocean waves, sea sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para concentrarse</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr"/>
@@ -4814,8 +4890,9 @@
 Composed around a root of 319.5 Hz, the low octave of 639 Hz, in just intonation, yo mode.
 Breathing cycle: from 6.0 down to 5.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #639Hz</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4826,8 +4903,9 @@
 Compuesta con raíz en 319.5 Hz, la octava grave de 639 Hz, en entonación justa, modo yo.
 Ciclo respiratorio: de 6.0 a 5.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #639Hz</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -4842,7 +4920,7 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>639 hz, música 639 hz, música para concentrarse, focus music, concentración, yo, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>focus music, 639 hz, 639 hz music, study music, deep focus, work music, rainforest sounds, birdsong, nature sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para concentrarse</t>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr"/>
@@ -4923,8 +5001,9 @@
 Composed around a root of 370.5 Hz, the low octave of 741 Hz, in just intonation, yo mode.
 Breathing cycle: from 6.0 down to 5.5 breaths per minute, 40 % inhale / 60 % exhale.
 Original composition, synthesized from scratch, ambience included. No third-party samples.
-Chapters:
-00:00 [fill in after editing]</t>
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #741Hz</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -4935,8 +5014,9 @@
 Compuesta con raíz en 370.5 Hz, la octava grave de 741 Hz, en entonación justa, modo yo.
 Ciclo respiratorio: de 6.0 a 5.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
-Capítulos:
-00:00 [completar tras el montaje]</t>
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#FocusMusic #Meditation #741Hz</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -4951,7 +5031,7 @@
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>741 hz, música 741 hz, música para concentrarse, focus music, concentración, yo, música relajante, meditación, relajación, entonación justa, composición original, meditation music, relaxing music, sleep music, singing bowls, just intonation</t>
+          <t>focus music, 741 hz, 741 hz music, study music, deep focus, work music, ocean waves, birdsong, nature sounds, relaxing music, meditation music, calming music, ambient music, just intonation, original composition, Rin, música para concentrarse</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
OBRA-012 publicada; lo publicado se guarda en publicadas.csv
El catálogo se regenera desde cero, así que la URL y la fecha de cada video
publicado viven en un archivo aparte que generar_catalogo.py vuelve a aplicar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -1927,7 +1927,11 @@
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr"/>
-      <c r="L13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>https://youtu.be/-ywSggvwt2E</t>
+        </is>
+      </c>
       <c r="M13" s="2" t="n">
         <v>528</v>
       </c>
@@ -1959,10 +1963,14 @@
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="U13" s="4" t="inlineStr"/>
+          <t>publicada</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="V13" s="4" t="inlineStr"/>
       <c r="W13" s="4" t="inlineStr"/>
       <c r="X13" s="5">

</xml_diff>

<commit_message>
Subida automática de Shorts con Make
- hacer_short.py: además del Short, short-<n>-web.mp4 en HEVC bajo 5 MB (el
  límite de archivo del plan gratuito de Make)
- cola_shorts.py: la cola de subida para la hoja Rin_Shorts, intercalando obras
- shorts_catalogo.py: la descripción de YouTube incluye el enlace del video largo
- hashtags de los videos largos en minúscula
- shorts.md: el escenario «Rin - Shorts a YouTube»

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -676,7 +676,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #432Hz</t>
+#sleepmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -689,7 +689,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #432Hz</t>
+#sleepmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>#SleepMusic #Meditation #432Hz</t>
+          <t>#sleepmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -787,7 +787,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #528Hz</t>
+#sleepmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -800,7 +800,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #528Hz</t>
+#sleepmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>#SleepMusic #Meditation #528Hz</t>
+          <t>#sleepmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -898,7 +898,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #396Hz</t>
+#sleepmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -911,7 +911,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #396Hz</t>
+#sleepmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>#SleepMusic #Meditation #396Hz</t>
+          <t>#sleepmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -1009,7 +1009,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #528Hz</t>
+#sleepmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1022,7 +1022,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #528Hz</t>
+#sleepmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>#SleepMusic #Meditation #528Hz</t>
+          <t>#sleepmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -1120,7 +1120,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #432Hz</t>
+#sleepmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1133,7 +1133,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #432Hz</t>
+#sleepmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>#SleepMusic #Meditation #432Hz</t>
+          <t>#sleepmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -1231,7 +1231,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #417Hz</t>
+#sleepmusic #meditation #417hz</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1244,7 +1244,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #417Hz</t>
+#sleepmusic #meditation #417hz</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>#SleepMusic #Meditation #417Hz</t>
+          <t>#sleepmusic #meditation #417hz</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -1342,7 +1342,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #396Hz</t>
+#sleepmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1355,7 +1355,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #396Hz</t>
+#sleepmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>#SleepMusic #Meditation #396Hz</t>
+          <t>#sleepmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
@@ -1453,7 +1453,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #432Hz</t>
+#sleepmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1466,7 +1466,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#SleepMusic #Meditation #432Hz</t>
+#sleepmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>#SleepMusic #Meditation #432Hz</t>
+          <t>#sleepmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -1564,7 +1564,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #396Hz</t>
+#relaxingmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1577,7 +1577,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #396Hz</t>
+#relaxingmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #396Hz</t>
+          <t>#relaxingmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
@@ -1675,7 +1675,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #432Hz</t>
+#relaxingmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1688,7 +1688,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #432Hz</t>
+#relaxingmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #432Hz</t>
+          <t>#relaxingmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
@@ -1786,7 +1786,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #528Hz</t>
+#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1799,7 +1799,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #528Hz</t>
+#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #528Hz</t>
+          <t>#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
@@ -1897,7 +1897,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #528Hz</t>
+#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1910,7 +1910,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #528Hz</t>
+#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #528Hz</t>
+          <t>#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
@@ -2016,7 +2016,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #432Hz</t>
+#relaxingmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -2029,7 +2029,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #432Hz</t>
+#relaxingmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #432Hz</t>
+          <t>#relaxingmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
@@ -2127,7 +2127,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #528Hz</t>
+#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -2140,7 +2140,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #528Hz</t>
+#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #528Hz</t>
+          <t>#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
@@ -2238,7 +2238,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #639Hz</t>
+#relaxingmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2251,7 +2251,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #639Hz</t>
+#relaxingmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #639Hz</t>
+          <t>#relaxingmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
@@ -2357,7 +2357,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #417Hz</t>
+#relaxingmusic #meditation #417hz</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -2370,7 +2370,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #417Hz</t>
+#relaxingmusic #meditation #417hz</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -2380,7 +2380,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #417Hz</t>
+          <t>#relaxingmusic #meditation #417hz</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
@@ -2468,7 +2468,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #417Hz</t>
+#meditationmusic #meditation #417hz</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2481,7 +2481,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #417Hz</t>
+#meditationmusic #meditation #417hz</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>#MeditationMusic #Meditation #417Hz</t>
+          <t>#meditationmusic #meditation #417hz</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
@@ -2579,7 +2579,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #528Hz</t>
+#meditationmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -2592,7 +2592,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #528Hz</t>
+#meditationmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>#MeditationMusic #Meditation #528Hz</t>
+          <t>#meditationmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
@@ -2690,7 +2690,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #432Hz</t>
+#meditationmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2703,7 +2703,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #432Hz</t>
+#meditationmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>#MeditationMusic #Meditation #432Hz</t>
+          <t>#meditationmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
@@ -2801,7 +2801,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #528Hz</t>
+#meditationmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -2814,7 +2814,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #528Hz</t>
+#meditationmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -2824,7 +2824,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>#MeditationMusic #Meditation #528Hz</t>
+          <t>#meditationmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -2912,7 +2912,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #396Hz</t>
+#meditationmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2925,7 +2925,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #396Hz</t>
+#meditationmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>#MeditationMusic #Meditation #396Hz</t>
+          <t>#meditationmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
@@ -3023,7 +3023,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #639Hz</t>
+#meditationmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -3036,7 +3036,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #639Hz</t>
+#meditationmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>#MeditationMusic #Meditation #639Hz</t>
+          <t>#meditationmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
@@ -3134,7 +3134,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #528Hz</t>
+#meditationmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -3147,7 +3147,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #528Hz</t>
+#meditationmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>#MeditationMusic #Meditation #528Hz</t>
+          <t>#meditationmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
@@ -3245,7 +3245,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #432Hz</t>
+#meditationmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -3258,7 +3258,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#MeditationMusic #Meditation #432Hz</t>
+#meditationmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -3268,7 +3268,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>#MeditationMusic #Meditation #432Hz</t>
+          <t>#meditationmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
@@ -3356,7 +3356,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #528Hz</t>
+#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -3369,7 +3369,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #528Hz</t>
+#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #528Hz</t>
+          <t>#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
@@ -3467,7 +3467,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #432Hz</t>
+#relaxingmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -3480,7 +3480,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #432Hz</t>
+#relaxingmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -3490,7 +3490,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #432Hz</t>
+          <t>#relaxingmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
@@ -3578,7 +3578,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #396Hz</t>
+#relaxingmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3591,7 +3591,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #396Hz</t>
+#relaxingmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -3601,7 +3601,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #396Hz</t>
+          <t>#relaxingmusic #meditation #396hz</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
@@ -3689,7 +3689,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #417Hz</t>
+#relaxingmusic #meditation #417hz</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -3702,7 +3702,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #417Hz</t>
+#relaxingmusic #meditation #417hz</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -3712,7 +3712,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #417Hz</t>
+          <t>#relaxingmusic #meditation #417hz</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
@@ -3800,7 +3800,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #639Hz</t>
+#relaxingmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3813,7 +3813,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #639Hz</t>
+#relaxingmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3823,7 +3823,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #639Hz</t>
+          <t>#relaxingmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
@@ -3911,7 +3911,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #741Hz</t>
+#relaxingmusic #meditation #741hz</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -3924,7 +3924,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #741Hz</t>
+#relaxingmusic #meditation #741hz</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -3934,7 +3934,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #741Hz</t>
+          <t>#relaxingmusic #meditation #741hz</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
@@ -4022,7 +4022,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #852Hz</t>
+#relaxingmusic #meditation #852hz</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -4035,7 +4035,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #852Hz</t>
+#relaxingmusic #meditation #852hz</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -4045,7 +4045,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #852Hz</t>
+          <t>#relaxingmusic #meditation #852hz</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
@@ -4133,7 +4133,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #528Hz</t>
+#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -4146,7 +4146,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#RelaxingMusic #Meditation #528Hz</t>
+#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>#RelaxingMusic #Meditation #528Hz</t>
+          <t>#relaxingmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
@@ -4244,7 +4244,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #639Hz</t>
+#focusmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -4257,7 +4257,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #639Hz</t>
+#focusmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>#FocusMusic #Meditation #639Hz</t>
+          <t>#focusmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
@@ -4355,7 +4355,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #528Hz</t>
+#focusmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -4368,7 +4368,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #528Hz</t>
+#focusmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>#FocusMusic #Meditation #528Hz</t>
+          <t>#focusmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
@@ -4466,7 +4466,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #741Hz</t>
+#focusmusic #meditation #741hz</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -4479,7 +4479,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #741Hz</t>
+#focusmusic #meditation #741hz</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -4489,7 +4489,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>#FocusMusic #Meditation #741Hz</t>
+          <t>#focusmusic #meditation #741hz</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
@@ -4577,7 +4577,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #852Hz</t>
+#focusmusic #meditation #852hz</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -4590,7 +4590,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #852Hz</t>
+#focusmusic #meditation #852hz</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -4600,7 +4600,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>#FocusMusic #Meditation #852Hz</t>
+          <t>#focusmusic #meditation #852hz</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -4688,7 +4688,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #432Hz</t>
+#focusmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4701,7 +4701,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #432Hz</t>
+#focusmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -4711,7 +4711,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>#FocusMusic #Meditation #432Hz</t>
+          <t>#focusmusic #meditation #432hz</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
@@ -4799,7 +4799,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #528Hz</t>
+#focusmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -4812,7 +4812,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #528Hz</t>
+#focusmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>#FocusMusic #Meditation #528Hz</t>
+          <t>#focusmusic #meditation #528hz</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
@@ -4910,7 +4910,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #639Hz</t>
+#focusmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4923,7 +4923,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #639Hz</t>
+#focusmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>#FocusMusic #Meditation #639Hz</t>
+          <t>#focusmusic #meditation #639hz</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
@@ -5021,7 +5021,7 @@
 Original composition, synthesized from scratch, ambience included. No third-party samples.
 Best at low volume.
 Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #741Hz</t>
+#focusmusic #meditation #741hz</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -5034,7 +5034,7 @@
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
 Mejor a volumen bajo.
 Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#FocusMusic #Meditation #741Hz</t>
+#focusmusic #meditation #741hz</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -5044,7 +5044,7 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>#FocusMusic #Meditation #741Hz</t>
+          <t>#focusmusic #meditation #741hz</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
@@ -9231,6 +9231,7 @@
         <is>
           <t>Save this for the next hard moment.
 Full piece (10 min): Music for Anxiety · Zen Temple · 528 Hz · A Brief Pause · 10 Minutes
+https://youtu.be/-ywSggvwt2E
 #anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
         </is>
       </c>
@@ -9307,6 +9308,7 @@
         <is>
           <t>Headphones on. Exhale slowly.
 Full piece (10 min): Music for Anxiety · Zen Temple · 528 Hz · A Brief Pause · 10 Minutes
+https://youtu.be/-ywSggvwt2E
 #anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
         </is>
       </c>
@@ -9383,6 +9385,7 @@
         <is>
           <t>Stay for one full breath.
 Full piece (10 min): Music for Anxiety · Zen Temple · 528 Hz · A Brief Pause · 10 Minutes
+https://youtu.be/-ywSggvwt2E
 #anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
         </is>
       </c>
@@ -9459,6 +9462,7 @@
         <is>
           <t>A small pause in the middle of the day.
 Full piece (10 min): Music for Anxiety · Zen Temple · 528 Hz · A Brief Pause · 10 Minutes
+https://youtu.be/-ywSggvwt2E
 #anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
         </is>
       </c>
@@ -9535,6 +9539,7 @@
         <is>
           <t>Send this to someone who needs a pause.
 Full piece (10 min): Music for Anxiety · Zen Temple · 528 Hz · A Brief Pause · 10 Minutes
+https://youtu.be/-ywSggvwt2E
 #anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
         </is>
       </c>
@@ -10331,6 +10336,7 @@
         <is>
           <t>Save this for the next hard moment.
 Full piece (15 min): Music for Anxiety · Ocean and Birds · 639 Hz · Before You Begin · 15 Minutes
+https://youtu.be/nN2uPKczsrc
 #anxietyrelief #calm #relaxingmusic #639hz #shorts</t>
         </is>
       </c>
@@ -10407,6 +10413,7 @@
         <is>
           <t>Headphones on. Exhale slowly.
 Full piece (15 min): Music for Anxiety · Ocean and Birds · 639 Hz · Before You Begin · 15 Minutes
+https://youtu.be/nN2uPKczsrc
 #anxietyrelief #calm #relaxingmusic #639hz #shorts</t>
         </is>
       </c>
@@ -10483,6 +10490,7 @@
         <is>
           <t>Stay for one full breath.
 Full piece (15 min): Music for Anxiety · Ocean and Birds · 639 Hz · Before You Begin · 15 Minutes
+https://youtu.be/nN2uPKczsrc
 #anxietyrelief #calm #relaxingmusic #639hz #shorts</t>
         </is>
       </c>
@@ -10559,6 +10567,7 @@
         <is>
           <t>A small pause in the middle of the day.
 Full piece (15 min): Music for Anxiety · Ocean and Birds · 639 Hz · Before You Begin · 15 Minutes
+https://youtu.be/nN2uPKczsrc
 #anxietyrelief #calm #relaxingmusic #639hz #shorts</t>
         </is>
       </c>
@@ -10635,6 +10644,7 @@
         <is>
           <t>Send this to someone who needs a pause.
 Full piece (15 min): Music for Anxiety · Ocean and Birds · 639 Hz · Before You Begin · 15 Minutes
+https://youtu.be/nN2uPKczsrc
 #anxietyrelief #calm #relaxingmusic #639hz #shorts</t>
         </is>
       </c>

</xml_diff>

<commit_message>
OBRA-020 publicada; sus Shorts, a la cola de Make
- publicadas.csv: OBRA-020
- shorts_catalogo.py: sin hashtags repetidos en la descripción de TikTok
  (en Meditar salía #meditation dos veces)
- shorts.md: cómo se agregan los Shorts de una obra nueva a la hoja

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -2833,7 +2833,11 @@
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr"/>
-      <c r="L21" s="4" t="inlineStr"/>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>https://youtu.be/QvcXe4ZDq8o</t>
+        </is>
+      </c>
       <c r="M21" s="2" t="n">
         <v>528</v>
       </c>
@@ -2865,10 +2869,14 @@
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="U21" s="4" t="inlineStr"/>
+          <t>publicada</t>
+        </is>
+      </c>
+      <c r="U21" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
       <c r="V21" s="4" t="inlineStr"/>
       <c r="W21" s="4" t="inlineStr"/>
       <c r="X21" s="5">
@@ -11098,7 +11106,7 @@
       <c r="N82" s="3" t="inlineStr">
         <is>
           <t>Save this for your next sit. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #417hz #meditation</t>
+#meditationmusic #meditation #mindfulness #417hz</t>
         </is>
       </c>
       <c r="O82" s="4" t="inlineStr">
@@ -11170,7 +11178,7 @@
       <c r="N83" s="3" t="inlineStr">
         <is>
           <t>Close your eyes for 45 seconds. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #417hz #meditation</t>
+#meditationmusic #meditation #mindfulness #417hz</t>
         </is>
       </c>
       <c r="O83" s="4" t="inlineStr">
@@ -11242,7 +11250,7 @@
       <c r="N84" s="3" t="inlineStr">
         <is>
           <t>Listen until the sound fades. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #417hz #meditation</t>
+#meditationmusic #meditation #mindfulness #417hz</t>
         </is>
       </c>
       <c r="O84" s="4" t="inlineStr">
@@ -11314,7 +11322,7 @@
       <c r="N85" s="3" t="inlineStr">
         <is>
           <t>A minute of stillness. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #417hz #meditation</t>
+#meditationmusic #meditation #mindfulness #417hz</t>
         </is>
       </c>
       <c r="O85" s="4" t="inlineStr">
@@ -11386,7 +11394,7 @@
       <c r="N86" s="3" t="inlineStr">
         <is>
           <t>Send this to someone who meditates. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #417hz #meditation</t>
+#meditationmusic #meditation #mindfulness #417hz</t>
         </is>
       </c>
       <c r="O86" s="4" t="inlineStr">
@@ -11458,7 +11466,7 @@
       <c r="N87" s="3" t="inlineStr">
         <is>
           <t>Save this for your next sit. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O87" s="4" t="inlineStr">
@@ -11530,7 +11538,7 @@
       <c r="N88" s="3" t="inlineStr">
         <is>
           <t>Close your eyes for 45 seconds. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O88" s="4" t="inlineStr">
@@ -11602,7 +11610,7 @@
       <c r="N89" s="3" t="inlineStr">
         <is>
           <t>Listen until the sound fades. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O89" s="4" t="inlineStr">
@@ -11674,7 +11682,7 @@
       <c r="N90" s="3" t="inlineStr">
         <is>
           <t>A minute of stillness. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O90" s="4" t="inlineStr">
@@ -11746,7 +11754,7 @@
       <c r="N91" s="3" t="inlineStr">
         <is>
           <t>Send this to someone who meditates. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O91" s="4" t="inlineStr">
@@ -11818,7 +11826,7 @@
       <c r="N92" s="3" t="inlineStr">
         <is>
           <t>Save this for your next sit. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #432hz #meditation</t>
+#meditationmusic #meditation #mindfulness #432hz</t>
         </is>
       </c>
       <c r="O92" s="4" t="inlineStr">
@@ -11890,7 +11898,7 @@
       <c r="N93" s="3" t="inlineStr">
         <is>
           <t>Close your eyes for 45 seconds. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #432hz #meditation</t>
+#meditationmusic #meditation #mindfulness #432hz</t>
         </is>
       </c>
       <c r="O93" s="4" t="inlineStr">
@@ -11962,7 +11970,7 @@
       <c r="N94" s="3" t="inlineStr">
         <is>
           <t>Listen until the sound fades. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #432hz #meditation</t>
+#meditationmusic #meditation #mindfulness #432hz</t>
         </is>
       </c>
       <c r="O94" s="4" t="inlineStr">
@@ -12034,7 +12042,7 @@
       <c r="N95" s="3" t="inlineStr">
         <is>
           <t>A minute of stillness. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #432hz #meditation</t>
+#meditationmusic #meditation #mindfulness #432hz</t>
         </is>
       </c>
       <c r="O95" s="4" t="inlineStr">
@@ -12106,7 +12114,7 @@
       <c r="N96" s="3" t="inlineStr">
         <is>
           <t>Send this to someone who meditates. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #432hz #meditation</t>
+#meditationmusic #meditation #mindfulness #432hz</t>
         </is>
       </c>
       <c r="O96" s="4" t="inlineStr">
@@ -12161,6 +12169,7 @@
         <is>
           <t>Save this for your next sit.
 Full piece (30 min): Meditation Music · Rain on Leaves · 528 Hz · Strike and Silence · 30 Minutes
+https://youtu.be/QvcXe4ZDq8o
 #meditationmusic #meditation #mindfulness #528hz #shorts</t>
         </is>
       </c>
@@ -12169,7 +12178,11 @@
           <t>meditation music, mindfulness, 528 hz, rain on leaves, Rin</t>
         </is>
       </c>
-      <c r="L97" s="2" t="inlineStr"/>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/QvcXe4ZDq8o</t>
+        </is>
+      </c>
       <c r="M97" s="2" t="inlineStr">
         <is>
           <t>528 Hz · meditate</t>
@@ -12178,7 +12191,7 @@
       <c r="N97" s="3" t="inlineStr">
         <is>
           <t>Save this for your next sit. Full 30 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O97" s="4" t="inlineStr">
@@ -12233,6 +12246,7 @@
         <is>
           <t>Close your eyes for 45 seconds.
 Full piece (30 min): Meditation Music · Rain on Leaves · 528 Hz · Strike and Silence · 30 Minutes
+https://youtu.be/QvcXe4ZDq8o
 #meditationmusic #meditation #mindfulness #528hz #shorts</t>
         </is>
       </c>
@@ -12241,7 +12255,11 @@
           <t>meditation music, mindfulness, 528 hz, rain on leaves, Rin</t>
         </is>
       </c>
-      <c r="L98" s="2" t="inlineStr"/>
+      <c r="L98" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/QvcXe4ZDq8o</t>
+        </is>
+      </c>
       <c r="M98" s="2" t="inlineStr">
         <is>
           <t>528 Hz · stillness</t>
@@ -12250,7 +12268,7 @@
       <c r="N98" s="3" t="inlineStr">
         <is>
           <t>Close your eyes for 45 seconds. Full 30 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O98" s="4" t="inlineStr">
@@ -12305,6 +12323,7 @@
         <is>
           <t>Listen until the sound fades.
 Full piece (30 min): Meditation Music · Rain on Leaves · 528 Hz · Strike and Silence · 30 Minutes
+https://youtu.be/QvcXe4ZDq8o
 #meditationmusic #meditation #mindfulness #528hz #shorts</t>
         </is>
       </c>
@@ -12313,7 +12332,11 @@
           <t>meditation music, mindfulness, 528 hz, rain on leaves, Rin</t>
         </is>
       </c>
-      <c r="L99" s="2" t="inlineStr"/>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/QvcXe4ZDq8o</t>
+        </is>
+      </c>
       <c r="M99" s="2" t="inlineStr">
         <is>
           <t>528 Hz · listen</t>
@@ -12322,7 +12345,7 @@
       <c r="N99" s="3" t="inlineStr">
         <is>
           <t>Listen until the sound fades. Full 30 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O99" s="4" t="inlineStr">
@@ -12377,6 +12400,7 @@
         <is>
           <t>A minute of stillness.
 Full piece (30 min): Meditation Music · Rain on Leaves · 528 Hz · Strike and Silence · 30 Minutes
+https://youtu.be/QvcXe4ZDq8o
 #meditationmusic #meditation #mindfulness #528hz #shorts</t>
         </is>
       </c>
@@ -12385,7 +12409,11 @@
           <t>meditation music, mindfulness, 528 hz, rain on leaves, Rin</t>
         </is>
       </c>
-      <c r="L100" s="2" t="inlineStr"/>
+      <c r="L100" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/QvcXe4ZDq8o</t>
+        </is>
+      </c>
       <c r="M100" s="2" t="inlineStr">
         <is>
           <t>528 Hz · sit</t>
@@ -12394,7 +12422,7 @@
       <c r="N100" s="3" t="inlineStr">
         <is>
           <t>A minute of stillness. Full 30 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O100" s="4" t="inlineStr">
@@ -12449,6 +12477,7 @@
         <is>
           <t>Send this to someone who meditates.
 Full piece (30 min): Meditation Music · Rain on Leaves · 528 Hz · Strike and Silence · 30 Minutes
+https://youtu.be/QvcXe4ZDq8o
 #meditationmusic #meditation #mindfulness #528hz #shorts</t>
         </is>
       </c>
@@ -12457,7 +12486,11 @@
           <t>meditation music, mindfulness, 528 hz, rain on leaves, Rin</t>
         </is>
       </c>
-      <c r="L101" s="2" t="inlineStr"/>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/QvcXe4ZDq8o</t>
+        </is>
+      </c>
       <c r="M101" s="2" t="inlineStr">
         <is>
           <t>528 Hz · silence</t>
@@ -12466,7 +12499,7 @@
       <c r="N101" s="3" t="inlineStr">
         <is>
           <t>Send this to someone who meditates. Full 30 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O101" s="4" t="inlineStr">
@@ -12538,7 +12571,7 @@
       <c r="N102" s="3" t="inlineStr">
         <is>
           <t>Save this for your next sit. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #396hz #meditation</t>
+#meditationmusic #meditation #mindfulness #396hz</t>
         </is>
       </c>
       <c r="O102" s="4" t="inlineStr">
@@ -12610,7 +12643,7 @@
       <c r="N103" s="3" t="inlineStr">
         <is>
           <t>Close your eyes for 45 seconds. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #396hz #meditation</t>
+#meditationmusic #meditation #mindfulness #396hz</t>
         </is>
       </c>
       <c r="O103" s="4" t="inlineStr">
@@ -12682,7 +12715,7 @@
       <c r="N104" s="3" t="inlineStr">
         <is>
           <t>Listen until the sound fades. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #396hz #meditation</t>
+#meditationmusic #meditation #mindfulness #396hz</t>
         </is>
       </c>
       <c r="O104" s="4" t="inlineStr">
@@ -12754,7 +12787,7 @@
       <c r="N105" s="3" t="inlineStr">
         <is>
           <t>A minute of stillness. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #396hz #meditation</t>
+#meditationmusic #meditation #mindfulness #396hz</t>
         </is>
       </c>
       <c r="O105" s="4" t="inlineStr">
@@ -12826,7 +12859,7 @@
       <c r="N106" s="3" t="inlineStr">
         <is>
           <t>Send this to someone who meditates. Full 45 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #396hz #meditation</t>
+#meditationmusic #meditation #mindfulness #396hz</t>
         </is>
       </c>
       <c r="O106" s="4" t="inlineStr">
@@ -12898,7 +12931,7 @@
       <c r="N107" s="3" t="inlineStr">
         <is>
           <t>Save this for your next sit. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #639hz #meditation</t>
+#meditationmusic #meditation #mindfulness #639hz</t>
         </is>
       </c>
       <c r="O107" s="4" t="inlineStr">
@@ -12970,7 +13003,7 @@
       <c r="N108" s="3" t="inlineStr">
         <is>
           <t>Close your eyes for 45 seconds. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #639hz #meditation</t>
+#meditationmusic #meditation #mindfulness #639hz</t>
         </is>
       </c>
       <c r="O108" s="4" t="inlineStr">
@@ -13042,7 +13075,7 @@
       <c r="N109" s="3" t="inlineStr">
         <is>
           <t>Listen until the sound fades. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #639hz #meditation</t>
+#meditationmusic #meditation #mindfulness #639hz</t>
         </is>
       </c>
       <c r="O109" s="4" t="inlineStr">
@@ -13114,7 +13147,7 @@
       <c r="N110" s="3" t="inlineStr">
         <is>
           <t>A minute of stillness. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #639hz #meditation</t>
+#meditationmusic #meditation #mindfulness #639hz</t>
         </is>
       </c>
       <c r="O110" s="4" t="inlineStr">
@@ -13186,7 +13219,7 @@
       <c r="N111" s="3" t="inlineStr">
         <is>
           <t>Send this to someone who meditates. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #639hz #meditation</t>
+#meditationmusic #meditation #mindfulness #639hz</t>
         </is>
       </c>
       <c r="O111" s="4" t="inlineStr">
@@ -13258,7 +13291,7 @@
       <c r="N112" s="3" t="inlineStr">
         <is>
           <t>Save this for your next sit. Full 20 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O112" s="4" t="inlineStr">
@@ -13330,7 +13363,7 @@
       <c r="N113" s="3" t="inlineStr">
         <is>
           <t>Close your eyes for 45 seconds. Full 20 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O113" s="4" t="inlineStr">
@@ -13402,7 +13435,7 @@
       <c r="N114" s="3" t="inlineStr">
         <is>
           <t>Listen until the sound fades. Full 20 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O114" s="4" t="inlineStr">
@@ -13474,7 +13507,7 @@
       <c r="N115" s="3" t="inlineStr">
         <is>
           <t>A minute of stillness. Full 20 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O115" s="4" t="inlineStr">
@@ -13546,7 +13579,7 @@
       <c r="N116" s="3" t="inlineStr">
         <is>
           <t>Send this to someone who meditates. Full 20 min piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #528hz #meditation</t>
+#meditationmusic #meditation #mindfulness #528hz</t>
         </is>
       </c>
       <c r="O116" s="4" t="inlineStr">
@@ -13618,7 +13651,7 @@
       <c r="N117" s="3" t="inlineStr">
         <is>
           <t>Save this for your next sit. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #432hz #meditation</t>
+#meditationmusic #meditation #mindfulness #432hz</t>
         </is>
       </c>
       <c r="O117" s="4" t="inlineStr">
@@ -13690,7 +13723,7 @@
       <c r="N118" s="3" t="inlineStr">
         <is>
           <t>Close your eyes for 45 seconds. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #432hz #meditation</t>
+#meditationmusic #meditation #mindfulness #432hz</t>
         </is>
       </c>
       <c r="O118" s="4" t="inlineStr">
@@ -13762,7 +13795,7 @@
       <c r="N119" s="3" t="inlineStr">
         <is>
           <t>Listen until the sound fades. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #432hz #meditation</t>
+#meditationmusic #meditation #mindfulness #432hz</t>
         </is>
       </c>
       <c r="O119" s="4" t="inlineStr">
@@ -13834,7 +13867,7 @@
       <c r="N120" s="3" t="inlineStr">
         <is>
           <t>A minute of stillness. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #432hz #meditation</t>
+#meditationmusic #meditation #mindfulness #432hz</t>
         </is>
       </c>
       <c r="O120" s="4" t="inlineStr">
@@ -13906,7 +13939,7 @@
       <c r="N121" s="3" t="inlineStr">
         <is>
           <t>Send this to someone who meditates. Full 1 h piece on YouTube: Rin.
-#meditationmusic #meditation #mindfulness #432hz #meditation</t>
+#meditationmusic #meditation #mindfulness #432hz</t>
         </is>
       </c>
       <c r="O121" s="4" t="inlineStr">

</xml_diff>

<commit_message>
OBRA-006 publicada; workflow para borrar el video largo de una Release
- publicadas.csv: OBRA-006 (https://youtu.be/cECOoUGLqes)
- catálogo y hoja de Shorts regenerados: los 7 de OBRA-006 enlazan al video
- borrar-video.yml: quita solo <OBRA>-video.mp4 de la Release de una obra que
  ya está en publicadas.csv (los Shorts, la miniatura y los textos quedan)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -1284,7 +1284,11 @@
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr"/>
-      <c r="L7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>https://youtu.be/cECOoUGLqes</t>
+        </is>
+      </c>
       <c r="M7" s="2" t="n">
         <v>417</v>
       </c>
@@ -1319,10 +1323,14 @@
       </c>
       <c r="U7" s="4" t="inlineStr">
         <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V7" s="4" t="inlineStr"/>
+          <t>publicada</t>
+        </is>
+      </c>
+      <c r="V7" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
       <c r="W7" s="4" t="inlineStr"/>
       <c r="X7" s="4" t="inlineStr"/>
       <c r="Y7" s="5">
@@ -7925,6 +7933,7 @@
         <is>
           <t>Save this for tonight.
 Full piece (90 min): Sleep Music · Ocean Waves · 417 Hz · Before Dawn · 90 Minutes
+https://youtu.be/cECOoUGLqes
 #sleepmusic #sleep #relaxingmusic #417hz #shorts</t>
         </is>
       </c>
@@ -7933,7 +7942,11 @@
           <t>sleep music, deep sleep, 417 hz, ocean waves, Rin</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/cECOoUGLqes</t>
+        </is>
+      </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
           <t>417 Hz · sleep</t>
@@ -7997,6 +8010,7 @@
         <is>
           <t>Lights off, volume low.
 Full piece (90 min): Sleep Music · Ocean Waves · 417 Hz · Before Dawn · 90 Minutes
+https://youtu.be/cECOoUGLqes
 #sleepmusic #sleep #relaxingmusic #417hz #shorts</t>
         </is>
       </c>
@@ -8005,7 +8019,11 @@
           <t>sleep music, deep sleep, 417 hz, ocean waves, Rin</t>
         </is>
       </c>
-      <c r="L38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/cECOoUGLqes</t>
+        </is>
+      </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
           <t>417 Hz · night</t>
@@ -8069,6 +8087,7 @@
         <is>
           <t>Stay until your breathing slows.
 Full piece (90 min): Sleep Music · Ocean Waves · 417 Hz · Before Dawn · 90 Minutes
+https://youtu.be/cECOoUGLqes
 #sleepmusic #sleep #relaxingmusic #417hz #shorts</t>
         </is>
       </c>
@@ -8077,7 +8096,11 @@
           <t>sleep music, deep sleep, 417 hz, ocean waves, Rin</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/cECOoUGLqes</t>
+        </is>
+      </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
           <t>417 Hz · rest</t>
@@ -8141,6 +8164,7 @@
         <is>
           <t>The quiet hour before sleep.
 Full piece (90 min): Sleep Music · Ocean Waves · 417 Hz · Before Dawn · 90 Minutes
+https://youtu.be/cECOoUGLqes
 #sleepmusic #sleep #relaxingmusic #417hz #shorts</t>
         </is>
       </c>
@@ -8149,7 +8173,11 @@
           <t>sleep music, deep sleep, 417 hz, ocean waves, Rin</t>
         </is>
       </c>
-      <c r="L40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/cECOoUGLqes</t>
+        </is>
+      </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
           <t>417 Hz · dark room</t>
@@ -8213,6 +8241,7 @@
         <is>
           <t>Send this to someone who can't sleep.
 Full piece (90 min): Sleep Music · Ocean Waves · 417 Hz · Before Dawn · 90 Minutes
+https://youtu.be/cECOoUGLqes
 #sleepmusic #sleep #relaxingmusic #417hz #shorts</t>
         </is>
       </c>
@@ -8221,7 +8250,11 @@
           <t>sleep music, deep sleep, 417 hz, ocean waves, Rin</t>
         </is>
       </c>
-      <c r="L41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/cECOoUGLqes</t>
+        </is>
+      </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
           <t>417 Hz · drift off</t>
@@ -8285,6 +8318,7 @@
         <is>
           <t>Turn the brightness down and stay.
 Full piece (90 min): Sleep Music · Ocean Waves · 417 Hz · Before Dawn · 90 Minutes
+https://youtu.be/cECOoUGLqes
 #sleepmusic #sleep #relaxingmusic #417hz #shorts</t>
         </is>
       </c>
@@ -8293,7 +8327,11 @@
           <t>sleep music, deep sleep, 417 hz, ocean waves, Rin</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/cECOoUGLqes</t>
+        </is>
+      </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
           <t>417 Hz · lights off</t>
@@ -8357,6 +8395,7 @@
         <is>
           <t>Play it as the last thing tonight.
 Full piece (90 min): Sleep Music · Ocean Waves · 417 Hz · Before Dawn · 90 Minutes
+https://youtu.be/cECOoUGLqes
 #sleepmusic #sleep #relaxingmusic #417hz #shorts</t>
         </is>
       </c>
@@ -8365,7 +8404,11 @@
           <t>sleep music, deep sleep, 417 hz, ocean waves, Rin</t>
         </is>
       </c>
-      <c r="L43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/cECOoUGLqes</t>
+        </is>
+      </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
           <t>417 Hz · deep rest</t>

</xml_diff>

<commit_message>
OBRA-041 «Stop Overthinking»: ambiente jardín, pájaros y campanas del templo
- ambiente nuevo «jardin»: pájaros con furin sueltos y bajos, afinados a la
  raíz, y el mar muy lejos (capas.py jardin); paleta jade en el mandala, anillos
  que salen cada 12 s (5 resp/min)
- OBRA-041: Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop
  Overthinking · 1 Hour (hirajoshi, 6 → 4.5 resp/min)
- capas.py recibe la raíz de la obra (antes las campanitas del templo zen
  sonaban siempre en 528 Hz, aunque la obra fuera de 432)
- montar.py: el bucle va siempre en HEVC (≈40 % menos peso) y el audio sube
  de 256 a 320 kbps

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$Y$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$281</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$Y$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$288</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y41"/>
+  <dimension ref="A1:Y42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 1540 audio/OBRA-009_capa.wav --semilla 555819 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-009_396_kumoi.wav audio/OBRA-009_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-009_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 1540 audio/OBRA-009_capa.wav --semilla 555819 --raiz 396 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-009_396_kumoi.wav audio/OBRA-009_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-009_capa.wav</t>
         </is>
       </c>
       <c r="U10" s="4" t="inlineStr">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 1840 audio/OBRA-010_capa.wav --semilla 739461 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-010_432_hirajoshi.wav audio/OBRA-010_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-010_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 1840 audio/OBRA-010_capa.wav --semilla 739461 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-010_432_hirajoshi.wav audio/OBRA-010_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-010_capa.wav</t>
         </is>
       </c>
       <c r="U11" s="4" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 1240 audio/OBRA-011_capa.wav --semilla 913368 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-011_528_hirajoshi.wav audio/OBRA-011_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-011_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 1240 audio/OBRA-011_capa.wav --semilla 913368 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-011_528_hirajoshi.wav audio/OBRA-011_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-011_capa.wav</t>
         </is>
       </c>
       <c r="U12" s="4" t="inlineStr">
@@ -2010,7 +2010,7 @@
       </c>
       <c r="T13" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 640 audio/OBRA-012_capa.wav --semilla 43734 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-012_528_shin.wav audio/OBRA-012_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-012_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 640 audio/OBRA-012_capa.wav --semilla 43734 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-012_528_shin.wav audio/OBRA-012_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-012_capa.wav</t>
         </is>
       </c>
       <c r="U13" s="4" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 1240 audio/OBRA-013_capa.wav --semilla 627771 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-013_432_hirajoshi.wav audio/OBRA-013_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-013_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 1240 audio/OBRA-013_capa.wav --semilla 627771 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-013_432_hirajoshi.wav audio/OBRA-013_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-013_capa.wav</t>
         </is>
       </c>
       <c r="U14" s="4" t="inlineStr">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="T15" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-014_capa.wav --semilla 310137 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-014_528_yo.wav audio/OBRA-014_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-014_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-014_capa.wav --semilla 310137 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-014_528_yo.wav audio/OBRA-014_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-014_capa.wav</t>
         </is>
       </c>
       <c r="U15" s="4" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="T16" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 940 audio/OBRA-015_capa.wav --semilla 592463 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-015_639_yo.wav audio/OBRA-015_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-015_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 940 audio/OBRA-015_capa.wav --semilla 592463 --raiz 639 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-015_639_yo.wav audio/OBRA-015_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-015_capa.wav</t>
         </is>
       </c>
       <c r="U16" s="4" t="inlineStr">
@@ -2478,7 +2478,7 @@
       </c>
       <c r="T17" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py ancestral 1840 audio/OBRA-016_capa.wav --semilla 250697 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-016_417_kumoi.wav audio/OBRA-016_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-016_capa.wav</t>
+          <t>python3 03-composicion/capas.py ancestral 1840 audio/OBRA-016_capa.wav --semilla 250697 --raiz 417 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-016_417_kumoi.wav audio/OBRA-016_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-016_capa.wav</t>
         </is>
       </c>
       <c r="U17" s="4" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-017_capa.wav --semilla 714152 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-017_417_hirajoshi.wav audio/OBRA-017_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-017_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-017_capa.wav --semilla 714152 --raiz 417 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-017_417_hirajoshi.wav audio/OBRA-017_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-017_capa.wav</t>
         </is>
       </c>
       <c r="U18" s="4" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-018_capa.wav --semilla 735455 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-018_528_hirajoshi.wav audio/OBRA-018_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-018_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-018_capa.wav --semilla 735455 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-018_528_hirajoshi.wav audio/OBRA-018_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-018_capa.wav</t>
         </is>
       </c>
       <c r="U19" s="4" t="inlineStr">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="T20" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-019_capa.wav --semilla 627577 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-019_432_shin.wav audio/OBRA-019_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-019_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-019_capa.wav --semilla 627577 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-019_432_shin.wav audio/OBRA-019_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-019_capa.wav</t>
         </is>
       </c>
       <c r="U20" s="4" t="inlineStr">
@@ -2938,7 +2938,7 @@
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py ancestral 1840 audio/OBRA-020_capa.wav --semilla 632595 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-020_528_shin.wav audio/OBRA-020_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-020_capa.wav</t>
+          <t>python3 03-composicion/capas.py ancestral 1840 audio/OBRA-020_capa.wav --semilla 632595 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-020_528_shin.wav audio/OBRA-020_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-020_capa.wav</t>
         </is>
       </c>
       <c r="U21" s="4" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-021_capa.wav --semilla 864630 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-021_396_kumoi.wav audio/OBRA-021_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-021_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-021_capa.wav --semilla 864630 --raiz 396 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-021_396_kumoi.wav audio/OBRA-021_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-021_capa.wav</t>
         </is>
       </c>
       <c r="U22" s="4" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-022_capa.wav --semilla 335798 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-022_639_yo.wav audio/OBRA-022_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-022_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-022_capa.wav --semilla 335798 --raiz 639 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-022_639_yo.wav audio/OBRA-022_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-022_capa.wav</t>
         </is>
       </c>
       <c r="U23" s="4" t="inlineStr">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="T24" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-023_capa.wav --semilla 299306 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-023_528_shin.wav audio/OBRA-023_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-023_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-023_capa.wav --semilla 299306 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-023_528_shin.wav audio/OBRA-023_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-023_capa.wav</t>
         </is>
       </c>
       <c r="U24" s="4" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py ancestral 3640 audio/OBRA-024_capa.wav --semilla 926202 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-024_432_kumoi.wav audio/OBRA-024_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-024_capa.wav</t>
+          <t>python3 03-composicion/capas.py ancestral 3640 audio/OBRA-024_capa.wav --semilla 926202 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-024_432_kumoi.wav audio/OBRA-024_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-024_capa.wav</t>
         </is>
       </c>
       <c r="U25" s="4" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="T26" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 3640 audio/OBRA-025_capa.wav --semilla 454078 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-025_528_hirajoshi.wav audio/OBRA-025_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-025_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 3640 audio/OBRA-025_capa.wav --semilla 454078 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-025_528_hirajoshi.wav audio/OBRA-025_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-025_capa.wav</t>
         </is>
       </c>
       <c r="U26" s="4" t="inlineStr">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="T28" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py ancestral 3640 audio/OBRA-027_capa.wav --semilla 338018 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-027_396_kumoi.wav audio/OBRA-027_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-027_capa.wav</t>
+          <t>python3 03-composicion/capas.py ancestral 3640 audio/OBRA-027_capa.wav --semilla 338018 --raiz 396 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-027_396_kumoi.wav audio/OBRA-027_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-027_capa.wav</t>
         </is>
       </c>
       <c r="U28" s="4" t="inlineStr">
@@ -3854,7 +3854,7 @@
       </c>
       <c r="T29" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-028_capa.wav --semilla 409966 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-028_417_hirajoshi.wav audio/OBRA-028_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-028_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-028_capa.wav --semilla 409966 --raiz 417 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-028_417_hirajoshi.wav audio/OBRA-028_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-028_capa.wav</t>
         </is>
       </c>
       <c r="U29" s="4" t="inlineStr">
@@ -3968,7 +3968,7 @@
       </c>
       <c r="T30" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 3640 audio/OBRA-029_capa.wav --semilla 133046 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-029_639_yo.wav audio/OBRA-029_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-029_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 3640 audio/OBRA-029_capa.wav --semilla 133046 --raiz 639 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-029_639_yo.wav audio/OBRA-029_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-029_capa.wav</t>
         </is>
       </c>
       <c r="U30" s="4" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="T31" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 2740 audio/OBRA-030_capa.wav --semilla 244487 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-030_741_yo.wav audio/OBRA-030_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-030_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 2740 audio/OBRA-030_capa.wav --semilla 244487 --raiz 741 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-030_741_yo.wav audio/OBRA-030_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-030_capa.wav</t>
         </is>
       </c>
       <c r="U31" s="4" t="inlineStr">
@@ -4196,7 +4196,7 @@
       </c>
       <c r="T32" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-031_capa.wav --semilla 288169 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-031_852_hirajoshi.wav audio/OBRA-031_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-031_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-031_capa.wav --semilla 288169 --raiz 852 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-031_852_hirajoshi.wav audio/OBRA-031_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-031_capa.wav</t>
         </is>
       </c>
       <c r="U32" s="4" t="inlineStr">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="T33" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 10840 audio/OBRA-032_capa.wav --semilla 638156 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-032_528_hirajoshi.wav audio/OBRA-032_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-032_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 10840 audio/OBRA-032_capa.wav --semilla 638156 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-032_528_hirajoshi.wav audio/OBRA-032_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-032_capa.wav</t>
         </is>
       </c>
       <c r="U33" s="4" t="inlineStr">
@@ -4424,7 +4424,7 @@
       </c>
       <c r="T34" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 7240 audio/OBRA-033_capa.wav --semilla 112334 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-033_639_yo.wav audio/OBRA-033_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-033_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 7240 audio/OBRA-033_capa.wav --semilla 112334 --raiz 639 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-033_639_yo.wav audio/OBRA-033_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-033_capa.wav</t>
         </is>
       </c>
       <c r="U34" s="4" t="inlineStr">
@@ -4538,7 +4538,7 @@
       </c>
       <c r="T35" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 10840 audio/OBRA-034_capa.wav --semilla 249239 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-034_528_yo.wav audio/OBRA-034_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-034_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 10840 audio/OBRA-034_capa.wav --semilla 249239 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-034_528_yo.wav audio/OBRA-034_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-034_capa.wav</t>
         </is>
       </c>
       <c r="U35" s="4" t="inlineStr">
@@ -4652,7 +4652,7 @@
       </c>
       <c r="T36" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 7240 audio/OBRA-035_capa.wav --semilla 74636 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-035_741_yo.wav audio/OBRA-035_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-035_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 7240 audio/OBRA-035_capa.wav --semilla 74636 --raiz 741 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-035_741_yo.wav audio/OBRA-035_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-035_capa.wav</t>
         </is>
       </c>
       <c r="U36" s="4" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="T37" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 5440 audio/OBRA-036_capa.wav --semilla 903477 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-036_852_yo.wav audio/OBRA-036_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-036_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 5440 audio/OBRA-036_capa.wav --semilla 903477 --raiz 852 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-036_852_yo.wav audio/OBRA-036_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-036_capa.wav</t>
         </is>
       </c>
       <c r="U37" s="4" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="T38" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 7240 audio/OBRA-037_capa.wav --semilla 718809 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-037_432_yo.wav audio/OBRA-037_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-037_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 7240 audio/OBRA-037_capa.wav --semilla 718809 --raiz 432 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-037_432_yo.wav audio/OBRA-037_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-037_capa.wav</t>
         </is>
       </c>
       <c r="U38" s="4" t="inlineStr">
@@ -5108,7 +5108,7 @@
       </c>
       <c r="T40" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 5440 audio/OBRA-039_capa.wav --semilla 281608 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-039_639_yo.wav audio/OBRA-039_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-039_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 5440 audio/OBRA-039_capa.wav --semilla 281608 --raiz 639 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-039_639_yo.wav audio/OBRA-039_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-039_capa.wav</t>
         </is>
       </c>
       <c r="U40" s="4" t="inlineStr">
@@ -5222,7 +5222,7 @@
       </c>
       <c r="T41" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py aves 10840 audio/OBRA-040_capa.wav --semilla 883876 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-040_741_yo.wav audio/OBRA-040_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-040_capa.wav</t>
+          <t>python3 03-composicion/capas.py aves 10840 audio/OBRA-040_capa.wav --semilla 883876 --raiz 741 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-040_741_yo.wav audio/OBRA-040_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-040_capa.wav</t>
         </is>
       </c>
       <c r="U41" s="4" t="inlineStr">
@@ -5238,8 +5238,122 @@
         <v/>
       </c>
     </row>
+    <row r="42" ht="58" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Música para momentos de ansiedad · Pájaros y campanas del templo · 432 Hz · Dejar de pensar · 1 hora</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Ansiedad</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>jardin</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Stop Overthinking · 1 Hour
+To accompany a pause when your mind won't stop.
+Ambience: birds and temple bells.
+Composed around a root of 432 Hz, in just intonation, hirajoshi mode.
+Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
+Original composition, synthesized from scratch, ambience included. No third-party samples.
+Best at low volume.
+Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#relaxingmusic #meditation #432hz</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Dejar de pensar · 1 hora
+Para acompañar un momento de pausa cuando la cabeza no para.
+Ambiente: pájaros y campanas del templo.
+Compuesta con raíz en 432 Hz, en entonación justa, modo hirajoshi.
+Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
+Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#relaxingmusic #meditation #432hz</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>60 MIN</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>#relaxingmusic #meditation #432hz</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>music for anxiety, 432 hz, 432 hz music, anxiety relief, stress relief, calming music, birdsong, wind chimes, zen garden, relaxing music, meditation music, ambient music, just intonation, original composition, Rin, música para momentos de ansiedad</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr"/>
+      <c r="L42" s="4" t="inlineStr"/>
+      <c r="M42" s="2" t="n">
+        <v>432</v>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>hirajoshi</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>medio</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="n">
+        <v>304617</v>
+      </c>
+      <c r="Q42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R42" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="S42" s="3" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/compositor.py --minutos 60 --raiz 432 --modo hirajoshi --semilla 304617 --caracter sin-cuenco</t>
+        </is>
+      </c>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/capas.py jardin 3640 audio/OBRA-041_capa.wav --semilla 304617 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-041_432_hirajoshi.wav audio/OBRA-041_final.wav --fondo mar --nivel-fondo -8 --nivel-capa 0 --capa audio/OBRA-041_capa.wav</t>
+        </is>
+      </c>
+      <c r="U42" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="V42" s="4" t="inlineStr"/>
+      <c r="W42" s="4" t="inlineStr"/>
+      <c r="X42" s="4" t="inlineStr"/>
+      <c r="Y42" s="5">
+        <f>IFERROR(X42/W42*1000,"")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Y41"/>
+  <autoFilter ref="A1:Y42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5250,7 +5364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S281"/>
+  <dimension ref="A1:S288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -25671,8 +25785,512 @@
       <c r="R281" s="4" t="inlineStr"/>
       <c r="S281" s="4" t="inlineStr"/>
     </row>
+    <row r="282" ht="58" customHeight="1">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041-S1</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D282" s="2" t="inlineStr">
+        <is>
+          <t>short-1.mp4</t>
+        </is>
+      </c>
+      <c r="E282" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="F282" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G282" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H282" s="2" t="inlineStr">
+        <is>
+          <t>for when your mind won't stop</t>
+        </is>
+      </c>
+      <c r="I282" s="3" t="inlineStr">
+        <is>
+          <t>For when your mind won't stop · 432 Hz · Birds and Temple Bells</t>
+        </is>
+      </c>
+      <c r="J282" s="3" t="inlineStr">
+        <is>
+          <t>Save this for the next hard moment.
+Full piece (1 h): Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour
+#anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K282" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
+        </is>
+      </c>
+      <c r="L282" s="2" t="inlineStr"/>
+      <c r="M282" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · calm</t>
+        </is>
+      </c>
+      <c r="N282" s="3" t="inlineStr">
+        <is>
+          <t>Save this for the next hard moment. Full 1 h piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O282" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P282" s="4" t="inlineStr"/>
+      <c r="Q282" s="4" t="inlineStr"/>
+      <c r="R282" s="4" t="inlineStr"/>
+      <c r="S282" s="4" t="inlineStr"/>
+    </row>
+    <row r="283" ht="58" customHeight="1">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041-S2</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>short-2.mp4</t>
+        </is>
+      </c>
+      <c r="E283" s="2" t="n">
+        <v>961</v>
+      </c>
+      <c r="F283" s="2" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G283" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H283" s="2" t="inlineStr">
+        <is>
+          <t>breathe out longer than you breathe in</t>
+        </is>
+      </c>
+      <c r="I283" s="3" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in · 432 Hz · Birds and Temple Bells</t>
+        </is>
+      </c>
+      <c r="J283" s="3" t="inlineStr">
+        <is>
+          <t>Headphones on. Exhale slowly.
+Full piece (1 h): Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour
+#anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K283" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
+        </is>
+      </c>
+      <c r="L283" s="2" t="inlineStr"/>
+      <c r="M283" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · exhale</t>
+        </is>
+      </c>
+      <c r="N283" s="3" t="inlineStr">
+        <is>
+          <t>Headphones on. Exhale slowly. Full 1 h piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O283" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P283" s="4" t="inlineStr"/>
+      <c r="Q283" s="4" t="inlineStr"/>
+      <c r="R283" s="4" t="inlineStr"/>
+      <c r="S283" s="4" t="inlineStr"/>
+    </row>
+    <row r="284" ht="58" customHeight="1">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041-S3</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D284" s="2" t="inlineStr">
+        <is>
+          <t>short-3.mp4</t>
+        </is>
+      </c>
+      <c r="E284" s="2" t="n">
+        <v>1832</v>
+      </c>
+      <c r="F284" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G284" s="2" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H284" s="2" t="inlineStr">
+        <is>
+          <t>a pause, just for you</t>
+        </is>
+      </c>
+      <c r="I284" s="3" t="inlineStr">
+        <is>
+          <t>A pause, just for you · 432 Hz · Birds and Temple Bells</t>
+        </is>
+      </c>
+      <c r="J284" s="3" t="inlineStr">
+        <is>
+          <t>Stay for one full breath.
+Full piece (1 h): Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour
+#anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K284" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
+        </is>
+      </c>
+      <c r="L284" s="2" t="inlineStr"/>
+      <c r="M284" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · pause</t>
+        </is>
+      </c>
+      <c r="N284" s="3" t="inlineStr">
+        <is>
+          <t>Stay for one full breath. Full 1 h piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O284" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P284" s="4" t="inlineStr"/>
+      <c r="Q284" s="4" t="inlineStr"/>
+      <c r="R284" s="4" t="inlineStr"/>
+      <c r="S284" s="4" t="inlineStr"/>
+    </row>
+    <row r="285" ht="58" customHeight="1">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041-S4</t>
+        </is>
+      </c>
+      <c r="B285" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041</t>
+        </is>
+      </c>
+      <c r="C285" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D285" s="2" t="inlineStr">
+        <is>
+          <t>short-4.mp4</t>
+        </is>
+      </c>
+      <c r="E285" s="2" t="n">
+        <v>2704</v>
+      </c>
+      <c r="F285" s="2" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="G285" s="2" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="H285" s="2" t="inlineStr">
+        <is>
+          <t>slow down, one breath at a time</t>
+        </is>
+      </c>
+      <c r="I285" s="3" t="inlineStr">
+        <is>
+          <t>Slow down, one breath at a time · 432 Hz · Birds and Temple Bells</t>
+        </is>
+      </c>
+      <c r="J285" s="3" t="inlineStr">
+        <is>
+          <t>A small pause in the middle of the day.
+Full piece (1 h): Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour
+#anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K285" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
+        </is>
+      </c>
+      <c r="L285" s="2" t="inlineStr"/>
+      <c r="M285" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · breathe</t>
+        </is>
+      </c>
+      <c r="N285" s="3" t="inlineStr">
+        <is>
+          <t>A small pause in the middle of the day. Full 1 h piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O285" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P285" s="4" t="inlineStr"/>
+      <c r="Q285" s="4" t="inlineStr"/>
+      <c r="R285" s="4" t="inlineStr"/>
+      <c r="S285" s="4" t="inlineStr"/>
+    </row>
+    <row r="286" ht="58" customHeight="1">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041-S5</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>short-5.mp4</t>
+        </is>
+      </c>
+      <c r="E286" s="2" t="n">
+        <v>3575</v>
+      </c>
+      <c r="F286" s="2" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="G286" s="2" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="H286" s="2" t="inlineStr">
+        <is>
+          <t>before you begin</t>
+        </is>
+      </c>
+      <c r="I286" s="3" t="inlineStr">
+        <is>
+          <t>Before you begin · 432 Hz · Birds and Temple Bells</t>
+        </is>
+      </c>
+      <c r="J286" s="3" t="inlineStr">
+        <is>
+          <t>Send this to someone who needs a pause.
+Full piece (1 h): Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour
+#anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K286" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
+        </is>
+      </c>
+      <c r="L286" s="2" t="inlineStr"/>
+      <c r="M286" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · slow down</t>
+        </is>
+      </c>
+      <c r="N286" s="3" t="inlineStr">
+        <is>
+          <t>Send this to someone who needs a pause. Full 1 h piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O286" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P286" s="4" t="inlineStr"/>
+      <c r="Q286" s="4" t="inlineStr"/>
+      <c r="R286" s="4" t="inlineStr"/>
+      <c r="S286" s="4" t="inlineStr"/>
+    </row>
+    <row r="287" ht="58" customHeight="1">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041-S6</t>
+        </is>
+      </c>
+      <c r="B287" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>short-6.mp4</t>
+        </is>
+      </c>
+      <c r="E287" s="2" t="n">
+        <v>526</v>
+      </c>
+      <c r="F287" s="2" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="G287" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H287" s="2" t="inlineStr">
+        <is>
+          <t>you can put it down for now</t>
+        </is>
+      </c>
+      <c r="I287" s="3" t="inlineStr">
+        <is>
+          <t>You can put it down for now · 432 Hz · Birds and Temple Bells</t>
+        </is>
+      </c>
+      <c r="J287" s="3" t="inlineStr">
+        <is>
+          <t>Breathe with the sound for a moment.
+Full piece (1 h): Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour
+#anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K287" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
+        </is>
+      </c>
+      <c r="L287" s="2" t="inlineStr"/>
+      <c r="M287" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · let go</t>
+        </is>
+      </c>
+      <c r="N287" s="3" t="inlineStr">
+        <is>
+          <t>Breathe with the sound for a moment. Full 1 h piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O287" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P287" s="4" t="inlineStr"/>
+      <c r="Q287" s="4" t="inlineStr"/>
+      <c r="R287" s="4" t="inlineStr"/>
+      <c r="S287" s="4" t="inlineStr"/>
+    </row>
+    <row r="288" ht="58" customHeight="1">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041-S7</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-041</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>short-7.mp4</t>
+        </is>
+      </c>
+      <c r="E288" s="2" t="n">
+        <v>2268</v>
+      </c>
+      <c r="F288" s="2" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G288" s="2" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="H288" s="2" t="inlineStr">
+        <is>
+          <t>one minute of quiet</t>
+        </is>
+      </c>
+      <c r="I288" s="3" t="inlineStr">
+        <is>
+          <t>One minute of quiet · 432 Hz · Birds and Temple Bells</t>
+        </is>
+      </c>
+      <c r="J288" s="3" t="inlineStr">
+        <is>
+          <t>Come back to this when you need it.
+Full piece (1 h): Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour
+#anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K288" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
+        </is>
+      </c>
+      <c r="L288" s="2" t="inlineStr"/>
+      <c r="M288" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · quiet</t>
+        </is>
+      </c>
+      <c r="N288" s="3" t="inlineStr">
+        <is>
+          <t>Come back to this when you need it. Full 1 h piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O288" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P288" s="4" t="inlineStr"/>
+      <c r="Q288" s="4" t="inlineStr"/>
+      <c r="R288" s="4" t="inlineStr"/>
+      <c r="S288" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S281"/>
+  <autoFilter ref="A1:S288"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -25707,7 +26325,7 @@
         </is>
       </c>
       <c r="B2" s="7">
-        <f>COUNTA(Catálogo!A2:A41)</f>
+        <f>COUNTA(Catálogo!A2:A42)</f>
         <v/>
       </c>
     </row>
@@ -25718,7 +26336,7 @@
         </is>
       </c>
       <c r="B3" s="7">
-        <f>COUNTIF(Catálogo!U2:U41,"pendiente")</f>
+        <f>COUNTIF(Catálogo!U2:U42,"pendiente")</f>
         <v/>
       </c>
     </row>
@@ -25729,7 +26347,7 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>COUNTIF(Catálogo!U2:U41,"compuesta")</f>
+        <f>COUNTIF(Catálogo!U2:U42,"compuesta")</f>
         <v/>
       </c>
     </row>
@@ -25740,7 +26358,7 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF(Catálogo!U2:U41,"montada")</f>
+        <f>COUNTIF(Catálogo!U2:U42,"montada")</f>
         <v/>
       </c>
     </row>
@@ -25751,7 +26369,7 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF(Catálogo!U2:U41,"publicada")</f>
+        <f>COUNTIF(Catálogo!U2:U42,"publicada")</f>
         <v/>
       </c>
     </row>
@@ -25791,15 +26409,15 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Catálogo!D2:D41,A10)</f>
+        <f>COUNTIF(Catálogo!D2:D42,A10)</f>
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>COUNTIFS(Catálogo!D2:D41,A10,Catálogo!U2:U41,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D42,A10,Catálogo!U2:U42,"publicada")</f>
         <v/>
       </c>
       <c r="D10" s="7">
-        <f>SUMIF(Catálogo!D2:D41,A10,Catálogo!R2:R41)</f>
+        <f>SUMIF(Catálogo!D2:D42,A10,Catálogo!R2:R42)</f>
         <v/>
       </c>
     </row>
@@ -25810,15 +26428,15 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Catálogo!D2:D41,A11)</f>
+        <f>COUNTIF(Catálogo!D2:D42,A11)</f>
         <v/>
       </c>
       <c r="C11" s="7">
-        <f>COUNTIFS(Catálogo!D2:D41,A11,Catálogo!U2:U41,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D42,A11,Catálogo!U2:U42,"publicada")</f>
         <v/>
       </c>
       <c r="D11" s="7">
-        <f>SUMIF(Catálogo!D2:D41,A11,Catálogo!R2:R41)</f>
+        <f>SUMIF(Catálogo!D2:D42,A11,Catálogo!R2:R42)</f>
         <v/>
       </c>
     </row>
@@ -25829,15 +26447,15 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Catálogo!D2:D41,A12)</f>
+        <f>COUNTIF(Catálogo!D2:D42,A12)</f>
         <v/>
       </c>
       <c r="C12" s="7">
-        <f>COUNTIFS(Catálogo!D2:D41,A12,Catálogo!U2:U41,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D42,A12,Catálogo!U2:U42,"publicada")</f>
         <v/>
       </c>
       <c r="D12" s="7">
-        <f>SUMIF(Catálogo!D2:D41,A12,Catálogo!R2:R41)</f>
+        <f>SUMIF(Catálogo!D2:D42,A12,Catálogo!R2:R42)</f>
         <v/>
       </c>
     </row>
@@ -25848,15 +26466,15 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Catálogo!D2:D41,A13)</f>
+        <f>COUNTIF(Catálogo!D2:D42,A13)</f>
         <v/>
       </c>
       <c r="C13" s="7">
-        <f>COUNTIFS(Catálogo!D2:D41,A13,Catálogo!U2:U41,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D42,A13,Catálogo!U2:U42,"publicada")</f>
         <v/>
       </c>
       <c r="D13" s="7">
-        <f>SUMIF(Catálogo!D2:D41,A13,Catálogo!R2:R41)</f>
+        <f>SUMIF(Catálogo!D2:D42,A13,Catálogo!R2:R42)</f>
         <v/>
       </c>
     </row>
@@ -25867,15 +26485,15 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Catálogo!D2:D41,A14)</f>
+        <f>COUNTIF(Catálogo!D2:D42,A14)</f>
         <v/>
       </c>
       <c r="C14" s="7">
-        <f>COUNTIFS(Catálogo!D2:D41,A14,Catálogo!U2:U41,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D42,A14,Catálogo!U2:U42,"publicada")</f>
         <v/>
       </c>
       <c r="D14" s="7">
-        <f>SUMIF(Catálogo!D2:D41,A14,Catálogo!R2:R41)</f>
+        <f>SUMIF(Catálogo!D2:D42,A14,Catálogo!R2:R42)</f>
         <v/>
       </c>
     </row>
@@ -25912,7 +26530,7 @@
         </is>
       </c>
       <c r="B18" s="7">
-        <f>SUM(Catálogo!W2:W41)</f>
+        <f>SUM(Catálogo!W2:W42)</f>
         <v/>
       </c>
     </row>
@@ -25923,7 +26541,7 @@
         </is>
       </c>
       <c r="B19" s="7">
-        <f>SUM(Catálogo!X2:X41)</f>
+        <f>SUM(Catálogo!X2:X42)</f>
         <v/>
       </c>
     </row>
@@ -26066,7 +26684,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Ambiente aprobado en escucha: mar, mar-aves, zen, selva o lluvia-tambor.</t>
+          <t>Ambiente aprobado en escucha: mar, mar-aves, zen, selva, lluvia-tambor o jardin.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
OBRA-042 «Calm Your Nervous System» (3 h, Zen Temple, 528 Hz) y títulos con la promesa primero
- generar_catalogo.py: PROMESA por obra: título, descripción y etiquetas con la
  promesa primero y las palabras clave de la búsqueda en EE. UU. (análisis del
  27/09); OBRA-041 con lo publicado, OBRA-042 nueva
- OBRA-042: Zen Temple (el ambiente de los Shorts que más retienen), 528 Hz
  shin, 3 horas, tono 35 (bronce, distinto del rojo publicado)
- montar.py: más de 2,5 h va con HEVC crf 33 para no pasar los 2 GB
- shorts_catalogo.py / render_redes.py: el ambiente sale del ambiente y no de
  la posición en el título
- OBRA-041 publicada: https://youtu.be/LRXFSFZO_uI

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$Y$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$288</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$Y$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$295</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y42"/>
+  <dimension ref="A1:Y43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5246,7 +5246,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour</t>
+          <t>Stop Overthinking 🌿 Calming Music for Anxiety · Birdsong &amp; Temple Bells · 432 Hz · 1 Hour</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -5266,15 +5266,12 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Stop Overthinking · 1 Hour
-To accompany a pause when your mind won't stop.
-Ambience: birds and temple bells.
-Composed around a root of 432 Hz, in just intonation, hirajoshi mode.
-Breathing cycle: from 6.0 down to 4.5 breaths per minute, 40 % inhale / 60 % exhale.
-Original composition, synthesized from scratch, ambience included. No third-party samples.
-Best at low volume.
-Subscribe for new pieces: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
-#relaxingmusic #meditation #432hz</t>
+          <t>One hour to stop overthinking. Calming music for anxiety with birdsong and soft temple bells, and a slower breath.
+The music slows from 6 to 4.5 breaths per minute: breathe out longer than you breathe in, and let it lead.
+🎧 Headphones, low volume. You don't have to solve anything tonight. Just listen.
+🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+Original composition by Rin, synthesized from scratch in just intonation around 432 Hz, hirajoshi mode. No samples.
+#calmingmusic #musicforanxiety #432hz</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -5297,16 +5294,20 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>#relaxingmusic #meditation #432hz</t>
+          <t>#calmingmusic #musicforanxiety #432hz</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>music for anxiety, 432 hz, 432 hz music, anxiety relief, stress relief, calming music, birdsong, wind chimes, zen garden, relaxing music, meditation music, ambient music, just intonation, original composition, Rin, música para momentos de ansiedad</t>
+          <t>stop overthinking, stop overthinking music, calming music, music for anxiety, calming music for anxiety, anxiety relief, stress relief music, calm your nervous system, nervous system regulation, relaxing music, meditation music, calm music, birdsong, birds singing, temple bells, wind chimes, zen garden, 432 hz, 432 hz music, rin, música para la ansiedad</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr"/>
-      <c r="L42" s="4" t="inlineStr"/>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>https://youtu.be/LRXFSFZO_uI</t>
+        </is>
+      </c>
       <c r="M42" s="2" t="n">
         <v>432</v>
       </c>
@@ -5341,10 +5342,14 @@
       </c>
       <c r="U42" s="4" t="inlineStr">
         <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V42" s="4" t="inlineStr"/>
+          <t>publicada</t>
+        </is>
+      </c>
+      <c r="V42" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
       <c r="W42" s="4" t="inlineStr"/>
       <c r="X42" s="4" t="inlineStr"/>
       <c r="Y42" s="5">
@@ -5352,8 +5357,119 @@
         <v/>
       </c>
     </row>
+    <row r="43" ht="58" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Música para momentos de ansiedad · Templo zen · 528 Hz · Calmar el sistema nervioso · 3 horas</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Ansiedad</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>zen</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Three hours of calm for an anxious mind and a restless night. Soft zen temple bells over a warm, steady drone.
+The music slows from 6 to 4.5 breaths per minute: breathe out longer than you breathe in, and let your body follow.
+🌙 Play it low while you rest, read, work or fall asleep.
+🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+Original composition by Rin, synthesized from scratch in just intonation around 528 Hz, shin mode. No samples.
+#calmingmusic #sleepmusic #528hz</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Calmar el sistema nervioso · 3 horas
+Para acompañar un momento de pausa cuando la cabeza no para.
+Ambiente: templo zen.
+Compuesta con raíz en 528 Hz, en entonación justa, modo shin.
+Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
+Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#relaxingmusic #meditation #528hz</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>180 MIN</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>#calmingmusic #sleepmusic #528hz</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>calm your nervous system, nervous system regulation, calming music, music for anxiety, anxiety relief, sleep music, meditation for sleep, deep sleep music, stress relief music, zen music, zen temple, temple bells, 528 hz, 528 hz music, relaxing music, meditation music, 3 hours, rin, música para la ansiedad</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr"/>
+      <c r="L43" s="4" t="inlineStr"/>
+      <c r="M43" s="2" t="n">
+        <v>528</v>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>shin</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>medio</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="n">
+        <v>266691</v>
+      </c>
+      <c r="Q43" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="R43" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="S43" s="3" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/compositor.py --minutos 180 --raiz 528 --modo shin --semilla 266691 --caracter sin-cuenco</t>
+        </is>
+      </c>
+      <c r="T43" s="2" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/capas.py zen 10840 audio/OBRA-042_capa.wav --semilla 266691 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-042_528_shin.wav audio/OBRA-042_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-042_capa.wav</t>
+        </is>
+      </c>
+      <c r="U43" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="V43" s="4" t="inlineStr"/>
+      <c r="W43" s="4" t="inlineStr"/>
+      <c r="X43" s="4" t="inlineStr"/>
+      <c r="Y43" s="5">
+        <f>IFERROR(X43/W43*1000,"")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Y42"/>
+  <autoFilter ref="A1:Y43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5364,7 +5480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S288"/>
+  <dimension ref="A1:S295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -25826,7 +25942,8 @@
       <c r="J282" s="3" t="inlineStr">
         <is>
           <t>Save this for the next hard moment.
-Full piece (1 h): Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour
+Full piece (1 h): Stop Overthinking 🌿 Calming Music for Anxiety · Birdsong &amp; Temple Bells · 432 Hz · 1 Hour
+https://youtu.be/LRXFSFZO_uI
 #anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
@@ -25835,7 +25952,11 @@
           <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
         </is>
       </c>
-      <c r="L282" s="2" t="inlineStr"/>
+      <c r="L282" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/LRXFSFZO_uI</t>
+        </is>
+      </c>
       <c r="M282" s="2" t="inlineStr">
         <is>
           <t>432 Hz · calm</t>
@@ -25898,7 +26019,8 @@
       <c r="J283" s="3" t="inlineStr">
         <is>
           <t>Headphones on. Exhale slowly.
-Full piece (1 h): Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour
+Full piece (1 h): Stop Overthinking 🌿 Calming Music for Anxiety · Birdsong &amp; Temple Bells · 432 Hz · 1 Hour
+https://youtu.be/LRXFSFZO_uI
 #anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
@@ -25907,7 +26029,11 @@
           <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
         </is>
       </c>
-      <c r="L283" s="2" t="inlineStr"/>
+      <c r="L283" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/LRXFSFZO_uI</t>
+        </is>
+      </c>
       <c r="M283" s="2" t="inlineStr">
         <is>
           <t>432 Hz · exhale</t>
@@ -25970,7 +26096,8 @@
       <c r="J284" s="3" t="inlineStr">
         <is>
           <t>Stay for one full breath.
-Full piece (1 h): Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour
+Full piece (1 h): Stop Overthinking 🌿 Calming Music for Anxiety · Birdsong &amp; Temple Bells · 432 Hz · 1 Hour
+https://youtu.be/LRXFSFZO_uI
 #anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
@@ -25979,7 +26106,11 @@
           <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
         </is>
       </c>
-      <c r="L284" s="2" t="inlineStr"/>
+      <c r="L284" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/LRXFSFZO_uI</t>
+        </is>
+      </c>
       <c r="M284" s="2" t="inlineStr">
         <is>
           <t>432 Hz · pause</t>
@@ -26042,7 +26173,8 @@
       <c r="J285" s="3" t="inlineStr">
         <is>
           <t>A small pause in the middle of the day.
-Full piece (1 h): Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour
+Full piece (1 h): Stop Overthinking 🌿 Calming Music for Anxiety · Birdsong &amp; Temple Bells · 432 Hz · 1 Hour
+https://youtu.be/LRXFSFZO_uI
 #anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
@@ -26051,7 +26183,11 @@
           <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
         </is>
       </c>
-      <c r="L285" s="2" t="inlineStr"/>
+      <c r="L285" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/LRXFSFZO_uI</t>
+        </is>
+      </c>
       <c r="M285" s="2" t="inlineStr">
         <is>
           <t>432 Hz · breathe</t>
@@ -26114,7 +26250,8 @@
       <c r="J286" s="3" t="inlineStr">
         <is>
           <t>Send this to someone who needs a pause.
-Full piece (1 h): Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour
+Full piece (1 h): Stop Overthinking 🌿 Calming Music for Anxiety · Birdsong &amp; Temple Bells · 432 Hz · 1 Hour
+https://youtu.be/LRXFSFZO_uI
 #anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
@@ -26123,7 +26260,11 @@
           <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
         </is>
       </c>
-      <c r="L286" s="2" t="inlineStr"/>
+      <c r="L286" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/LRXFSFZO_uI</t>
+        </is>
+      </c>
       <c r="M286" s="2" t="inlineStr">
         <is>
           <t>432 Hz · slow down</t>
@@ -26186,7 +26327,8 @@
       <c r="J287" s="3" t="inlineStr">
         <is>
           <t>Breathe with the sound for a moment.
-Full piece (1 h): Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour
+Full piece (1 h): Stop Overthinking 🌿 Calming Music for Anxiety · Birdsong &amp; Temple Bells · 432 Hz · 1 Hour
+https://youtu.be/LRXFSFZO_uI
 #anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
@@ -26195,7 +26337,11 @@
           <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
         </is>
       </c>
-      <c r="L287" s="2" t="inlineStr"/>
+      <c r="L287" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/LRXFSFZO_uI</t>
+        </is>
+      </c>
       <c r="M287" s="2" t="inlineStr">
         <is>
           <t>432 Hz · let go</t>
@@ -26258,7 +26404,8 @@
       <c r="J288" s="3" t="inlineStr">
         <is>
           <t>Come back to this when you need it.
-Full piece (1 h): Music for Anxiety · Birds and Temple Bells · 432 Hz · Stop Overthinking · 1 Hour
+Full piece (1 h): Stop Overthinking 🌿 Calming Music for Anxiety · Birdsong &amp; Temple Bells · 432 Hz · 1 Hour
+https://youtu.be/LRXFSFZO_uI
 #anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
@@ -26267,7 +26414,11 @@
           <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
         </is>
       </c>
-      <c r="L288" s="2" t="inlineStr"/>
+      <c r="L288" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/LRXFSFZO_uI</t>
+        </is>
+      </c>
       <c r="M288" s="2" t="inlineStr">
         <is>
           <t>432 Hz · quiet</t>
@@ -26289,8 +26440,512 @@
       <c r="R288" s="4" t="inlineStr"/>
       <c r="S288" s="4" t="inlineStr"/>
     </row>
+    <row r="289" ht="58" customHeight="1">
+      <c r="A289" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042-S1</t>
+        </is>
+      </c>
+      <c r="B289" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D289" s="2" t="inlineStr">
+        <is>
+          <t>short-1.mp4</t>
+        </is>
+      </c>
+      <c r="E289" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="F289" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G289" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H289" s="2" t="inlineStr">
+        <is>
+          <t>for when your mind won't stop</t>
+        </is>
+      </c>
+      <c r="I289" s="3" t="inlineStr">
+        <is>
+          <t>For when your mind won't stop · 528 Hz · Zen Temple</t>
+        </is>
+      </c>
+      <c r="J289" s="3" t="inlineStr">
+        <is>
+          <t>Save this for the next hard moment.
+Full piece (3 h): Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours
+#anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
+        </is>
+      </c>
+      <c r="K289" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
+        </is>
+      </c>
+      <c r="L289" s="2" t="inlineStr"/>
+      <c r="M289" s="2" t="inlineStr">
+        <is>
+          <t>528 Hz · calm</t>
+        </is>
+      </c>
+      <c r="N289" s="3" t="inlineStr">
+        <is>
+          <t>Save this for the next hard moment. Full 3 h piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #528hz #meditation</t>
+        </is>
+      </c>
+      <c r="O289" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P289" s="4" t="inlineStr"/>
+      <c r="Q289" s="4" t="inlineStr"/>
+      <c r="R289" s="4" t="inlineStr"/>
+      <c r="S289" s="4" t="inlineStr"/>
+    </row>
+    <row r="290" ht="58" customHeight="1">
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042-S2</t>
+        </is>
+      </c>
+      <c r="B290" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042</t>
+        </is>
+      </c>
+      <c r="C290" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D290" s="2" t="inlineStr">
+        <is>
+          <t>short-2.mp4</t>
+        </is>
+      </c>
+      <c r="E290" s="2" t="n">
+        <v>2761</v>
+      </c>
+      <c r="F290" s="2" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G290" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H290" s="2" t="inlineStr">
+        <is>
+          <t>breathe out longer than you breathe in</t>
+        </is>
+      </c>
+      <c r="I290" s="3" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in · 528 Hz · Zen Temple</t>
+        </is>
+      </c>
+      <c r="J290" s="3" t="inlineStr">
+        <is>
+          <t>Headphones on. Exhale slowly.
+Full piece (3 h): Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours
+#anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
+        </is>
+      </c>
+      <c r="K290" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
+        </is>
+      </c>
+      <c r="L290" s="2" t="inlineStr"/>
+      <c r="M290" s="2" t="inlineStr">
+        <is>
+          <t>528 Hz · exhale</t>
+        </is>
+      </c>
+      <c r="N290" s="3" t="inlineStr">
+        <is>
+          <t>Headphones on. Exhale slowly. Full 3 h piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #528hz #meditation</t>
+        </is>
+      </c>
+      <c r="O290" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P290" s="4" t="inlineStr"/>
+      <c r="Q290" s="4" t="inlineStr"/>
+      <c r="R290" s="4" t="inlineStr"/>
+      <c r="S290" s="4" t="inlineStr"/>
+    </row>
+    <row r="291" ht="58" customHeight="1">
+      <c r="A291" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042-S3</t>
+        </is>
+      </c>
+      <c r="B291" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042</t>
+        </is>
+      </c>
+      <c r="C291" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D291" s="2" t="inlineStr">
+        <is>
+          <t>short-3.mp4</t>
+        </is>
+      </c>
+      <c r="E291" s="2" t="n">
+        <v>5432</v>
+      </c>
+      <c r="F291" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G291" s="2" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H291" s="2" t="inlineStr">
+        <is>
+          <t>a pause, just for you</t>
+        </is>
+      </c>
+      <c r="I291" s="3" t="inlineStr">
+        <is>
+          <t>A pause, just for you · 528 Hz · Zen Temple</t>
+        </is>
+      </c>
+      <c r="J291" s="3" t="inlineStr">
+        <is>
+          <t>Stay for one full breath.
+Full piece (3 h): Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours
+#anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
+        </is>
+      </c>
+      <c r="K291" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
+        </is>
+      </c>
+      <c r="L291" s="2" t="inlineStr"/>
+      <c r="M291" s="2" t="inlineStr">
+        <is>
+          <t>528 Hz · pause</t>
+        </is>
+      </c>
+      <c r="N291" s="3" t="inlineStr">
+        <is>
+          <t>Stay for one full breath. Full 3 h piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #528hz #meditation</t>
+        </is>
+      </c>
+      <c r="O291" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P291" s="4" t="inlineStr"/>
+      <c r="Q291" s="4" t="inlineStr"/>
+      <c r="R291" s="4" t="inlineStr"/>
+      <c r="S291" s="4" t="inlineStr"/>
+    </row>
+    <row r="292" ht="58" customHeight="1">
+      <c r="A292" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042-S4</t>
+        </is>
+      </c>
+      <c r="B292" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042</t>
+        </is>
+      </c>
+      <c r="C292" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D292" s="2" t="inlineStr">
+        <is>
+          <t>short-4.mp4</t>
+        </is>
+      </c>
+      <c r="E292" s="2" t="n">
+        <v>8104</v>
+      </c>
+      <c r="F292" s="2" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="G292" s="2" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="H292" s="2" t="inlineStr">
+        <is>
+          <t>slow down, one breath at a time</t>
+        </is>
+      </c>
+      <c r="I292" s="3" t="inlineStr">
+        <is>
+          <t>Slow down, one breath at a time · 528 Hz · Zen Temple</t>
+        </is>
+      </c>
+      <c r="J292" s="3" t="inlineStr">
+        <is>
+          <t>A small pause in the middle of the day.
+Full piece (3 h): Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours
+#anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
+        </is>
+      </c>
+      <c r="K292" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
+        </is>
+      </c>
+      <c r="L292" s="2" t="inlineStr"/>
+      <c r="M292" s="2" t="inlineStr">
+        <is>
+          <t>528 Hz · breathe</t>
+        </is>
+      </c>
+      <c r="N292" s="3" t="inlineStr">
+        <is>
+          <t>A small pause in the middle of the day. Full 3 h piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #528hz #meditation</t>
+        </is>
+      </c>
+      <c r="O292" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P292" s="4" t="inlineStr"/>
+      <c r="Q292" s="4" t="inlineStr"/>
+      <c r="R292" s="4" t="inlineStr"/>
+      <c r="S292" s="4" t="inlineStr"/>
+    </row>
+    <row r="293" ht="58" customHeight="1">
+      <c r="A293" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042-S5</t>
+        </is>
+      </c>
+      <c r="B293" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042</t>
+        </is>
+      </c>
+      <c r="C293" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D293" s="2" t="inlineStr">
+        <is>
+          <t>short-5.mp4</t>
+        </is>
+      </c>
+      <c r="E293" s="2" t="n">
+        <v>10775</v>
+      </c>
+      <c r="F293" s="2" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="G293" s="2" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="H293" s="2" t="inlineStr">
+        <is>
+          <t>before you begin</t>
+        </is>
+      </c>
+      <c r="I293" s="3" t="inlineStr">
+        <is>
+          <t>Before you begin · 528 Hz · Zen Temple</t>
+        </is>
+      </c>
+      <c r="J293" s="3" t="inlineStr">
+        <is>
+          <t>Send this to someone who needs a pause.
+Full piece (3 h): Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours
+#anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
+        </is>
+      </c>
+      <c r="K293" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
+        </is>
+      </c>
+      <c r="L293" s="2" t="inlineStr"/>
+      <c r="M293" s="2" t="inlineStr">
+        <is>
+          <t>528 Hz · slow down</t>
+        </is>
+      </c>
+      <c r="N293" s="3" t="inlineStr">
+        <is>
+          <t>Send this to someone who needs a pause. Full 3 h piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #528hz #meditation</t>
+        </is>
+      </c>
+      <c r="O293" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P293" s="4" t="inlineStr"/>
+      <c r="Q293" s="4" t="inlineStr"/>
+      <c r="R293" s="4" t="inlineStr"/>
+      <c r="S293" s="4" t="inlineStr"/>
+    </row>
+    <row r="294" ht="58" customHeight="1">
+      <c r="A294" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042-S6</t>
+        </is>
+      </c>
+      <c r="B294" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042</t>
+        </is>
+      </c>
+      <c r="C294" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D294" s="2" t="inlineStr">
+        <is>
+          <t>short-6.mp4</t>
+        </is>
+      </c>
+      <c r="E294" s="2" t="n">
+        <v>1426</v>
+      </c>
+      <c r="F294" s="2" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="G294" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H294" s="2" t="inlineStr">
+        <is>
+          <t>you can put it down for now</t>
+        </is>
+      </c>
+      <c r="I294" s="3" t="inlineStr">
+        <is>
+          <t>You can put it down for now · 528 Hz · Zen Temple</t>
+        </is>
+      </c>
+      <c r="J294" s="3" t="inlineStr">
+        <is>
+          <t>Breathe with the sound for a moment.
+Full piece (3 h): Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours
+#anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
+        </is>
+      </c>
+      <c r="K294" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
+        </is>
+      </c>
+      <c r="L294" s="2" t="inlineStr"/>
+      <c r="M294" s="2" t="inlineStr">
+        <is>
+          <t>528 Hz · let go</t>
+        </is>
+      </c>
+      <c r="N294" s="3" t="inlineStr">
+        <is>
+          <t>Breathe with the sound for a moment. Full 3 h piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #528hz #meditation</t>
+        </is>
+      </c>
+      <c r="O294" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P294" s="4" t="inlineStr"/>
+      <c r="Q294" s="4" t="inlineStr"/>
+      <c r="R294" s="4" t="inlineStr"/>
+      <c r="S294" s="4" t="inlineStr"/>
+    </row>
+    <row r="295" ht="58" customHeight="1">
+      <c r="A295" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042-S7</t>
+        </is>
+      </c>
+      <c r="B295" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-042</t>
+        </is>
+      </c>
+      <c r="C295" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D295" s="2" t="inlineStr">
+        <is>
+          <t>short-7.mp4</t>
+        </is>
+      </c>
+      <c r="E295" s="2" t="n">
+        <v>6768</v>
+      </c>
+      <c r="F295" s="2" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G295" s="2" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="H295" s="2" t="inlineStr">
+        <is>
+          <t>one minute of quiet</t>
+        </is>
+      </c>
+      <c r="I295" s="3" t="inlineStr">
+        <is>
+          <t>One minute of quiet · 528 Hz · Zen Temple</t>
+        </is>
+      </c>
+      <c r="J295" s="3" t="inlineStr">
+        <is>
+          <t>Come back to this when you need it.
+Full piece (3 h): Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours
+#anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
+        </is>
+      </c>
+      <c r="K295" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
+        </is>
+      </c>
+      <c r="L295" s="2" t="inlineStr"/>
+      <c r="M295" s="2" t="inlineStr">
+        <is>
+          <t>528 Hz · quiet</t>
+        </is>
+      </c>
+      <c r="N295" s="3" t="inlineStr">
+        <is>
+          <t>Come back to this when you need it. Full 3 h piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #528hz #meditation</t>
+        </is>
+      </c>
+      <c r="O295" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P295" s="4" t="inlineStr"/>
+      <c r="Q295" s="4" t="inlineStr"/>
+      <c r="R295" s="4" t="inlineStr"/>
+      <c r="S295" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S288"/>
+  <autoFilter ref="A1:S295"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26325,7 +26980,7 @@
         </is>
       </c>
       <c r="B2" s="7">
-        <f>COUNTA(Catálogo!A2:A42)</f>
+        <f>COUNTA(Catálogo!A2:A43)</f>
         <v/>
       </c>
     </row>
@@ -26336,7 +26991,7 @@
         </is>
       </c>
       <c r="B3" s="7">
-        <f>COUNTIF(Catálogo!U2:U42,"pendiente")</f>
+        <f>COUNTIF(Catálogo!U2:U43,"pendiente")</f>
         <v/>
       </c>
     </row>
@@ -26347,7 +27002,7 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>COUNTIF(Catálogo!U2:U42,"compuesta")</f>
+        <f>COUNTIF(Catálogo!U2:U43,"compuesta")</f>
         <v/>
       </c>
     </row>
@@ -26358,7 +27013,7 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF(Catálogo!U2:U42,"montada")</f>
+        <f>COUNTIF(Catálogo!U2:U43,"montada")</f>
         <v/>
       </c>
     </row>
@@ -26369,7 +27024,7 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF(Catálogo!U2:U42,"publicada")</f>
+        <f>COUNTIF(Catálogo!U2:U43,"publicada")</f>
         <v/>
       </c>
     </row>
@@ -26409,15 +27064,15 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Catálogo!D2:D42,A10)</f>
+        <f>COUNTIF(Catálogo!D2:D43,A10)</f>
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>COUNTIFS(Catálogo!D2:D42,A10,Catálogo!U2:U42,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D43,A10,Catálogo!U2:U43,"publicada")</f>
         <v/>
       </c>
       <c r="D10" s="7">
-        <f>SUMIF(Catálogo!D2:D42,A10,Catálogo!R2:R42)</f>
+        <f>SUMIF(Catálogo!D2:D43,A10,Catálogo!R2:R43)</f>
         <v/>
       </c>
     </row>
@@ -26428,15 +27083,15 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Catálogo!D2:D42,A11)</f>
+        <f>COUNTIF(Catálogo!D2:D43,A11)</f>
         <v/>
       </c>
       <c r="C11" s="7">
-        <f>COUNTIFS(Catálogo!D2:D42,A11,Catálogo!U2:U42,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D43,A11,Catálogo!U2:U43,"publicada")</f>
         <v/>
       </c>
       <c r="D11" s="7">
-        <f>SUMIF(Catálogo!D2:D42,A11,Catálogo!R2:R42)</f>
+        <f>SUMIF(Catálogo!D2:D43,A11,Catálogo!R2:R43)</f>
         <v/>
       </c>
     </row>
@@ -26447,15 +27102,15 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Catálogo!D2:D42,A12)</f>
+        <f>COUNTIF(Catálogo!D2:D43,A12)</f>
         <v/>
       </c>
       <c r="C12" s="7">
-        <f>COUNTIFS(Catálogo!D2:D42,A12,Catálogo!U2:U42,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D43,A12,Catálogo!U2:U43,"publicada")</f>
         <v/>
       </c>
       <c r="D12" s="7">
-        <f>SUMIF(Catálogo!D2:D42,A12,Catálogo!R2:R42)</f>
+        <f>SUMIF(Catálogo!D2:D43,A12,Catálogo!R2:R43)</f>
         <v/>
       </c>
     </row>
@@ -26466,15 +27121,15 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Catálogo!D2:D42,A13)</f>
+        <f>COUNTIF(Catálogo!D2:D43,A13)</f>
         <v/>
       </c>
       <c r="C13" s="7">
-        <f>COUNTIFS(Catálogo!D2:D42,A13,Catálogo!U2:U42,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D43,A13,Catálogo!U2:U43,"publicada")</f>
         <v/>
       </c>
       <c r="D13" s="7">
-        <f>SUMIF(Catálogo!D2:D42,A13,Catálogo!R2:R42)</f>
+        <f>SUMIF(Catálogo!D2:D43,A13,Catálogo!R2:R43)</f>
         <v/>
       </c>
     </row>
@@ -26485,15 +27140,15 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Catálogo!D2:D42,A14)</f>
+        <f>COUNTIF(Catálogo!D2:D43,A14)</f>
         <v/>
       </c>
       <c r="C14" s="7">
-        <f>COUNTIFS(Catálogo!D2:D42,A14,Catálogo!U2:U42,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D43,A14,Catálogo!U2:U43,"publicada")</f>
         <v/>
       </c>
       <c r="D14" s="7">
-        <f>SUMIF(Catálogo!D2:D42,A14,Catálogo!R2:R42)</f>
+        <f>SUMIF(Catálogo!D2:D43,A14,Catálogo!R2:R43)</f>
         <v/>
       </c>
     </row>
@@ -26530,7 +27185,7 @@
         </is>
       </c>
       <c r="B18" s="7">
-        <f>SUM(Catálogo!W2:W42)</f>
+        <f>SUM(Catálogo!W2:W43)</f>
         <v/>
       </c>
     </row>
@@ -26541,7 +27196,7 @@
         </is>
       </c>
       <c r="B19" s="7">
-        <f>SUM(Catálogo!X2:X42)</f>
+        <f>SUM(Catálogo!X2:X43)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
OBRA-042 publicada (tt0cPixnquE) y TikTok «Calm your nervous system», 3 min
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -5422,7 +5422,11 @@
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr"/>
-      <c r="L43" s="4" t="inlineStr"/>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>https://youtu.be/tt0cPixnquE</t>
+        </is>
+      </c>
       <c r="M43" s="2" t="n">
         <v>528</v>
       </c>
@@ -5457,10 +5461,14 @@
       </c>
       <c r="U43" s="4" t="inlineStr">
         <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V43" s="4" t="inlineStr"/>
+          <t>publicada</t>
+        </is>
+      </c>
+      <c r="V43" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="W43" s="4" t="inlineStr"/>
       <c r="X43" s="4" t="inlineStr"/>
       <c r="Y43" s="5">
@@ -26482,6 +26490,7 @@
         <is>
           <t>Save this for the next hard moment.
 Full piece (3 h): Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours
+https://youtu.be/tt0cPixnquE
 #anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
         </is>
       </c>
@@ -26490,7 +26499,11 @@
           <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
         </is>
       </c>
-      <c r="L289" s="2" t="inlineStr"/>
+      <c r="L289" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/tt0cPixnquE</t>
+        </is>
+      </c>
       <c r="M289" s="2" t="inlineStr">
         <is>
           <t>528 Hz · calm</t>
@@ -26554,6 +26567,7 @@
         <is>
           <t>Headphones on. Exhale slowly.
 Full piece (3 h): Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours
+https://youtu.be/tt0cPixnquE
 #anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
         </is>
       </c>
@@ -26562,7 +26576,11 @@
           <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
         </is>
       </c>
-      <c r="L290" s="2" t="inlineStr"/>
+      <c r="L290" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/tt0cPixnquE</t>
+        </is>
+      </c>
       <c r="M290" s="2" t="inlineStr">
         <is>
           <t>528 Hz · exhale</t>
@@ -26626,6 +26644,7 @@
         <is>
           <t>Stay for one full breath.
 Full piece (3 h): Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours
+https://youtu.be/tt0cPixnquE
 #anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
         </is>
       </c>
@@ -26634,7 +26653,11 @@
           <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
         </is>
       </c>
-      <c r="L291" s="2" t="inlineStr"/>
+      <c r="L291" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/tt0cPixnquE</t>
+        </is>
+      </c>
       <c r="M291" s="2" t="inlineStr">
         <is>
           <t>528 Hz · pause</t>
@@ -26698,6 +26721,7 @@
         <is>
           <t>A small pause in the middle of the day.
 Full piece (3 h): Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours
+https://youtu.be/tt0cPixnquE
 #anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
         </is>
       </c>
@@ -26706,7 +26730,11 @@
           <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
         </is>
       </c>
-      <c r="L292" s="2" t="inlineStr"/>
+      <c r="L292" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/tt0cPixnquE</t>
+        </is>
+      </c>
       <c r="M292" s="2" t="inlineStr">
         <is>
           <t>528 Hz · breathe</t>
@@ -26770,6 +26798,7 @@
         <is>
           <t>Send this to someone who needs a pause.
 Full piece (3 h): Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours
+https://youtu.be/tt0cPixnquE
 #anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
         </is>
       </c>
@@ -26778,7 +26807,11 @@
           <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
         </is>
       </c>
-      <c r="L293" s="2" t="inlineStr"/>
+      <c r="L293" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/tt0cPixnquE</t>
+        </is>
+      </c>
       <c r="M293" s="2" t="inlineStr">
         <is>
           <t>528 Hz · slow down</t>
@@ -26842,6 +26875,7 @@
         <is>
           <t>Breathe with the sound for a moment.
 Full piece (3 h): Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours
+https://youtu.be/tt0cPixnquE
 #anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
         </is>
       </c>
@@ -26850,7 +26884,11 @@
           <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
         </is>
       </c>
-      <c r="L294" s="2" t="inlineStr"/>
+      <c r="L294" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/tt0cPixnquE</t>
+        </is>
+      </c>
       <c r="M294" s="2" t="inlineStr">
         <is>
           <t>528 Hz · let go</t>
@@ -26914,6 +26952,7 @@
         <is>
           <t>Come back to this when you need it.
 Full piece (3 h): Calm Your Nervous System 🌿 Zen Temple Bells · 528 Hz · Music for Anxiety &amp; Sleep · 3 Hours
+https://youtu.be/tt0cPixnquE
 #anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
         </is>
       </c>
@@ -26922,7 +26961,11 @@
           <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
         </is>
       </c>
-      <c r="L295" s="2" t="inlineStr"/>
+      <c r="L295" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/tt0cPixnquE</t>
+        </is>
+      </c>
       <c r="M295" s="2" t="inlineStr">
         <is>
           <t>528 Hz · quiet</t>

</xml_diff>

<commit_message>
OBRA-043: Dark Screen Sleep Music (lluvia suave, pantalla negra a los 3 min) y 3 Shorts por obra desde la 43
La tendencia que más crece en el nicho (vidIQ, 29/09): «dark screen sleep music»
+269 % en un mes, 54 % EE. UU., competencia baja. Los videos que explotan en
canales chicos de EE. UU. son pantalla negra, lluvia y «fall asleep fast».

- ambiente.py: fondo «lluvia», sin tambor ni pulso, la receta de tao.py
- montar.py: pantalla_oscura(): mandala 3 min, fundido de 30 s y negro
  repetido sin recodificar (el archivo pesa mucho menos)
- mandala: paleta «lluvia», azul pizarra de noche, olas cada 16 s
- miniatura: la promesa en grande (variante D) para la 43
- Shorts: 3 por obra desde la 43 (principio, medio y final); las 42 anteriores
  siguen con 7, ya armados y en la cola

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$Y$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$295</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$Z$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$298</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y43"/>
+  <dimension ref="A1:Z44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -510,13 +510,14 @@
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="6" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="62" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
     <col width="62" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="10" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
-    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="62" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -612,35 +613,40 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>pantalla_oscura_min</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>comando_regeneracion</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>comando_ambiente</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>estado</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>fecha_publicacion</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>vistas</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>suscriptores</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>subs_por_1000</t>
         </is>
@@ -737,26 +743,29 @@
       <c r="R2" s="2" t="n">
         <v>180</v>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="S2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 432 --modo shin --semilla 505716 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T2" s="2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-001_432_shin.wav audio/OBRA-001_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="U2" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V2" s="4" t="inlineStr"/>
+      <c r="V2" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W2" s="4" t="inlineStr"/>
       <c r="X2" s="4" t="inlineStr"/>
-      <c r="Y2" s="5">
-        <f>IFERROR(X2/W2*1000,"")</f>
+      <c r="Y2" s="4" t="inlineStr"/>
+      <c r="Z2" s="5">
+        <f>IFERROR(Y2/X2*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -851,26 +860,29 @@
       <c r="R3" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="S3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 528 --modo kumoi --semilla 443547 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T3" s="2" t="inlineStr">
+      <c r="U3" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-002_528_kumoi.wav audio/OBRA-002_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="U3" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V3" s="4" t="inlineStr"/>
+      <c r="V3" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W3" s="4" t="inlineStr"/>
       <c r="X3" s="4" t="inlineStr"/>
-      <c r="Y3" s="5">
-        <f>IFERROR(X3/W3*1000,"")</f>
+      <c r="Y3" s="4" t="inlineStr"/>
+      <c r="Z3" s="5">
+        <f>IFERROR(Y3/X3*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -965,26 +977,29 @@
       <c r="R4" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="S4" s="3" t="inlineStr">
+      <c r="S4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 396 --modo kumoi --semilla 692584 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T4" s="2" t="inlineStr">
+      <c r="U4" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-003_396_kumoi.wav audio/OBRA-003_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="U4" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V4" s="4" t="inlineStr"/>
+      <c r="V4" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W4" s="4" t="inlineStr"/>
       <c r="X4" s="4" t="inlineStr"/>
-      <c r="Y4" s="5">
-        <f>IFERROR(X4/W4*1000,"")</f>
+      <c r="Y4" s="4" t="inlineStr"/>
+      <c r="Z4" s="5">
+        <f>IFERROR(Y4/X4*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1079,26 +1094,29 @@
       <c r="R5" s="2" t="n">
         <v>180</v>
       </c>
-      <c r="S5" s="3" t="inlineStr">
+      <c r="S5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 528 --modo shin --semilla 751043 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T5" s="2" t="inlineStr">
+      <c r="U5" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-004_528_shin.wav audio/OBRA-004_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="U5" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V5" s="4" t="inlineStr"/>
+      <c r="V5" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W5" s="4" t="inlineStr"/>
       <c r="X5" s="4" t="inlineStr"/>
-      <c r="Y5" s="5">
-        <f>IFERROR(X5/W5*1000,"")</f>
+      <c r="Y5" s="4" t="inlineStr"/>
+      <c r="Z5" s="5">
+        <f>IFERROR(Y5/X5*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1193,26 +1211,29 @@
       <c r="R6" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="S6" s="3" t="inlineStr">
+      <c r="S6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 432 --modo kumoi --semilla 531725 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T6" s="2" t="inlineStr">
+      <c r="U6" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-005_432_kumoi.wav audio/OBRA-005_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="U6" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V6" s="4" t="inlineStr"/>
+      <c r="V6" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W6" s="4" t="inlineStr"/>
       <c r="X6" s="4" t="inlineStr"/>
-      <c r="Y6" s="5">
-        <f>IFERROR(X6/W6*1000,"")</f>
+      <c r="Y6" s="4" t="inlineStr"/>
+      <c r="Z6" s="5">
+        <f>IFERROR(Y6/X6*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1311,30 +1332,33 @@
       <c r="R7" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="S7" s="3" t="inlineStr">
+      <c r="S7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 90 --raiz 417 --modo kumoi --semilla 813147 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T7" s="2" t="inlineStr">
+      <c r="U7" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-006_417_kumoi.wav audio/OBRA-006_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="U7" s="4" t="inlineStr">
+      <c r="V7" s="4" t="inlineStr">
         <is>
           <t>publicada</t>
         </is>
       </c>
-      <c r="V7" s="4" t="inlineStr">
+      <c r="W7" s="4" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="W7" s="4" t="inlineStr"/>
       <c r="X7" s="4" t="inlineStr"/>
-      <c r="Y7" s="5">
-        <f>IFERROR(X7/W7*1000,"")</f>
+      <c r="Y7" s="4" t="inlineStr"/>
+      <c r="Z7" s="5">
+        <f>IFERROR(Y7/X7*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1429,26 +1453,29 @@
       <c r="R8" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="S8" s="3" t="inlineStr">
+      <c r="S8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 396 --modo shin --semilla 885916 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T8" s="2" t="inlineStr">
+      <c r="U8" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-007_396_shin.wav audio/OBRA-007_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="U8" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V8" s="4" t="inlineStr"/>
+      <c r="V8" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W8" s="4" t="inlineStr"/>
       <c r="X8" s="4" t="inlineStr"/>
-      <c r="Y8" s="5">
-        <f>IFERROR(X8/W8*1000,"")</f>
+      <c r="Y8" s="4" t="inlineStr"/>
+      <c r="Z8" s="5">
+        <f>IFERROR(Y8/X8*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1543,26 +1570,29 @@
       <c r="R9" s="2" t="n">
         <v>180</v>
       </c>
-      <c r="S9" s="3" t="inlineStr">
+      <c r="S9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 432 --modo kumoi --semilla 295910 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T9" s="2" t="inlineStr">
+      <c r="U9" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-008_432_kumoi.wav audio/OBRA-008_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="U9" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V9" s="4" t="inlineStr"/>
+      <c r="V9" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W9" s="4" t="inlineStr"/>
       <c r="X9" s="4" t="inlineStr"/>
-      <c r="Y9" s="5">
-        <f>IFERROR(X9/W9*1000,"")</f>
+      <c r="Y9" s="4" t="inlineStr"/>
+      <c r="Z9" s="5">
+        <f>IFERROR(Y9/X9*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1657,26 +1687,29 @@
       <c r="R10" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="S10" s="3" t="inlineStr">
+      <c r="S10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 25 --raiz 396 --modo kumoi --semilla 555819 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T10" s="2" t="inlineStr">
+      <c r="U10" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 1540 audio/OBRA-009_capa.wav --semilla 555819 --raiz 396 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-009_396_kumoi.wav audio/OBRA-009_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-009_capa.wav</t>
         </is>
       </c>
-      <c r="U10" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V10" s="4" t="inlineStr"/>
+      <c r="V10" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W10" s="4" t="inlineStr"/>
       <c r="X10" s="4" t="inlineStr"/>
-      <c r="Y10" s="5">
-        <f>IFERROR(X10/W10*1000,"")</f>
+      <c r="Y10" s="4" t="inlineStr"/>
+      <c r="Z10" s="5">
+        <f>IFERROR(Y10/X10*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1771,26 +1804,29 @@
       <c r="R11" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="S11" s="3" t="inlineStr">
+      <c r="S11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 30 --raiz 432 --modo hirajoshi --semilla 739461 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T11" s="2" t="inlineStr">
+      <c r="U11" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 1840 audio/OBRA-010_capa.wav --semilla 739461 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-010_432_hirajoshi.wav audio/OBRA-010_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-010_capa.wav</t>
         </is>
       </c>
-      <c r="U11" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V11" s="4" t="inlineStr"/>
+      <c r="V11" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W11" s="4" t="inlineStr"/>
       <c r="X11" s="4" t="inlineStr"/>
-      <c r="Y11" s="5">
-        <f>IFERROR(X11/W11*1000,"")</f>
+      <c r="Y11" s="4" t="inlineStr"/>
+      <c r="Z11" s="5">
+        <f>IFERROR(Y11/X11*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1885,26 +1921,29 @@
       <c r="R12" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="S12" s="3" t="inlineStr">
+      <c r="S12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 20 --raiz 528 --modo hirajoshi --semilla 913368 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T12" s="2" t="inlineStr">
+      <c r="U12" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 1240 audio/OBRA-011_capa.wav --semilla 913368 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-011_528_hirajoshi.wav audio/OBRA-011_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-011_capa.wav</t>
         </is>
       </c>
-      <c r="U12" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V12" s="4" t="inlineStr"/>
+      <c r="V12" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W12" s="4" t="inlineStr"/>
       <c r="X12" s="4" t="inlineStr"/>
-      <c r="Y12" s="5">
-        <f>IFERROR(X12/W12*1000,"")</f>
+      <c r="Y12" s="4" t="inlineStr"/>
+      <c r="Z12" s="5">
+        <f>IFERROR(Y12/X12*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2003,30 +2042,33 @@
       <c r="R13" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="S13" s="3" t="inlineStr">
+      <c r="S13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 10 --raiz 528 --modo shin --semilla 43734 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T13" s="2" t="inlineStr">
+      <c r="U13" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 640 audio/OBRA-012_capa.wav --semilla 43734 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-012_528_shin.wav audio/OBRA-012_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-012_capa.wav</t>
         </is>
       </c>
-      <c r="U13" s="4" t="inlineStr">
+      <c r="V13" s="4" t="inlineStr">
         <is>
           <t>publicada</t>
         </is>
       </c>
-      <c r="V13" s="4" t="inlineStr">
+      <c r="W13" s="4" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="W13" s="4" t="inlineStr"/>
       <c r="X13" s="4" t="inlineStr"/>
-      <c r="Y13" s="5">
-        <f>IFERROR(X13/W13*1000,"")</f>
+      <c r="Y13" s="4" t="inlineStr"/>
+      <c r="Z13" s="5">
+        <f>IFERROR(Y13/X13*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2121,26 +2163,29 @@
       <c r="R14" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="S14" s="3" t="inlineStr">
+      <c r="S14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 20 --raiz 432 --modo hirajoshi --semilla 627771 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T14" s="2" t="inlineStr">
+      <c r="U14" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 1240 audio/OBRA-013_capa.wav --semilla 627771 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-013_432_hirajoshi.wav audio/OBRA-013_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-013_capa.wav</t>
         </is>
       </c>
-      <c r="U14" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V14" s="4" t="inlineStr"/>
+      <c r="V14" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W14" s="4" t="inlineStr"/>
       <c r="X14" s="4" t="inlineStr"/>
-      <c r="Y14" s="5">
-        <f>IFERROR(X14/W14*1000,"")</f>
+      <c r="Y14" s="4" t="inlineStr"/>
+      <c r="Z14" s="5">
+        <f>IFERROR(Y14/X14*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2235,26 +2280,29 @@
       <c r="R15" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="S15" s="3" t="inlineStr">
+      <c r="S15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 20 --raiz 528 --modo yo --semilla 310137 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T15" s="2" t="inlineStr">
+      <c r="U15" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-014_capa.wav --semilla 310137 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-014_528_yo.wav audio/OBRA-014_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-014_capa.wav</t>
         </is>
       </c>
-      <c r="U15" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V15" s="4" t="inlineStr"/>
+      <c r="V15" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W15" s="4" t="inlineStr"/>
       <c r="X15" s="4" t="inlineStr"/>
-      <c r="Y15" s="5">
-        <f>IFERROR(X15/W15*1000,"")</f>
+      <c r="Y15" s="4" t="inlineStr"/>
+      <c r="Z15" s="5">
+        <f>IFERROR(Y15/X15*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2353,30 +2401,33 @@
       <c r="R16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="S16" s="3" t="inlineStr">
+      <c r="S16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 15 --raiz 639 --modo yo --semilla 592463 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T16" s="2" t="inlineStr">
+      <c r="U16" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 940 audio/OBRA-015_capa.wav --semilla 592463 --raiz 639 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-015_639_yo.wav audio/OBRA-015_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-015_capa.wav</t>
         </is>
       </c>
-      <c r="U16" s="4" t="inlineStr">
+      <c r="V16" s="4" t="inlineStr">
         <is>
           <t>publicada</t>
         </is>
       </c>
-      <c r="V16" s="4" t="inlineStr">
+      <c r="W16" s="4" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="W16" s="4" t="inlineStr"/>
       <c r="X16" s="4" t="inlineStr"/>
-      <c r="Y16" s="5">
-        <f>IFERROR(X16/W16*1000,"")</f>
+      <c r="Y16" s="4" t="inlineStr"/>
+      <c r="Z16" s="5">
+        <f>IFERROR(Y16/X16*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2471,26 +2522,29 @@
       <c r="R17" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="S17" s="3" t="inlineStr">
+      <c r="S17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 30 --raiz 417 --modo kumoi --semilla 250697 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T17" s="2" t="inlineStr">
+      <c r="U17" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py ancestral 1840 audio/OBRA-016_capa.wav --semilla 250697 --raiz 417 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-016_417_kumoi.wav audio/OBRA-016_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-016_capa.wav</t>
         </is>
       </c>
-      <c r="U17" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V17" s="4" t="inlineStr"/>
+      <c r="V17" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W17" s="4" t="inlineStr"/>
       <c r="X17" s="4" t="inlineStr"/>
-      <c r="Y17" s="5">
-        <f>IFERROR(X17/W17*1000,"")</f>
+      <c r="Y17" s="4" t="inlineStr"/>
+      <c r="Z17" s="5">
+        <f>IFERROR(Y17/X17*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2585,26 +2639,29 @@
       <c r="R18" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="S18" s="3" t="inlineStr">
+      <c r="S18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 45 --raiz 417 --modo hirajoshi --semilla 714152 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T18" s="2" t="inlineStr">
+      <c r="U18" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-017_capa.wav --semilla 714152 --raiz 417 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-017_417_hirajoshi.wav audio/OBRA-017_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-017_capa.wav</t>
         </is>
       </c>
-      <c r="U18" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V18" s="4" t="inlineStr"/>
+      <c r="V18" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W18" s="4" t="inlineStr"/>
       <c r="X18" s="4" t="inlineStr"/>
-      <c r="Y18" s="5">
-        <f>IFERROR(X18/W18*1000,"")</f>
+      <c r="Y18" s="4" t="inlineStr"/>
+      <c r="Z18" s="5">
+        <f>IFERROR(Y18/X18*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2699,26 +2756,29 @@
       <c r="R19" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="S19" s="3" t="inlineStr">
+      <c r="S19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 45 --raiz 528 --modo hirajoshi --semilla 735455 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T19" s="2" t="inlineStr">
+      <c r="U19" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-018_capa.wav --semilla 735455 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-018_528_hirajoshi.wav audio/OBRA-018_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-018_capa.wav</t>
         </is>
       </c>
-      <c r="U19" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V19" s="4" t="inlineStr"/>
+      <c r="V19" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W19" s="4" t="inlineStr"/>
       <c r="X19" s="4" t="inlineStr"/>
-      <c r="Y19" s="5">
-        <f>IFERROR(X19/W19*1000,"")</f>
+      <c r="Y19" s="4" t="inlineStr"/>
+      <c r="Z19" s="5">
+        <f>IFERROR(Y19/X19*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2813,26 +2873,29 @@
       <c r="R20" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="S20" s="3" t="inlineStr">
+      <c r="S20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 432 --modo shin --semilla 627577 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T20" s="2" t="inlineStr">
+      <c r="U20" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-019_capa.wav --semilla 627577 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-019_432_shin.wav audio/OBRA-019_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-019_capa.wav</t>
         </is>
       </c>
-      <c r="U20" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V20" s="4" t="inlineStr"/>
+      <c r="V20" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W20" s="4" t="inlineStr"/>
       <c r="X20" s="4" t="inlineStr"/>
-      <c r="Y20" s="5">
-        <f>IFERROR(X20/W20*1000,"")</f>
+      <c r="Y20" s="4" t="inlineStr"/>
+      <c r="Z20" s="5">
+        <f>IFERROR(Y20/X20*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2931,30 +2994,33 @@
       <c r="R21" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="S21" s="3" t="inlineStr">
+      <c r="S21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 30 --raiz 528 --modo shin --semilla 632595 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T21" s="2" t="inlineStr">
+      <c r="U21" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py ancestral 1840 audio/OBRA-020_capa.wav --semilla 632595 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-020_528_shin.wav audio/OBRA-020_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-020_capa.wav</t>
         </is>
       </c>
-      <c r="U21" s="4" t="inlineStr">
+      <c r="V21" s="4" t="inlineStr">
         <is>
           <t>publicada</t>
         </is>
       </c>
-      <c r="V21" s="4" t="inlineStr">
+      <c r="W21" s="4" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="W21" s="4" t="inlineStr"/>
       <c r="X21" s="4" t="inlineStr"/>
-      <c r="Y21" s="5">
-        <f>IFERROR(X21/W21*1000,"")</f>
+      <c r="Y21" s="4" t="inlineStr"/>
+      <c r="Z21" s="5">
+        <f>IFERROR(Y21/X21*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3049,26 +3115,29 @@
       <c r="R22" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="S22" s="3" t="inlineStr">
+      <c r="S22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 45 --raiz 396 --modo kumoi --semilla 864630 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T22" s="2" t="inlineStr">
+      <c r="U22" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-021_capa.wav --semilla 864630 --raiz 396 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-021_396_kumoi.wav audio/OBRA-021_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-021_capa.wav</t>
         </is>
       </c>
-      <c r="U22" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V22" s="4" t="inlineStr"/>
+      <c r="V22" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W22" s="4" t="inlineStr"/>
       <c r="X22" s="4" t="inlineStr"/>
-      <c r="Y22" s="5">
-        <f>IFERROR(X22/W22*1000,"")</f>
+      <c r="Y22" s="4" t="inlineStr"/>
+      <c r="Z22" s="5">
+        <f>IFERROR(Y22/X22*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3163,26 +3232,29 @@
       <c r="R23" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="S23" s="3" t="inlineStr">
+      <c r="S23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T23" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 639 --modo yo --semilla 335798 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T23" s="2" t="inlineStr">
+      <c r="U23" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-022_capa.wav --semilla 335798 --raiz 639 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-022_639_yo.wav audio/OBRA-022_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-022_capa.wav</t>
         </is>
       </c>
-      <c r="U23" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V23" s="4" t="inlineStr"/>
+      <c r="V23" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W23" s="4" t="inlineStr"/>
       <c r="X23" s="4" t="inlineStr"/>
-      <c r="Y23" s="5">
-        <f>IFERROR(X23/W23*1000,"")</f>
+      <c r="Y23" s="4" t="inlineStr"/>
+      <c r="Z23" s="5">
+        <f>IFERROR(Y23/X23*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3277,26 +3349,29 @@
       <c r="R24" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="S24" s="3" t="inlineStr">
+      <c r="S24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T24" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 20 --raiz 528 --modo shin --semilla 299306 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T24" s="2" t="inlineStr">
+      <c r="U24" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-023_capa.wav --semilla 299306 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-023_528_shin.wav audio/OBRA-023_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-023_capa.wav</t>
         </is>
       </c>
-      <c r="U24" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V24" s="4" t="inlineStr"/>
+      <c r="V24" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W24" s="4" t="inlineStr"/>
       <c r="X24" s="4" t="inlineStr"/>
-      <c r="Y24" s="5">
-        <f>IFERROR(X24/W24*1000,"")</f>
+      <c r="Y24" s="4" t="inlineStr"/>
+      <c r="Z24" s="5">
+        <f>IFERROR(Y24/X24*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3391,26 +3466,29 @@
       <c r="R25" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="S25" s="3" t="inlineStr">
+      <c r="S25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T25" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 432 --modo kumoi --semilla 926202 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T25" s="2" t="inlineStr">
+      <c r="U25" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py ancestral 3640 audio/OBRA-024_capa.wav --semilla 926202 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-024_432_kumoi.wav audio/OBRA-024_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-024_capa.wav</t>
         </is>
       </c>
-      <c r="U25" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V25" s="4" t="inlineStr"/>
+      <c r="V25" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W25" s="4" t="inlineStr"/>
       <c r="X25" s="4" t="inlineStr"/>
-      <c r="Y25" s="5">
-        <f>IFERROR(X25/W25*1000,"")</f>
+      <c r="Y25" s="4" t="inlineStr"/>
+      <c r="Z25" s="5">
+        <f>IFERROR(Y25/X25*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3505,26 +3583,29 @@
       <c r="R26" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="S26" s="3" t="inlineStr">
+      <c r="S26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T26" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 528 --modo hirajoshi --semilla 454078 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T26" s="2" t="inlineStr">
+      <c r="U26" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 3640 audio/OBRA-025_capa.wav --semilla 454078 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-025_528_hirajoshi.wav audio/OBRA-025_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-025_capa.wav</t>
         </is>
       </c>
-      <c r="U26" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V26" s="4" t="inlineStr"/>
+      <c r="V26" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W26" s="4" t="inlineStr"/>
       <c r="X26" s="4" t="inlineStr"/>
-      <c r="Y26" s="5">
-        <f>IFERROR(X26/W26*1000,"")</f>
+      <c r="Y26" s="4" t="inlineStr"/>
+      <c r="Z26" s="5">
+        <f>IFERROR(Y26/X26*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3619,26 +3700,29 @@
       <c r="R27" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="S27" s="3" t="inlineStr">
+      <c r="S27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T27" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 432 --modo kumoi --semilla 146597 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T27" s="2" t="inlineStr">
+      <c r="U27" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-026_432_kumoi.wav audio/OBRA-026_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="U27" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V27" s="4" t="inlineStr"/>
+      <c r="V27" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W27" s="4" t="inlineStr"/>
       <c r="X27" s="4" t="inlineStr"/>
-      <c r="Y27" s="5">
-        <f>IFERROR(X27/W27*1000,"")</f>
+      <c r="Y27" s="4" t="inlineStr"/>
+      <c r="Z27" s="5">
+        <f>IFERROR(Y27/X27*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3733,26 +3817,29 @@
       <c r="R28" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="S28" s="3" t="inlineStr">
+      <c r="S28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 396 --modo kumoi --semilla 338018 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T28" s="2" t="inlineStr">
+      <c r="U28" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py ancestral 3640 audio/OBRA-027_capa.wav --semilla 338018 --raiz 396 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-027_396_kumoi.wav audio/OBRA-027_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-027_capa.wav</t>
         </is>
       </c>
-      <c r="U28" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V28" s="4" t="inlineStr"/>
+      <c r="V28" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W28" s="4" t="inlineStr"/>
       <c r="X28" s="4" t="inlineStr"/>
-      <c r="Y28" s="5">
-        <f>IFERROR(X28/W28*1000,"")</f>
+      <c r="Y28" s="4" t="inlineStr"/>
+      <c r="Z28" s="5">
+        <f>IFERROR(Y28/X28*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3847,26 +3934,29 @@
       <c r="R29" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="S29" s="3" t="inlineStr">
+      <c r="S29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T29" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 45 --raiz 417 --modo hirajoshi --semilla 409966 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T29" s="2" t="inlineStr">
+      <c r="U29" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-028_capa.wav --semilla 409966 --raiz 417 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-028_417_hirajoshi.wav audio/OBRA-028_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-028_capa.wav</t>
         </is>
       </c>
-      <c r="U29" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V29" s="4" t="inlineStr"/>
+      <c r="V29" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W29" s="4" t="inlineStr"/>
       <c r="X29" s="4" t="inlineStr"/>
-      <c r="Y29" s="5">
-        <f>IFERROR(X29/W29*1000,"")</f>
+      <c r="Y29" s="4" t="inlineStr"/>
+      <c r="Z29" s="5">
+        <f>IFERROR(Y29/X29*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3961,26 +4051,29 @@
       <c r="R30" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="S30" s="3" t="inlineStr">
+      <c r="S30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T30" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 639 --modo yo --semilla 133046 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T30" s="2" t="inlineStr">
+      <c r="U30" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 3640 audio/OBRA-029_capa.wav --semilla 133046 --raiz 639 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-029_639_yo.wav audio/OBRA-029_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-029_capa.wav</t>
         </is>
       </c>
-      <c r="U30" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V30" s="4" t="inlineStr"/>
+      <c r="V30" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W30" s="4" t="inlineStr"/>
       <c r="X30" s="4" t="inlineStr"/>
-      <c r="Y30" s="5">
-        <f>IFERROR(X30/W30*1000,"")</f>
+      <c r="Y30" s="4" t="inlineStr"/>
+      <c r="Z30" s="5">
+        <f>IFERROR(Y30/X30*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4075,26 +4168,29 @@
       <c r="R31" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="S31" s="3" t="inlineStr">
+      <c r="S31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T31" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 45 --raiz 741 --modo yo --semilla 244487 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T31" s="2" t="inlineStr">
+      <c r="U31" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 2740 audio/OBRA-030_capa.wav --semilla 244487 --raiz 741 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-030_741_yo.wav audio/OBRA-030_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-030_capa.wav</t>
         </is>
       </c>
-      <c r="U31" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V31" s="4" t="inlineStr"/>
+      <c r="V31" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W31" s="4" t="inlineStr"/>
       <c r="X31" s="4" t="inlineStr"/>
-      <c r="Y31" s="5">
-        <f>IFERROR(X31/W31*1000,"")</f>
+      <c r="Y31" s="4" t="inlineStr"/>
+      <c r="Z31" s="5">
+        <f>IFERROR(Y31/X31*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4189,26 +4285,29 @@
       <c r="R32" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="S32" s="3" t="inlineStr">
+      <c r="S32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 45 --raiz 852 --modo hirajoshi --semilla 288169 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T32" s="2" t="inlineStr">
+      <c r="U32" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-031_capa.wav --semilla 288169 --raiz 852 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-031_852_hirajoshi.wav audio/OBRA-031_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-031_capa.wav</t>
         </is>
       </c>
-      <c r="U32" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V32" s="4" t="inlineStr"/>
+      <c r="V32" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W32" s="4" t="inlineStr"/>
       <c r="X32" s="4" t="inlineStr"/>
-      <c r="Y32" s="5">
-        <f>IFERROR(X32/W32*1000,"")</f>
+      <c r="Y32" s="4" t="inlineStr"/>
+      <c r="Z32" s="5">
+        <f>IFERROR(Y32/X32*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4303,26 +4402,29 @@
       <c r="R33" s="2" t="n">
         <v>180</v>
       </c>
-      <c r="S33" s="3" t="inlineStr">
+      <c r="S33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 528 --modo hirajoshi --semilla 638156 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T33" s="2" t="inlineStr">
+      <c r="U33" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 10840 audio/OBRA-032_capa.wav --semilla 638156 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-032_528_hirajoshi.wav audio/OBRA-032_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-032_capa.wav</t>
         </is>
       </c>
-      <c r="U33" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V33" s="4" t="inlineStr"/>
+      <c r="V33" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W33" s="4" t="inlineStr"/>
       <c r="X33" s="4" t="inlineStr"/>
-      <c r="Y33" s="5">
-        <f>IFERROR(X33/W33*1000,"")</f>
+      <c r="Y33" s="4" t="inlineStr"/>
+      <c r="Z33" s="5">
+        <f>IFERROR(Y33/X33*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4417,26 +4519,29 @@
       <c r="R34" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="S34" s="3" t="inlineStr">
+      <c r="S34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 639 --modo yo --semilla 112334 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T34" s="2" t="inlineStr">
+      <c r="U34" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 7240 audio/OBRA-033_capa.wav --semilla 112334 --raiz 639 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-033_639_yo.wav audio/OBRA-033_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-033_capa.wav</t>
         </is>
       </c>
-      <c r="U34" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V34" s="4" t="inlineStr"/>
+      <c r="V34" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W34" s="4" t="inlineStr"/>
       <c r="X34" s="4" t="inlineStr"/>
-      <c r="Y34" s="5">
-        <f>IFERROR(X34/W34*1000,"")</f>
+      <c r="Y34" s="4" t="inlineStr"/>
+      <c r="Z34" s="5">
+        <f>IFERROR(Y34/X34*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4531,26 +4636,29 @@
       <c r="R35" s="2" t="n">
         <v>180</v>
       </c>
-      <c r="S35" s="3" t="inlineStr">
+      <c r="S35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 528 --modo yo --semilla 249239 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T35" s="2" t="inlineStr">
+      <c r="U35" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 10840 audio/OBRA-034_capa.wav --semilla 249239 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-034_528_yo.wav audio/OBRA-034_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-034_capa.wav</t>
         </is>
       </c>
-      <c r="U35" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V35" s="4" t="inlineStr"/>
+      <c r="V35" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W35" s="4" t="inlineStr"/>
       <c r="X35" s="4" t="inlineStr"/>
-      <c r="Y35" s="5">
-        <f>IFERROR(X35/W35*1000,"")</f>
+      <c r="Y35" s="4" t="inlineStr"/>
+      <c r="Z35" s="5">
+        <f>IFERROR(Y35/X35*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4645,26 +4753,29 @@
       <c r="R36" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="S36" s="3" t="inlineStr">
+      <c r="S36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 741 --modo yo --semilla 74636 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T36" s="2" t="inlineStr">
+      <c r="U36" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 7240 audio/OBRA-035_capa.wav --semilla 74636 --raiz 741 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-035_741_yo.wav audio/OBRA-035_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-035_capa.wav</t>
         </is>
       </c>
-      <c r="U36" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V36" s="4" t="inlineStr"/>
+      <c r="V36" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W36" s="4" t="inlineStr"/>
       <c r="X36" s="4" t="inlineStr"/>
-      <c r="Y36" s="5">
-        <f>IFERROR(X36/W36*1000,"")</f>
+      <c r="Y36" s="4" t="inlineStr"/>
+      <c r="Z36" s="5">
+        <f>IFERROR(Y36/X36*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4759,26 +4870,29 @@
       <c r="R37" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="S37" s="3" t="inlineStr">
+      <c r="S37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T37" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 90 --raiz 852 --modo yo --semilla 903477 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T37" s="2" t="inlineStr">
+      <c r="U37" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 5440 audio/OBRA-036_capa.wav --semilla 903477 --raiz 852 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-036_852_yo.wav audio/OBRA-036_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-036_capa.wav</t>
         </is>
       </c>
-      <c r="U37" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V37" s="4" t="inlineStr"/>
+      <c r="V37" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W37" s="4" t="inlineStr"/>
       <c r="X37" s="4" t="inlineStr"/>
-      <c r="Y37" s="5">
-        <f>IFERROR(X37/W37*1000,"")</f>
+      <c r="Y37" s="4" t="inlineStr"/>
+      <c r="Z37" s="5">
+        <f>IFERROR(Y37/X37*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4873,26 +4987,29 @@
       <c r="R38" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="S38" s="3" t="inlineStr">
+      <c r="S38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T38" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 432 --modo yo --semilla 718809 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T38" s="2" t="inlineStr">
+      <c r="U38" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 7240 audio/OBRA-037_capa.wav --semilla 718809 --raiz 432 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-037_432_yo.wav audio/OBRA-037_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-037_capa.wav</t>
         </is>
       </c>
-      <c r="U38" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V38" s="4" t="inlineStr"/>
+      <c r="V38" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W38" s="4" t="inlineStr"/>
       <c r="X38" s="4" t="inlineStr"/>
-      <c r="Y38" s="5">
-        <f>IFERROR(X38/W38*1000,"")</f>
+      <c r="Y38" s="4" t="inlineStr"/>
+      <c r="Z38" s="5">
+        <f>IFERROR(Y38/X38*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4987,26 +5104,29 @@
       <c r="R39" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="S39" s="3" t="inlineStr">
+      <c r="S39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T39" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 528 --modo shin --semilla 203246 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T39" s="2" t="inlineStr">
+      <c r="U39" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-038_528_shin.wav audio/OBRA-038_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="U39" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V39" s="4" t="inlineStr"/>
+      <c r="V39" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W39" s="4" t="inlineStr"/>
       <c r="X39" s="4" t="inlineStr"/>
-      <c r="Y39" s="5">
-        <f>IFERROR(X39/W39*1000,"")</f>
+      <c r="Y39" s="4" t="inlineStr"/>
+      <c r="Z39" s="5">
+        <f>IFERROR(Y39/X39*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -5101,26 +5221,29 @@
       <c r="R40" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="S40" s="3" t="inlineStr">
+      <c r="S40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T40" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 90 --raiz 639 --modo yo --semilla 281608 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T40" s="2" t="inlineStr">
+      <c r="U40" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 5440 audio/OBRA-039_capa.wav --semilla 281608 --raiz 639 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-039_639_yo.wav audio/OBRA-039_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-039_capa.wav</t>
         </is>
       </c>
-      <c r="U40" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V40" s="4" t="inlineStr"/>
+      <c r="V40" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W40" s="4" t="inlineStr"/>
       <c r="X40" s="4" t="inlineStr"/>
-      <c r="Y40" s="5">
-        <f>IFERROR(X40/W40*1000,"")</f>
+      <c r="Y40" s="4" t="inlineStr"/>
+      <c r="Z40" s="5">
+        <f>IFERROR(Y40/X40*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -5215,26 +5338,29 @@
       <c r="R41" s="2" t="n">
         <v>180</v>
       </c>
-      <c r="S41" s="3" t="inlineStr">
+      <c r="S41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T41" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 741 --modo yo --semilla 883876 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="T41" s="2" t="inlineStr">
+      <c r="U41" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 10840 audio/OBRA-040_capa.wav --semilla 883876 --raiz 741 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-040_741_yo.wav audio/OBRA-040_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-040_capa.wav</t>
         </is>
       </c>
-      <c r="U41" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="V41" s="4" t="inlineStr"/>
+      <c r="V41" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="W41" s="4" t="inlineStr"/>
       <c r="X41" s="4" t="inlineStr"/>
-      <c r="Y41" s="5">
-        <f>IFERROR(X41/W41*1000,"")</f>
+      <c r="Y41" s="4" t="inlineStr"/>
+      <c r="Z41" s="5">
+        <f>IFERROR(Y41/X41*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -5330,30 +5456,33 @@
       <c r="R42" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="S42" s="3" t="inlineStr">
+      <c r="S42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T42" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 432 --modo hirajoshi --semilla 304617 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T42" s="2" t="inlineStr">
+      <c r="U42" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py jardin 3640 audio/OBRA-041_capa.wav --semilla 304617 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-041_432_hirajoshi.wav audio/OBRA-041_final.wav --fondo mar --nivel-fondo -8 --nivel-capa 0 --capa audio/OBRA-041_capa.wav</t>
         </is>
       </c>
-      <c r="U42" s="4" t="inlineStr">
+      <c r="V42" s="4" t="inlineStr">
         <is>
           <t>publicada</t>
         </is>
       </c>
-      <c r="V42" s="4" t="inlineStr">
+      <c r="W42" s="4" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="W42" s="4" t="inlineStr"/>
       <c r="X42" s="4" t="inlineStr"/>
-      <c r="Y42" s="5">
-        <f>IFERROR(X42/W42*1000,"")</f>
+      <c r="Y42" s="4" t="inlineStr"/>
+      <c r="Z42" s="5">
+        <f>IFERROR(Y42/X42*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -5449,35 +5578,152 @@
       <c r="R43" s="2" t="n">
         <v>180</v>
       </c>
-      <c r="S43" s="3" t="inlineStr">
+      <c r="S43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T43" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 528 --modo shin --semilla 266691 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="T43" s="2" t="inlineStr">
+      <c r="U43" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 10840 audio/OBRA-042_capa.wav --semilla 266691 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-042_528_shin.wav audio/OBRA-042_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-042_capa.wav</t>
         </is>
       </c>
-      <c r="U43" s="4" t="inlineStr">
+      <c r="V43" s="4" t="inlineStr">
         <is>
           <t>publicada</t>
         </is>
       </c>
-      <c r="V43" s="4" t="inlineStr">
+      <c r="W43" s="4" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="W43" s="4" t="inlineStr"/>
       <c r="X43" s="4" t="inlineStr"/>
-      <c r="Y43" s="5">
-        <f>IFERROR(X43/W43*1000,"")</f>
+      <c r="Y43" s="4" t="inlineStr"/>
+      <c r="Z43" s="5">
+        <f>IFERROR(Y43/X43*1000,"")</f>
         <v/>
       </c>
     </row>
+    <row r="44" ht="58" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-043</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Dark Screen Sleep Music 🌙 Gentle Rain for Deep Sleep · Fall Asleep Fast · 432 Hz · 3 Hours</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Música para dormir · Lluvia suave · 432 Hz · Pantalla oscura · 3 horas</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Dormir</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>lluvia</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Three hours of dark screen sleep music: gentle rain and a slow, warm drone for deep sleep.
+The screen fades to black after 3 minutes, so no light keeps you awake. The music slows to 3.5 breaths per minute: let your breathing follow it down.
+🌙 Lights off, phone face down, volume low. Nothing else to do tonight.
+🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+Original composition by Rin, synthesized from scratch in just intonation around 216 Hz, the low octave of 432 Hz, kumoi mode. No samples.
+#sleepmusic #darkscreen #432hz</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Pantalla oscura · 3 horas
+Para acompañar el sueño.
+Ambiente: lluvia suave.
+Compuesta con raíz en 216 Hz, la octava grave de 432 Hz, en entonación justa, modo kumoi.
+Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
+Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#sleepmusic #meditation #432hz</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>3 HOURS</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>#sleepmusic #darkscreen #432hz</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>dark screen sleep music, black screen sleep music, sleep music, deep sleep music, sleeping music for deep sleeping, fall asleep fast, rain sounds for sleeping, gentle rain, sleep music for anxiety, insomnia, cortisol reset, relaxing sleep music, music for sleep, 432 hz, 432 hz sleep music, 3 hours, rin, música para dormir</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr"/>
+      <c r="L44" s="4" t="inlineStr"/>
+      <c r="M44" s="2" t="n">
+        <v>432</v>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>kumoi</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>grave</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="n">
+        <v>615127</v>
+      </c>
+      <c r="Q44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R44" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="S44" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="T44" s="3" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/compositor.py --minutos 180 --raiz 432 --modo kumoi --semilla 615127 --caracter sin-cuenco --registro grave</t>
+        </is>
+      </c>
+      <c r="U44" s="2" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/ambiente.py audio/OBRA-043_432_kumoi.wav audio/OBRA-043_final.wav --fondo lluvia</t>
+        </is>
+      </c>
+      <c r="V44" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="W44" s="4" t="inlineStr"/>
+      <c r="X44" s="4" t="inlineStr"/>
+      <c r="Y44" s="4" t="inlineStr"/>
+      <c r="Z44" s="5">
+        <f>IFERROR(Y44/X44*1000,"")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Y43"/>
+  <autoFilter ref="A1:Z44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5488,7 +5734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S295"/>
+  <dimension ref="A1:S298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -26987,8 +27233,224 @@
       <c r="R295" s="4" t="inlineStr"/>
       <c r="S295" s="4" t="inlineStr"/>
     </row>
+    <row r="296" ht="58" customHeight="1">
+      <c r="A296" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-043-S1</t>
+        </is>
+      </c>
+      <c r="B296" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-043</t>
+        </is>
+      </c>
+      <c r="C296" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D296" s="2" t="inlineStr">
+        <is>
+          <t>short-1.mp4</t>
+        </is>
+      </c>
+      <c r="E296" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="F296" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G296" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H296" s="2" t="inlineStr">
+        <is>
+          <t>to fall asleep</t>
+        </is>
+      </c>
+      <c r="I296" s="3" t="inlineStr">
+        <is>
+          <t>To fall asleep · 432 Hz · Gentle Rain</t>
+        </is>
+      </c>
+      <c r="J296" s="3" t="inlineStr">
+        <is>
+          <t>Save this for tonight.
+Full piece (3 h): Dark Screen Sleep Music 🌙 Gentle Rain for Deep Sleep · Fall Asleep Fast · 432 Hz · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K296" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, gentle rain, Rin</t>
+        </is>
+      </c>
+      <c r="L296" s="2" t="inlineStr"/>
+      <c r="M296" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · sleep</t>
+        </is>
+      </c>
+      <c r="N296" s="3" t="inlineStr">
+        <is>
+          <t>Save this for tonight. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O296" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P296" s="4" t="inlineStr"/>
+      <c r="Q296" s="4" t="inlineStr"/>
+      <c r="R296" s="4" t="inlineStr"/>
+      <c r="S296" s="4" t="inlineStr"/>
+    </row>
+    <row r="297" ht="58" customHeight="1">
+      <c r="A297" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-043-S2</t>
+        </is>
+      </c>
+      <c r="B297" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-043</t>
+        </is>
+      </c>
+      <c r="C297" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D297" s="2" t="inlineStr">
+        <is>
+          <t>short-2.mp4</t>
+        </is>
+      </c>
+      <c r="E297" s="2" t="n">
+        <v>5432</v>
+      </c>
+      <c r="F297" s="2" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G297" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H297" s="2" t="inlineStr">
+        <is>
+          <t>let the day go quiet</t>
+        </is>
+      </c>
+      <c r="I297" s="3" t="inlineStr">
+        <is>
+          <t>Let the day go quiet · 432 Hz · Gentle Rain</t>
+        </is>
+      </c>
+      <c r="J297" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, volume low.
+Full piece (3 h): Dark Screen Sleep Music 🌙 Gentle Rain for Deep Sleep · Fall Asleep Fast · 432 Hz · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K297" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, gentle rain, Rin</t>
+        </is>
+      </c>
+      <c r="L297" s="2" t="inlineStr"/>
+      <c r="M297" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · night</t>
+        </is>
+      </c>
+      <c r="N297" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, volume low. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O297" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P297" s="4" t="inlineStr"/>
+      <c r="Q297" s="4" t="inlineStr"/>
+      <c r="R297" s="4" t="inlineStr"/>
+      <c r="S297" s="4" t="inlineStr"/>
+    </row>
+    <row r="298" ht="58" customHeight="1">
+      <c r="A298" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-043-S3</t>
+        </is>
+      </c>
+      <c r="B298" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-043</t>
+        </is>
+      </c>
+      <c r="C298" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D298" s="2" t="inlineStr">
+        <is>
+          <t>short-3.mp4</t>
+        </is>
+      </c>
+      <c r="E298" s="2" t="n">
+        <v>10775</v>
+      </c>
+      <c r="F298" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G298" s="2" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H298" s="2" t="inlineStr">
+        <is>
+          <t>lights off, breathe slower</t>
+        </is>
+      </c>
+      <c r="I298" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, breathe slower · 432 Hz · Gentle Rain</t>
+        </is>
+      </c>
+      <c r="J298" s="3" t="inlineStr">
+        <is>
+          <t>Stay until your breathing slows.
+Full piece (3 h): Dark Screen Sleep Music 🌙 Gentle Rain for Deep Sleep · Fall Asleep Fast · 432 Hz · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K298" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, gentle rain, Rin</t>
+        </is>
+      </c>
+      <c r="L298" s="2" t="inlineStr"/>
+      <c r="M298" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · rest</t>
+        </is>
+      </c>
+      <c r="N298" s="3" t="inlineStr">
+        <is>
+          <t>Stay until your breathing slows. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O298" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P298" s="4" t="inlineStr"/>
+      <c r="Q298" s="4" t="inlineStr"/>
+      <c r="R298" s="4" t="inlineStr"/>
+      <c r="S298" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S295"/>
+  <autoFilter ref="A1:S298"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27023,7 +27485,7 @@
         </is>
       </c>
       <c r="B2" s="7">
-        <f>COUNTA(Catálogo!A2:A43)</f>
+        <f>COUNTA(Catálogo!A2:A44)</f>
         <v/>
       </c>
     </row>
@@ -27034,7 +27496,7 @@
         </is>
       </c>
       <c r="B3" s="7">
-        <f>COUNTIF(Catálogo!U2:U43,"pendiente")</f>
+        <f>COUNTIF(Catálogo!V2:V44,"pendiente")</f>
         <v/>
       </c>
     </row>
@@ -27045,7 +27507,7 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>COUNTIF(Catálogo!U2:U43,"compuesta")</f>
+        <f>COUNTIF(Catálogo!V2:V44,"compuesta")</f>
         <v/>
       </c>
     </row>
@@ -27056,7 +27518,7 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF(Catálogo!U2:U43,"montada")</f>
+        <f>COUNTIF(Catálogo!V2:V44,"montada")</f>
         <v/>
       </c>
     </row>
@@ -27067,7 +27529,7 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF(Catálogo!U2:U43,"publicada")</f>
+        <f>COUNTIF(Catálogo!V2:V44,"publicada")</f>
         <v/>
       </c>
     </row>
@@ -27107,15 +27569,15 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Catálogo!D2:D43,A10)</f>
+        <f>COUNTIF(Catálogo!D2:D44,A10)</f>
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>COUNTIFS(Catálogo!D2:D43,A10,Catálogo!U2:U43,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D44,A10,Catálogo!V2:V44,"publicada")</f>
         <v/>
       </c>
       <c r="D10" s="7">
-        <f>SUMIF(Catálogo!D2:D43,A10,Catálogo!R2:R43)</f>
+        <f>SUMIF(Catálogo!D2:D44,A10,Catálogo!R2:R44)</f>
         <v/>
       </c>
     </row>
@@ -27126,15 +27588,15 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Catálogo!D2:D43,A11)</f>
+        <f>COUNTIF(Catálogo!D2:D44,A11)</f>
         <v/>
       </c>
       <c r="C11" s="7">
-        <f>COUNTIFS(Catálogo!D2:D43,A11,Catálogo!U2:U43,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D44,A11,Catálogo!V2:V44,"publicada")</f>
         <v/>
       </c>
       <c r="D11" s="7">
-        <f>SUMIF(Catálogo!D2:D43,A11,Catálogo!R2:R43)</f>
+        <f>SUMIF(Catálogo!D2:D44,A11,Catálogo!R2:R44)</f>
         <v/>
       </c>
     </row>
@@ -27145,15 +27607,15 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Catálogo!D2:D43,A12)</f>
+        <f>COUNTIF(Catálogo!D2:D44,A12)</f>
         <v/>
       </c>
       <c r="C12" s="7">
-        <f>COUNTIFS(Catálogo!D2:D43,A12,Catálogo!U2:U43,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D44,A12,Catálogo!V2:V44,"publicada")</f>
         <v/>
       </c>
       <c r="D12" s="7">
-        <f>SUMIF(Catálogo!D2:D43,A12,Catálogo!R2:R43)</f>
+        <f>SUMIF(Catálogo!D2:D44,A12,Catálogo!R2:R44)</f>
         <v/>
       </c>
     </row>
@@ -27164,15 +27626,15 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Catálogo!D2:D43,A13)</f>
+        <f>COUNTIF(Catálogo!D2:D44,A13)</f>
         <v/>
       </c>
       <c r="C13" s="7">
-        <f>COUNTIFS(Catálogo!D2:D43,A13,Catálogo!U2:U43,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D44,A13,Catálogo!V2:V44,"publicada")</f>
         <v/>
       </c>
       <c r="D13" s="7">
-        <f>SUMIF(Catálogo!D2:D43,A13,Catálogo!R2:R43)</f>
+        <f>SUMIF(Catálogo!D2:D44,A13,Catálogo!R2:R44)</f>
         <v/>
       </c>
     </row>
@@ -27183,15 +27645,15 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Catálogo!D2:D43,A14)</f>
+        <f>COUNTIF(Catálogo!D2:D44,A14)</f>
         <v/>
       </c>
       <c r="C14" s="7">
-        <f>COUNTIFS(Catálogo!D2:D43,A14,Catálogo!U2:U43,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D44,A14,Catálogo!V2:V44,"publicada")</f>
         <v/>
       </c>
       <c r="D14" s="7">
-        <f>SUMIF(Catálogo!D2:D43,A14,Catálogo!R2:R43)</f>
+        <f>SUMIF(Catálogo!D2:D44,A14,Catálogo!R2:R44)</f>
         <v/>
       </c>
     </row>
@@ -27228,7 +27690,7 @@
         </is>
       </c>
       <c r="B18" s="7">
-        <f>SUM(Catálogo!W2:W43)</f>
+        <f>SUM(Catálogo!X2:X44)</f>
         <v/>
       </c>
     </row>
@@ -27239,7 +27701,7 @@
         </is>
       </c>
       <c r="B19" s="7">
-        <f>SUM(Catálogo!X2:X43)</f>
+        <f>SUM(Catálogo!Y2:Y44)</f>
         <v/>
       </c>
     </row>
@@ -27270,7 +27732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -27382,7 +27844,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Ambiente aprobado en escucha: mar, mar-aves, zen, selva, lluvia-tambor o jardin.</t>
+          <t>Ambiente aprobado en escucha: mar, mar-aves, zen, selva, lluvia-tambor, jardin o lluvia.</t>
         </is>
       </c>
     </row>
@@ -27401,208 +27863,220 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>descripcion_optimizada</t>
+          <t>pantalla_oscura_min</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Descripción bilingüe lista para pegar. Solo falta añadir los capítulos tras el montaje.</t>
+          <t>Minutos de mandala antes de que la pantalla se funda a negro (videos para dormir). 0: el mandala dura todo el video.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>titulo_miniatura</t>
+          <t>descripcion_optimizada</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Texto de la miniatura: 2-4 palabras que COMPLETAN el título, nunca lo repiten.</t>
+          <t>Descripción bilingüe lista para pegar. Solo falta añadir los capítulos tras el montaje.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>hashtags</t>
+          <t>titulo_miniatura</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Tres, al final de la descripción.</t>
+          <t>Texto de la miniatura: 2-4 palabras que COMPLETAN el título, nunca lo repiten.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>etiquetas</t>
+          <t>hashtags</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Etiquetas del video, separadas por coma.</t>
+          <t>Tres, al final de la descripción.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>imagen_miniatura</t>
+          <t>etiquetas</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>AMARILLA. Ruta o URL de la portada una vez generada.</t>
+          <t>Etiquetas del video, separadas por coma.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>url_video</t>
+          <t>imagen_miniatura</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>AMARILLA. URL de YouTube una vez publicado.</t>
+          <t>AMARILLA. Ruta o URL de la portada una vez generada.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>raiz_hz / modo / registro / semilla</t>
+          <t>url_video</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Parámetros de composición. El registro grave baja una octava (Dormir y Concentración). La semilla regenera la obra idéntica.</t>
+          <t>AMARILLA. URL de YouTube una vez publicado.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>comando_regeneracion</t>
+          <t>raiz_hz / modo / registro / semilla</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Comando exacto. Copiar, pegar y ejecutar: devuelve el mismo audio bit a bit.</t>
+          <t>Parámetros de composición. El registro grave baja una octava (Dormir y Concentración). La semilla regenera la obra idéntica.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>estado</t>
+          <t>comando_regeneracion</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>AMARILLA. pendiente / compuesta / montada / publicada</t>
+          <t>Comando exacto. Copiar, pegar y ejecutar: devuelve el mismo audio bit a bit.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>fecha_publicacion</t>
+          <t>estado</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>AMARILLA. Formato AAAA-MM-DD.</t>
+          <t>AMARILLA. pendiente / compuesta / montada / publicada</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>vistas / suscriptores</t>
+          <t>fecha_publicacion</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>AMARILLA. Copiar de YouTube Studio a los 14 días de publicar.</t>
+          <t>AMARILLA. Formato AAAA-MM-DD.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
+          <t>vistas / suscriptores</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>AMARILLA. Copiar de YouTube Studio a los 14 días de publicar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
           <t>subs_por_1000</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Calculada. Es la métrica que decide el canal: por debajo de 1, el problema es la portada, no la música.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>Hoja Shorts</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>5 por obra. Cada uno cambia de tramo de la obra, encuadre, instante del mandala y frase.</t>
-        </is>
-      </c>
+      <c r="A26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>tiktok_portada</t>
+          <t>Hoja Shorts</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>El título de la portada en TikTok (el que se ve en el perfil). Distinto de la descripción.</t>
+          <t>5 por obra. Cada uno cambia de tramo de la obra, encuadre, instante del mandala y frase.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>tiktok_descripcion</t>
+          <t>tiktok_portada</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>El texto que acompaña al video en TikTok, con hashtags. En Metricool, nunca en el campo título.</t>
+          <t>El título de la portada en TikTok (el que se ve en el perfil). Distinto de la descripción.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
+          <t>tiktok_descripcion</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>El texto que acompaña al video en TikTok, con hashtags. En Metricool, nunca en el campo título.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
           <t>yt_video_relacionado</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>El video largo. En YouTube Studio va en «Video relacionado» del Short.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr"/>
-    </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>Ejemplo de fila rellenada</t>
         </is>
       </c>
-      <c r="B31" s="11" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>imagen_miniatura: portadas/obra-001.png | url_video: https://youtu.be/XXXXXXXXXXX | estado: publicada | fecha_publicacion: 2026-10-07 | vistas: 4820 | suscriptores: 11</t>
         </is>

</xml_diff>

<commit_message>
OBRA-044: Deep Sleep Theta Waves (mar lejano, theta que baja a delta, pantalla negra) y Shorts con frases de instrucción
La idea que dio YouTube Studio para el canal: pantalla oscura con ondas theta
para dormir. Comparada con la 43 (lluvia), dice qué sonido prefiere el público.

- capas.py theta: dos senos, uno por oído, en la tercera mayor justa de la raíz
  grave (270 Hz para 432): en la raíz misma temblaba contra el drone (108, 162,
  216, 324 Hz). Pulso 6 -> 4 -> 2 Hz en 3 h, por bloques de un minuto.
- ambiente «theta»: mar a -4 dB y la capa a -11 (a la altura de la obra)
- mandala «theta»: violeta de medianoche, espiral lenta de dos brazos
- Shorts desde la 44: solo frases de instrucción (la más vista del canal es
  «Breathe out longer than you breathe in»)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$Z$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$298</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$Z$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$301</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z44"/>
+  <dimension ref="A1:Z45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5730,8 +5730,122 @@
         <v/>
       </c>
     </row>
+    <row r="45" ht="58" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-044</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Deep Sleep Theta Waves 🌙 Turn Off Your Thoughts · Dark Screen · Fall Asleep Fast · 3 Hours</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Música para dormir · Mar lejano y ondas theta · 432 Hz · Ondas theta · 3 horas</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Dormir</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>theta</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Three hours of theta waves for deep sleep, over a distant ocean and a slow, warm drone.
+🎧 Use headphones: the left and right ears hear two tones 6 Hz apart. Over the hours the difference slows from theta (6 Hz, drifting off) to delta (2 Hz, deep sleep). The screen fades to black after 3 minutes.
+🌙 Lights off, phone face down, volume low. Let your thoughts go quiet.
+🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+Original composition by Rin, synthesized from scratch in just intonation around 216 Hz, the low octave of 432 Hz, shin mode. No samples.
+#thetawaves #sleepmusic #darkscreen</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Ondas theta · 3 horas
+Para acompañar el sueño.
+Ambiente: mar lejano y ondas theta.
+Compuesta con raíz en 216 Hz, la octava grave de 432 Hz, en entonación justa, modo shin.
+Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
+Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#sleepmusic #meditation #432hz</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>3 HOURS</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>#thetawaves #sleepmusic #darkscreen</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>theta waves, theta waves sleep, deep sleep theta waves, binaural beats, binaural beats for sleep, delta waves, dark screen sleep music, black screen sleep music, deep sleep music, fall asleep fast, turn off your thoughts, stop overthinking, sleep meditation, ocean waves, 432 hz, 3 hours, rin, música para dormir</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr"/>
+      <c r="L45" s="4" t="inlineStr"/>
+      <c r="M45" s="2" t="n">
+        <v>432</v>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>shin</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>grave</t>
+        </is>
+      </c>
+      <c r="P45" s="2" t="n">
+        <v>810318</v>
+      </c>
+      <c r="Q45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="S45" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="T45" s="3" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/compositor.py --minutos 180 --raiz 432 --modo shin --semilla 810318 --caracter sin-cuenco --registro grave</t>
+        </is>
+      </c>
+      <c r="U45" s="2" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/capas.py theta 10840 audio/OBRA-044_capa.wav --semilla 810318 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-044_432_shin.wav audio/OBRA-044_final.wav --fondo mar --nivel-fondo -4 --nivel-capa -11 --capa audio/OBRA-044_capa.wav</t>
+        </is>
+      </c>
+      <c r="V45" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="W45" s="4" t="inlineStr"/>
+      <c r="X45" s="4" t="inlineStr"/>
+      <c r="Y45" s="4" t="inlineStr"/>
+      <c r="Z45" s="5">
+        <f>IFERROR(Y45/X45*1000,"")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z44"/>
+  <autoFilter ref="A1:Z45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5742,7 +5856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S298"/>
+  <dimension ref="A1:S301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -27472,8 +27586,224 @@
       <c r="R298" s="4" t="inlineStr"/>
       <c r="S298" s="4" t="inlineStr"/>
     </row>
+    <row r="299" ht="58" customHeight="1">
+      <c r="A299" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-044-S1</t>
+        </is>
+      </c>
+      <c r="B299" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-044</t>
+        </is>
+      </c>
+      <c r="C299" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D299" s="2" t="inlineStr">
+        <is>
+          <t>short-1.mp4</t>
+        </is>
+      </c>
+      <c r="E299" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="F299" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G299" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H299" s="2" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in</t>
+        </is>
+      </c>
+      <c r="I299" s="3" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in · 432 Hz · Theta Waves</t>
+        </is>
+      </c>
+      <c r="J299" s="3" t="inlineStr">
+        <is>
+          <t>Save this for tonight.
+Full piece (3 h): Deep Sleep Theta Waves 🌙 Turn Off Your Thoughts · Dark Screen · Fall Asleep Fast · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K299" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, theta waves, Rin</t>
+        </is>
+      </c>
+      <c r="L299" s="2" t="inlineStr"/>
+      <c r="M299" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · sleep</t>
+        </is>
+      </c>
+      <c r="N299" s="3" t="inlineStr">
+        <is>
+          <t>Save this for tonight. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O299" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P299" s="4" t="inlineStr"/>
+      <c r="Q299" s="4" t="inlineStr"/>
+      <c r="R299" s="4" t="inlineStr"/>
+      <c r="S299" s="4" t="inlineStr"/>
+    </row>
+    <row r="300" ht="58" customHeight="1">
+      <c r="A300" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-044-S2</t>
+        </is>
+      </c>
+      <c r="B300" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-044</t>
+        </is>
+      </c>
+      <c r="C300" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D300" s="2" t="inlineStr">
+        <is>
+          <t>short-2.mp4</t>
+        </is>
+      </c>
+      <c r="E300" s="2" t="n">
+        <v>5432</v>
+      </c>
+      <c r="F300" s="2" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G300" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H300" s="2" t="inlineStr">
+        <is>
+          <t>Unclench your jaw. Let the pillow hold you</t>
+        </is>
+      </c>
+      <c r="I300" s="3" t="inlineStr">
+        <is>
+          <t>Unclench your jaw. Let the pillow hold you · 432 Hz · Theta Waves</t>
+        </is>
+      </c>
+      <c r="J300" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, volume low.
+Full piece (3 h): Deep Sleep Theta Waves 🌙 Turn Off Your Thoughts · Dark Screen · Fall Asleep Fast · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K300" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, theta waves, Rin</t>
+        </is>
+      </c>
+      <c r="L300" s="2" t="inlineStr"/>
+      <c r="M300" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · night</t>
+        </is>
+      </c>
+      <c r="N300" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, volume low. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O300" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P300" s="4" t="inlineStr"/>
+      <c r="Q300" s="4" t="inlineStr"/>
+      <c r="R300" s="4" t="inlineStr"/>
+      <c r="S300" s="4" t="inlineStr"/>
+    </row>
+    <row r="301" ht="58" customHeight="1">
+      <c r="A301" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-044-S3</t>
+        </is>
+      </c>
+      <c r="B301" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-044</t>
+        </is>
+      </c>
+      <c r="C301" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D301" s="2" t="inlineStr">
+        <is>
+          <t>short-3.mp4</t>
+        </is>
+      </c>
+      <c r="E301" s="2" t="n">
+        <v>10775</v>
+      </c>
+      <c r="F301" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G301" s="2" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H301" s="2" t="inlineStr">
+        <is>
+          <t>Close your eyes. Just listen</t>
+        </is>
+      </c>
+      <c r="I301" s="3" t="inlineStr">
+        <is>
+          <t>Close your eyes. Just listen · 432 Hz · Theta Waves</t>
+        </is>
+      </c>
+      <c r="J301" s="3" t="inlineStr">
+        <is>
+          <t>Stay until your breathing slows.
+Full piece (3 h): Deep Sleep Theta Waves 🌙 Turn Off Your Thoughts · Dark Screen · Fall Asleep Fast · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K301" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, theta waves, Rin</t>
+        </is>
+      </c>
+      <c r="L301" s="2" t="inlineStr"/>
+      <c r="M301" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · rest</t>
+        </is>
+      </c>
+      <c r="N301" s="3" t="inlineStr">
+        <is>
+          <t>Stay until your breathing slows. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O301" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P301" s="4" t="inlineStr"/>
+      <c r="Q301" s="4" t="inlineStr"/>
+      <c r="R301" s="4" t="inlineStr"/>
+      <c r="S301" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S298"/>
+  <autoFilter ref="A1:S301"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27508,7 +27838,7 @@
         </is>
       </c>
       <c r="B2" s="7">
-        <f>COUNTA(Catálogo!A2:A44)</f>
+        <f>COUNTA(Catálogo!A2:A45)</f>
         <v/>
       </c>
     </row>
@@ -27519,7 +27849,7 @@
         </is>
       </c>
       <c r="B3" s="7">
-        <f>COUNTIF(Catálogo!V2:V44,"pendiente")</f>
+        <f>COUNTIF(Catálogo!V2:V45,"pendiente")</f>
         <v/>
       </c>
     </row>
@@ -27530,7 +27860,7 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>COUNTIF(Catálogo!V2:V44,"compuesta")</f>
+        <f>COUNTIF(Catálogo!V2:V45,"compuesta")</f>
         <v/>
       </c>
     </row>
@@ -27541,7 +27871,7 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF(Catálogo!V2:V44,"montada")</f>
+        <f>COUNTIF(Catálogo!V2:V45,"montada")</f>
         <v/>
       </c>
     </row>
@@ -27552,7 +27882,7 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF(Catálogo!V2:V44,"publicada")</f>
+        <f>COUNTIF(Catálogo!V2:V45,"publicada")</f>
         <v/>
       </c>
     </row>
@@ -27592,15 +27922,15 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Catálogo!D2:D44,A10)</f>
+        <f>COUNTIF(Catálogo!D2:D45,A10)</f>
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>COUNTIFS(Catálogo!D2:D44,A10,Catálogo!V2:V44,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D45,A10,Catálogo!V2:V45,"publicada")</f>
         <v/>
       </c>
       <c r="D10" s="7">
-        <f>SUMIF(Catálogo!D2:D44,A10,Catálogo!R2:R44)</f>
+        <f>SUMIF(Catálogo!D2:D45,A10,Catálogo!R2:R45)</f>
         <v/>
       </c>
     </row>
@@ -27611,15 +27941,15 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Catálogo!D2:D44,A11)</f>
+        <f>COUNTIF(Catálogo!D2:D45,A11)</f>
         <v/>
       </c>
       <c r="C11" s="7">
-        <f>COUNTIFS(Catálogo!D2:D44,A11,Catálogo!V2:V44,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D45,A11,Catálogo!V2:V45,"publicada")</f>
         <v/>
       </c>
       <c r="D11" s="7">
-        <f>SUMIF(Catálogo!D2:D44,A11,Catálogo!R2:R44)</f>
+        <f>SUMIF(Catálogo!D2:D45,A11,Catálogo!R2:R45)</f>
         <v/>
       </c>
     </row>
@@ -27630,15 +27960,15 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Catálogo!D2:D44,A12)</f>
+        <f>COUNTIF(Catálogo!D2:D45,A12)</f>
         <v/>
       </c>
       <c r="C12" s="7">
-        <f>COUNTIFS(Catálogo!D2:D44,A12,Catálogo!V2:V44,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D45,A12,Catálogo!V2:V45,"publicada")</f>
         <v/>
       </c>
       <c r="D12" s="7">
-        <f>SUMIF(Catálogo!D2:D44,A12,Catálogo!R2:R44)</f>
+        <f>SUMIF(Catálogo!D2:D45,A12,Catálogo!R2:R45)</f>
         <v/>
       </c>
     </row>
@@ -27649,15 +27979,15 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Catálogo!D2:D44,A13)</f>
+        <f>COUNTIF(Catálogo!D2:D45,A13)</f>
         <v/>
       </c>
       <c r="C13" s="7">
-        <f>COUNTIFS(Catálogo!D2:D44,A13,Catálogo!V2:V44,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D45,A13,Catálogo!V2:V45,"publicada")</f>
         <v/>
       </c>
       <c r="D13" s="7">
-        <f>SUMIF(Catálogo!D2:D44,A13,Catálogo!R2:R44)</f>
+        <f>SUMIF(Catálogo!D2:D45,A13,Catálogo!R2:R45)</f>
         <v/>
       </c>
     </row>
@@ -27668,15 +27998,15 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Catálogo!D2:D44,A14)</f>
+        <f>COUNTIF(Catálogo!D2:D45,A14)</f>
         <v/>
       </c>
       <c r="C14" s="7">
-        <f>COUNTIFS(Catálogo!D2:D44,A14,Catálogo!V2:V44,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D45,A14,Catálogo!V2:V45,"publicada")</f>
         <v/>
       </c>
       <c r="D14" s="7">
-        <f>SUMIF(Catálogo!D2:D44,A14,Catálogo!R2:R44)</f>
+        <f>SUMIF(Catálogo!D2:D45,A14,Catálogo!R2:R45)</f>
         <v/>
       </c>
     </row>
@@ -27713,7 +28043,7 @@
         </is>
       </c>
       <c r="B18" s="7">
-        <f>SUM(Catálogo!X2:X44)</f>
+        <f>SUM(Catálogo!X2:X45)</f>
         <v/>
       </c>
     </row>
@@ -27724,7 +28054,7 @@
         </is>
       </c>
       <c r="B19" s="7">
-        <f>SUM(Catálogo!Y2:Y44)</f>
+        <f>SUM(Catálogo!Y2:Y45)</f>
         <v/>
       </c>
     </row>
@@ -27867,7 +28197,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Ambiente aprobado en escucha: mar, mar-aves, zen, selva, lluvia-tambor, jardin o lluvia.</t>
+          <t>Ambiente aprobado en escucha: mar, mar-aves, zen, selva, lluvia-tambor, jardin, lluvia o theta.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
OBRA-044: «usa auriculares» en la descripción, la traducción y los textos de Shorts y TikTok
Las ondas theta solo se perciben con auriculares: el aviso va en la primera
línea, la que se ve en la búsqueda, y al principio de los textos cortos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -5758,8 +5758,8 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Three hours of theta waves for deep sleep, over a distant ocean and a slow, warm drone.
-🎧 Use headphones: the left and right ears hear two tones 6 Hz apart. Over the hours the difference slows from theta (6 Hz, drifting off) to delta (2 Hz, deep sleep). The screen fades to black after 3 minutes.
+          <t>Three hours of theta waves for deep sleep, over a distant ocean and a slow, warm drone. 🎧 Use headphones for the best experience.
+With headphones, each ear hears a slightly different tone, 6 Hz apart. Over the hours the difference slows from theta (6 Hz, drifting off) to delta (2 Hz, deep sleep). The screen fades to black after 3 minutes.
 🌙 Lights off, phone face down, volume low. Let your thoughts go quiet.
 🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
 Original composition by Rin, synthesized from scratch in just intonation around 216 Hz, the low octave of 432 Hz, shin mode. No samples.
@@ -5771,6 +5771,7 @@
           <t>Ondas theta · 3 horas
 Para acompañar el sueño.
 Ambiente: mar lejano y ondas theta.
+🎧 Usa auriculares para una mejor experiencia: cada oído escucha un tono apenas distinto y la diferencia baja de theta (6 Hz) a delta (2 Hz).
 Compuesta con raíz en 216 Hz, la octava grave de 432 Hz, en entonación justa, modo shin.
 Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
@@ -27626,7 +27627,7 @@
       </c>
       <c r="J299" s="3" t="inlineStr">
         <is>
-          <t>Save this for tonight.
+          <t>🎧 Use headphones for the best experience. Save this for tonight.
 Full piece (3 h): Deep Sleep Theta Waves 🌙 Turn Off Your Thoughts · Dark Screen · Fall Asleep Fast · 3 Hours
 #sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
         </is>
@@ -27644,7 +27645,7 @@
       </c>
       <c r="N299" s="3" t="inlineStr">
         <is>
-          <t>Save this for tonight. Full 3 h piece on YouTube: Rin.
+          <t>🎧 Use headphones for the best experience. Save this for tonight. Full 3 h piece on YouTube: Rin.
 #sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
         </is>
       </c>
@@ -27698,7 +27699,7 @@
       </c>
       <c r="J300" s="3" t="inlineStr">
         <is>
-          <t>Lights off, volume low.
+          <t>🎧 Use headphones for the best experience. Lights off, volume low.
 Full piece (3 h): Deep Sleep Theta Waves 🌙 Turn Off Your Thoughts · Dark Screen · Fall Asleep Fast · 3 Hours
 #sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
         </is>
@@ -27716,7 +27717,7 @@
       </c>
       <c r="N300" s="3" t="inlineStr">
         <is>
-          <t>Lights off, volume low. Full 3 h piece on YouTube: Rin.
+          <t>🎧 Use headphones for the best experience. Lights off, volume low. Full 3 h piece on YouTube: Rin.
 #sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
         </is>
       </c>
@@ -27770,7 +27771,7 @@
       </c>
       <c r="J301" s="3" t="inlineStr">
         <is>
-          <t>Stay until your breathing slows.
+          <t>🎧 Use headphones for the best experience. Stay until your breathing slows.
 Full piece (3 h): Deep Sleep Theta Waves 🌙 Turn Off Your Thoughts · Dark Screen · Fall Asleep Fast · 3 Hours
 #sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
         </is>
@@ -27788,7 +27789,7 @@
       </c>
       <c r="N301" s="3" t="inlineStr">
         <is>
-          <t>Stay until your breathing slows. Full 3 h piece on YouTube: Rin.
+          <t>🎧 Use headphones for the best experience. Stay until your breathing slows. Full 3 h piece on YouTube: Rin.
 #sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Suscriptores por la psicología: invitación en pantalla y comentario fijado
- Videos para dormir: entre el 0:45 y el 2:30, mientras todavía miran, una
  línea chica abajo: «A new sleep piece every week · SUBSCRIBE · RIN». Al final
  del video ya duermen, así que la pantalla final no convierte.
- comentario_fijado en el catálogo: una pregunta fácil de contestar por
  intención (y propia en la 43 y la 44). Va en metadatos.json y en textos.txt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$Z$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$AA$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$301</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z45"/>
+  <dimension ref="A1:AA45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -511,13 +511,14 @@
     <col width="6" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="62" customWidth="1" min="20" max="20"/>
+    <col width="40" customWidth="1" min="20" max="20"/>
     <col width="62" customWidth="1" min="21" max="21"/>
-    <col width="13" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
-    <col width="10" customWidth="1" min="24" max="24"/>
-    <col width="13" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="62" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -618,35 +619,40 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>comentario_fijado</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>comando_regeneracion</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>comando_ambiente</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>estado</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>fecha_publicacion</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>vistas</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>suscriptores</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>subs_por_1000</t>
         </is>
@@ -746,26 +752,31 @@
       <c r="S2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>What keeps you awake at night? 🌙 Write it here and leave it with us. Then press play and let it go. A new sleep piece every week.</t>
+        </is>
+      </c>
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 432 --modo shin --semilla 505716 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U2" s="2" t="inlineStr">
+      <c r="V2" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-001_432_shin.wav audio/OBRA-001_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="V2" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W2" s="4" t="inlineStr"/>
+      <c r="W2" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X2" s="4" t="inlineStr"/>
       <c r="Y2" s="4" t="inlineStr"/>
-      <c r="Z2" s="5">
-        <f>IFERROR(Y2/X2*1000,"")</f>
+      <c r="Z2" s="4" t="inlineStr"/>
+      <c r="AA2" s="5">
+        <f>IFERROR(Z2/Y2*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -863,26 +874,31 @@
       <c r="S3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>What keeps you awake at night? 🌙 Write it here and leave it with us. Then press play and let it go. A new sleep piece every week.</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 528 --modo kumoi --semilla 443547 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U3" s="2" t="inlineStr">
+      <c r="V3" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-002_528_kumoi.wav audio/OBRA-002_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="V3" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W3" s="4" t="inlineStr"/>
+      <c r="W3" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X3" s="4" t="inlineStr"/>
       <c r="Y3" s="4" t="inlineStr"/>
-      <c r="Z3" s="5">
-        <f>IFERROR(Y3/X3*1000,"")</f>
+      <c r="Z3" s="4" t="inlineStr"/>
+      <c r="AA3" s="5">
+        <f>IFERROR(Z3/Y3*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -980,26 +996,31 @@
       <c r="S4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T4" s="3" t="inlineStr">
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>What keeps you awake at night? 🌙 Write it here and leave it with us. Then press play and let it go. A new sleep piece every week.</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 396 --modo kumoi --semilla 692584 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U4" s="2" t="inlineStr">
+      <c r="V4" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-003_396_kumoi.wav audio/OBRA-003_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="V4" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W4" s="4" t="inlineStr"/>
+      <c r="W4" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X4" s="4" t="inlineStr"/>
       <c r="Y4" s="4" t="inlineStr"/>
-      <c r="Z4" s="5">
-        <f>IFERROR(Y4/X4*1000,"")</f>
+      <c r="Z4" s="4" t="inlineStr"/>
+      <c r="AA4" s="5">
+        <f>IFERROR(Z4/Y4*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1097,26 +1118,31 @@
       <c r="S5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T5" s="3" t="inlineStr">
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>What keeps you awake at night? 🌙 Write it here and leave it with us. Then press play and let it go. A new sleep piece every week.</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 528 --modo shin --semilla 751043 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U5" s="2" t="inlineStr">
+      <c r="V5" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-004_528_shin.wav audio/OBRA-004_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="V5" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W5" s="4" t="inlineStr"/>
+      <c r="W5" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X5" s="4" t="inlineStr"/>
       <c r="Y5" s="4" t="inlineStr"/>
-      <c r="Z5" s="5">
-        <f>IFERROR(Y5/X5*1000,"")</f>
+      <c r="Z5" s="4" t="inlineStr"/>
+      <c r="AA5" s="5">
+        <f>IFERROR(Z5/Y5*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1214,26 +1240,31 @@
       <c r="S6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T6" s="3" t="inlineStr">
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>What keeps you awake at night? 🌙 Write it here and leave it with us. Then press play and let it go. A new sleep piece every week.</t>
+        </is>
+      </c>
+      <c r="U6" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 432 --modo kumoi --semilla 531725 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U6" s="2" t="inlineStr">
+      <c r="V6" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-005_432_kumoi.wav audio/OBRA-005_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="V6" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W6" s="4" t="inlineStr"/>
+      <c r="W6" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X6" s="4" t="inlineStr"/>
       <c r="Y6" s="4" t="inlineStr"/>
-      <c r="Z6" s="5">
-        <f>IFERROR(Y6/X6*1000,"")</f>
+      <c r="Z6" s="4" t="inlineStr"/>
+      <c r="AA6" s="5">
+        <f>IFERROR(Z6/Y6*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1335,30 +1366,35 @@
       <c r="S7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T7" s="3" t="inlineStr">
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>What keeps you awake at night? 🌙 Write it here and leave it with us. Then press play and let it go. A new sleep piece every week.</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 90 --raiz 417 --modo kumoi --semilla 813147 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U7" s="2" t="inlineStr">
+      <c r="V7" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-006_417_kumoi.wav audio/OBRA-006_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="V7" s="4" t="inlineStr">
+      <c r="W7" s="4" t="inlineStr">
         <is>
           <t>publicada</t>
         </is>
       </c>
-      <c r="W7" s="4" t="inlineStr">
+      <c r="X7" s="4" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="X7" s="4" t="inlineStr"/>
       <c r="Y7" s="4" t="inlineStr"/>
-      <c r="Z7" s="5">
-        <f>IFERROR(Y7/X7*1000,"")</f>
+      <c r="Z7" s="4" t="inlineStr"/>
+      <c r="AA7" s="5">
+        <f>IFERROR(Z7/Y7*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1456,26 +1492,31 @@
       <c r="S8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T8" s="3" t="inlineStr">
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>What keeps you awake at night? 🌙 Write it here and leave it with us. Then press play and let it go. A new sleep piece every week.</t>
+        </is>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 396 --modo shin --semilla 885916 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U8" s="2" t="inlineStr">
+      <c r="V8" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-007_396_shin.wav audio/OBRA-007_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="V8" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W8" s="4" t="inlineStr"/>
+      <c r="W8" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X8" s="4" t="inlineStr"/>
       <c r="Y8" s="4" t="inlineStr"/>
-      <c r="Z8" s="5">
-        <f>IFERROR(Y8/X8*1000,"")</f>
+      <c r="Z8" s="4" t="inlineStr"/>
+      <c r="AA8" s="5">
+        <f>IFERROR(Z8/Y8*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1573,26 +1614,31 @@
       <c r="S9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T9" s="3" t="inlineStr">
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>What keeps you awake at night? 🌙 Write it here and leave it with us. Then press play and let it go. A new sleep piece every week.</t>
+        </is>
+      </c>
+      <c r="U9" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 432 --modo kumoi --semilla 295910 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U9" s="2" t="inlineStr">
+      <c r="V9" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-008_432_kumoi.wav audio/OBRA-008_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="V9" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W9" s="4" t="inlineStr"/>
+      <c r="W9" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X9" s="4" t="inlineStr"/>
       <c r="Y9" s="4" t="inlineStr"/>
-      <c r="Z9" s="5">
-        <f>IFERROR(Y9/X9*1000,"")</f>
+      <c r="Z9" s="4" t="inlineStr"/>
+      <c r="AA9" s="5">
+        <f>IFERROR(Z9/Y9*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1690,26 +1736,31 @@
       <c r="S10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T10" s="3" t="inlineStr">
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>What's on your mind right now? 🌿 Write it here and leave it with us. Sometimes saying it is enough to set it down.</t>
+        </is>
+      </c>
+      <c r="U10" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 25 --raiz 396 --modo kumoi --semilla 555819 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U10" s="2" t="inlineStr">
+      <c r="V10" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 1540 audio/OBRA-009_capa.wav --semilla 555819 --raiz 396 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-009_396_kumoi.wav audio/OBRA-009_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-009_capa.wav</t>
         </is>
       </c>
-      <c r="V10" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W10" s="4" t="inlineStr"/>
+      <c r="W10" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X10" s="4" t="inlineStr"/>
       <c r="Y10" s="4" t="inlineStr"/>
-      <c r="Z10" s="5">
-        <f>IFERROR(Y10/X10*1000,"")</f>
+      <c r="Z10" s="4" t="inlineStr"/>
+      <c r="AA10" s="5">
+        <f>IFERROR(Z10/Y10*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1807,26 +1858,31 @@
       <c r="S11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T11" s="3" t="inlineStr">
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>What's on your mind right now? 🌿 Write it here and leave it with us. Sometimes saying it is enough to set it down.</t>
+        </is>
+      </c>
+      <c r="U11" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 30 --raiz 432 --modo hirajoshi --semilla 739461 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U11" s="2" t="inlineStr">
+      <c r="V11" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 1840 audio/OBRA-010_capa.wav --semilla 739461 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-010_432_hirajoshi.wav audio/OBRA-010_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-010_capa.wav</t>
         </is>
       </c>
-      <c r="V11" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W11" s="4" t="inlineStr"/>
+      <c r="W11" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X11" s="4" t="inlineStr"/>
       <c r="Y11" s="4" t="inlineStr"/>
-      <c r="Z11" s="5">
-        <f>IFERROR(Y11/X11*1000,"")</f>
+      <c r="Z11" s="4" t="inlineStr"/>
+      <c r="AA11" s="5">
+        <f>IFERROR(Z11/Y11*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -1924,26 +1980,31 @@
       <c r="S12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T12" s="3" t="inlineStr">
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>What's on your mind right now? 🌿 Write it here and leave it with us. Sometimes saying it is enough to set it down.</t>
+        </is>
+      </c>
+      <c r="U12" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 20 --raiz 528 --modo hirajoshi --semilla 913368 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U12" s="2" t="inlineStr">
+      <c r="V12" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 1240 audio/OBRA-011_capa.wav --semilla 913368 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-011_528_hirajoshi.wav audio/OBRA-011_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-011_capa.wav</t>
         </is>
       </c>
-      <c r="V12" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W12" s="4" t="inlineStr"/>
+      <c r="W12" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X12" s="4" t="inlineStr"/>
       <c r="Y12" s="4" t="inlineStr"/>
-      <c r="Z12" s="5">
-        <f>IFERROR(Y12/X12*1000,"")</f>
+      <c r="Z12" s="4" t="inlineStr"/>
+      <c r="AA12" s="5">
+        <f>IFERROR(Z12/Y12*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2045,30 +2106,35 @@
       <c r="S13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T13" s="3" t="inlineStr">
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>What's on your mind right now? 🌿 Write it here and leave it with us. Sometimes saying it is enough to set it down.</t>
+        </is>
+      </c>
+      <c r="U13" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 10 --raiz 528 --modo shin --semilla 43734 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U13" s="2" t="inlineStr">
+      <c r="V13" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 640 audio/OBRA-012_capa.wav --semilla 43734 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-012_528_shin.wav audio/OBRA-012_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-012_capa.wav</t>
         </is>
       </c>
-      <c r="V13" s="4" t="inlineStr">
+      <c r="W13" s="4" t="inlineStr">
         <is>
           <t>publicada</t>
         </is>
       </c>
-      <c r="W13" s="4" t="inlineStr">
+      <c r="X13" s="4" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="X13" s="4" t="inlineStr"/>
       <c r="Y13" s="4" t="inlineStr"/>
-      <c r="Z13" s="5">
-        <f>IFERROR(Y13/X13*1000,"")</f>
+      <c r="Z13" s="4" t="inlineStr"/>
+      <c r="AA13" s="5">
+        <f>IFERROR(Z13/Y13*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2166,26 +2232,31 @@
       <c r="S14" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T14" s="3" t="inlineStr">
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>What's on your mind right now? 🌿 Write it here and leave it with us. Sometimes saying it is enough to set it down.</t>
+        </is>
+      </c>
+      <c r="U14" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 20 --raiz 432 --modo hirajoshi --semilla 627771 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U14" s="2" t="inlineStr">
+      <c r="V14" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 1240 audio/OBRA-013_capa.wav --semilla 627771 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-013_432_hirajoshi.wav audio/OBRA-013_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-013_capa.wav</t>
         </is>
       </c>
-      <c r="V14" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W14" s="4" t="inlineStr"/>
+      <c r="W14" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X14" s="4" t="inlineStr"/>
       <c r="Y14" s="4" t="inlineStr"/>
-      <c r="Z14" s="5">
-        <f>IFERROR(Y14/X14*1000,"")</f>
+      <c r="Z14" s="4" t="inlineStr"/>
+      <c r="AA14" s="5">
+        <f>IFERROR(Z14/Y14*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2283,26 +2354,31 @@
       <c r="S15" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T15" s="3" t="inlineStr">
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>What's on your mind right now? 🌿 Write it here and leave it with us. Sometimes saying it is enough to set it down.</t>
+        </is>
+      </c>
+      <c r="U15" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 20 --raiz 528 --modo yo --semilla 310137 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U15" s="2" t="inlineStr">
+      <c r="V15" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-014_capa.wav --semilla 310137 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-014_528_yo.wav audio/OBRA-014_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-014_capa.wav</t>
         </is>
       </c>
-      <c r="V15" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W15" s="4" t="inlineStr"/>
+      <c r="W15" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X15" s="4" t="inlineStr"/>
       <c r="Y15" s="4" t="inlineStr"/>
-      <c r="Z15" s="5">
-        <f>IFERROR(Y15/X15*1000,"")</f>
+      <c r="Z15" s="4" t="inlineStr"/>
+      <c r="AA15" s="5">
+        <f>IFERROR(Z15/Y15*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2404,30 +2480,35 @@
       <c r="S16" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T16" s="3" t="inlineStr">
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>What's on your mind right now? 🌿 Write it here and leave it with us. Sometimes saying it is enough to set it down.</t>
+        </is>
+      </c>
+      <c r="U16" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 15 --raiz 639 --modo yo --semilla 592463 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U16" s="2" t="inlineStr">
+      <c r="V16" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 940 audio/OBRA-015_capa.wav --semilla 592463 --raiz 639 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-015_639_yo.wav audio/OBRA-015_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-015_capa.wav</t>
         </is>
       </c>
-      <c r="V16" s="4" t="inlineStr">
+      <c r="W16" s="4" t="inlineStr">
         <is>
           <t>publicada</t>
         </is>
       </c>
-      <c r="W16" s="4" t="inlineStr">
+      <c r="X16" s="4" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="X16" s="4" t="inlineStr"/>
       <c r="Y16" s="4" t="inlineStr"/>
-      <c r="Z16" s="5">
-        <f>IFERROR(Y16/X16*1000,"")</f>
+      <c r="Z16" s="4" t="inlineStr"/>
+      <c r="AA16" s="5">
+        <f>IFERROR(Z16/Y16*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2525,26 +2606,31 @@
       <c r="S17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T17" s="3" t="inlineStr">
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>What's on your mind right now? 🌿 Write it here and leave it with us. Sometimes saying it is enough to set it down.</t>
+        </is>
+      </c>
+      <c r="U17" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 30 --raiz 417 --modo kumoi --semilla 250697 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U17" s="2" t="inlineStr">
+      <c r="V17" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py ancestral 1840 audio/OBRA-016_capa.wav --semilla 250697 --raiz 417 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-016_417_kumoi.wav audio/OBRA-016_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-016_capa.wav</t>
         </is>
       </c>
-      <c r="V17" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W17" s="4" t="inlineStr"/>
+      <c r="W17" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X17" s="4" t="inlineStr"/>
       <c r="Y17" s="4" t="inlineStr"/>
-      <c r="Z17" s="5">
-        <f>IFERROR(Y17/X17*1000,"")</f>
+      <c r="Z17" s="4" t="inlineStr"/>
+      <c r="AA17" s="5">
+        <f>IFERROR(Z17/Y17*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2642,26 +2728,31 @@
       <c r="S18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T18" s="3" t="inlineStr">
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>Where are you listening from today? 🌿 A new piece every week.</t>
+        </is>
+      </c>
+      <c r="U18" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 45 --raiz 417 --modo hirajoshi --semilla 714152 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U18" s="2" t="inlineStr">
+      <c r="V18" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-017_capa.wav --semilla 714152 --raiz 417 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-017_417_hirajoshi.wav audio/OBRA-017_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-017_capa.wav</t>
         </is>
       </c>
-      <c r="V18" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W18" s="4" t="inlineStr"/>
+      <c r="W18" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X18" s="4" t="inlineStr"/>
       <c r="Y18" s="4" t="inlineStr"/>
-      <c r="Z18" s="5">
-        <f>IFERROR(Y18/X18*1000,"")</f>
+      <c r="Z18" s="4" t="inlineStr"/>
+      <c r="AA18" s="5">
+        <f>IFERROR(Z18/Y18*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2759,26 +2850,31 @@
       <c r="S19" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T19" s="3" t="inlineStr">
+      <c r="T19" s="2" t="inlineStr">
+        <is>
+          <t>Where are you listening from today? 🌿 A new piece every week.</t>
+        </is>
+      </c>
+      <c r="U19" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 45 --raiz 528 --modo hirajoshi --semilla 735455 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U19" s="2" t="inlineStr">
+      <c r="V19" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-018_capa.wav --semilla 735455 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-018_528_hirajoshi.wav audio/OBRA-018_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-018_capa.wav</t>
         </is>
       </c>
-      <c r="V19" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W19" s="4" t="inlineStr"/>
+      <c r="W19" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X19" s="4" t="inlineStr"/>
       <c r="Y19" s="4" t="inlineStr"/>
-      <c r="Z19" s="5">
-        <f>IFERROR(Y19/X19*1000,"")</f>
+      <c r="Z19" s="4" t="inlineStr"/>
+      <c r="AA19" s="5">
+        <f>IFERROR(Z19/Y19*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2876,26 +2972,31 @@
       <c r="S20" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T20" s="3" t="inlineStr">
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>Where are you listening from today? 🌿 A new piece every week.</t>
+        </is>
+      </c>
+      <c r="U20" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 432 --modo shin --semilla 627577 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U20" s="2" t="inlineStr">
+      <c r="V20" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-019_capa.wav --semilla 627577 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-019_432_shin.wav audio/OBRA-019_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-019_capa.wav</t>
         </is>
       </c>
-      <c r="V20" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W20" s="4" t="inlineStr"/>
+      <c r="W20" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X20" s="4" t="inlineStr"/>
       <c r="Y20" s="4" t="inlineStr"/>
-      <c r="Z20" s="5">
-        <f>IFERROR(Y20/X20*1000,"")</f>
+      <c r="Z20" s="4" t="inlineStr"/>
+      <c r="AA20" s="5">
+        <f>IFERROR(Z20/Y20*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -2997,30 +3098,35 @@
       <c r="S21" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T21" s="3" t="inlineStr">
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>Where are you listening from today? 🌿 A new piece every week.</t>
+        </is>
+      </c>
+      <c r="U21" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 30 --raiz 528 --modo shin --semilla 632595 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U21" s="2" t="inlineStr">
+      <c r="V21" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py ancestral 1840 audio/OBRA-020_capa.wav --semilla 632595 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-020_528_shin.wav audio/OBRA-020_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-020_capa.wav</t>
         </is>
       </c>
-      <c r="V21" s="4" t="inlineStr">
+      <c r="W21" s="4" t="inlineStr">
         <is>
           <t>publicada</t>
         </is>
       </c>
-      <c r="W21" s="4" t="inlineStr">
+      <c r="X21" s="4" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="X21" s="4" t="inlineStr"/>
       <c r="Y21" s="4" t="inlineStr"/>
-      <c r="Z21" s="5">
-        <f>IFERROR(Y21/X21*1000,"")</f>
+      <c r="Z21" s="4" t="inlineStr"/>
+      <c r="AA21" s="5">
+        <f>IFERROR(Z21/Y21*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3118,26 +3224,31 @@
       <c r="S22" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T22" s="3" t="inlineStr">
+      <c r="T22" s="2" t="inlineStr">
+        <is>
+          <t>Where are you listening from today? 🌿 A new piece every week.</t>
+        </is>
+      </c>
+      <c r="U22" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 45 --raiz 396 --modo kumoi --semilla 864630 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U22" s="2" t="inlineStr">
+      <c r="V22" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-021_capa.wav --semilla 864630 --raiz 396 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-021_396_kumoi.wav audio/OBRA-021_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-021_capa.wav</t>
         </is>
       </c>
-      <c r="V22" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W22" s="4" t="inlineStr"/>
+      <c r="W22" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X22" s="4" t="inlineStr"/>
       <c r="Y22" s="4" t="inlineStr"/>
-      <c r="Z22" s="5">
-        <f>IFERROR(Y22/X22*1000,"")</f>
+      <c r="Z22" s="4" t="inlineStr"/>
+      <c r="AA22" s="5">
+        <f>IFERROR(Z22/Y22*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3235,26 +3346,31 @@
       <c r="S23" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T23" s="3" t="inlineStr">
+      <c r="T23" s="2" t="inlineStr">
+        <is>
+          <t>Where are you listening from today? 🌿 A new piece every week.</t>
+        </is>
+      </c>
+      <c r="U23" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 639 --modo yo --semilla 335798 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U23" s="2" t="inlineStr">
+      <c r="V23" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-022_capa.wav --semilla 335798 --raiz 639 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-022_639_yo.wav audio/OBRA-022_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-022_capa.wav</t>
         </is>
       </c>
-      <c r="V23" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W23" s="4" t="inlineStr"/>
+      <c r="W23" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X23" s="4" t="inlineStr"/>
       <c r="Y23" s="4" t="inlineStr"/>
-      <c r="Z23" s="5">
-        <f>IFERROR(Y23/X23*1000,"")</f>
+      <c r="Z23" s="4" t="inlineStr"/>
+      <c r="AA23" s="5">
+        <f>IFERROR(Z23/Y23*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3352,26 +3468,31 @@
       <c r="S24" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T24" s="3" t="inlineStr">
+      <c r="T24" s="2" t="inlineStr">
+        <is>
+          <t>Where are you listening from today? 🌿 A new piece every week.</t>
+        </is>
+      </c>
+      <c r="U24" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 20 --raiz 528 --modo shin --semilla 299306 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U24" s="2" t="inlineStr">
+      <c r="V24" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-023_capa.wav --semilla 299306 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-023_528_shin.wav audio/OBRA-023_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-023_capa.wav</t>
         </is>
       </c>
-      <c r="V24" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W24" s="4" t="inlineStr"/>
+      <c r="W24" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X24" s="4" t="inlineStr"/>
       <c r="Y24" s="4" t="inlineStr"/>
-      <c r="Z24" s="5">
-        <f>IFERROR(Y24/X24*1000,"")</f>
+      <c r="Z24" s="4" t="inlineStr"/>
+      <c r="AA24" s="5">
+        <f>IFERROR(Z24/Y24*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3469,26 +3590,31 @@
       <c r="S25" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T25" s="3" t="inlineStr">
+      <c r="T25" s="2" t="inlineStr">
+        <is>
+          <t>Where are you listening from today? 🌿 A new piece every week.</t>
+        </is>
+      </c>
+      <c r="U25" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 432 --modo kumoi --semilla 926202 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U25" s="2" t="inlineStr">
+      <c r="V25" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py ancestral 3640 audio/OBRA-024_capa.wav --semilla 926202 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-024_432_kumoi.wav audio/OBRA-024_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-024_capa.wav</t>
         </is>
       </c>
-      <c r="V25" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W25" s="4" t="inlineStr"/>
+      <c r="W25" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X25" s="4" t="inlineStr"/>
       <c r="Y25" s="4" t="inlineStr"/>
-      <c r="Z25" s="5">
-        <f>IFERROR(Y25/X25*1000,"")</f>
+      <c r="Z25" s="4" t="inlineStr"/>
+      <c r="AA25" s="5">
+        <f>IFERROR(Z25/Y25*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3586,26 +3712,31 @@
       <c r="S26" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T26" s="3" t="inlineStr">
+      <c r="T26" s="2" t="inlineStr">
+        <is>
+          <t>What are you letting go of today? 🌿 Write one word.</t>
+        </is>
+      </c>
+      <c r="U26" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 528 --modo hirajoshi --semilla 454078 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U26" s="2" t="inlineStr">
+      <c r="V26" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 3640 audio/OBRA-025_capa.wav --semilla 454078 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-025_528_hirajoshi.wav audio/OBRA-025_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-025_capa.wav</t>
         </is>
       </c>
-      <c r="V26" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W26" s="4" t="inlineStr"/>
+      <c r="W26" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X26" s="4" t="inlineStr"/>
       <c r="Y26" s="4" t="inlineStr"/>
-      <c r="Z26" s="5">
-        <f>IFERROR(Y26/X26*1000,"")</f>
+      <c r="Z26" s="4" t="inlineStr"/>
+      <c r="AA26" s="5">
+        <f>IFERROR(Z26/Y26*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3703,26 +3834,31 @@
       <c r="S27" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T27" s="3" t="inlineStr">
+      <c r="T27" s="2" t="inlineStr">
+        <is>
+          <t>What are you letting go of today? 🌿 Write one word.</t>
+        </is>
+      </c>
+      <c r="U27" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 432 --modo kumoi --semilla 146597 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U27" s="2" t="inlineStr">
+      <c r="V27" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-026_432_kumoi.wav audio/OBRA-026_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="V27" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W27" s="4" t="inlineStr"/>
+      <c r="W27" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X27" s="4" t="inlineStr"/>
       <c r="Y27" s="4" t="inlineStr"/>
-      <c r="Z27" s="5">
-        <f>IFERROR(Y27/X27*1000,"")</f>
+      <c r="Z27" s="4" t="inlineStr"/>
+      <c r="AA27" s="5">
+        <f>IFERROR(Z27/Y27*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3820,26 +3956,31 @@
       <c r="S28" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T28" s="3" t="inlineStr">
+      <c r="T28" s="2" t="inlineStr">
+        <is>
+          <t>What are you letting go of today? 🌿 Write one word.</t>
+        </is>
+      </c>
+      <c r="U28" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 396 --modo kumoi --semilla 338018 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U28" s="2" t="inlineStr">
+      <c r="V28" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py ancestral 3640 audio/OBRA-027_capa.wav --semilla 338018 --raiz 396 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-027_396_kumoi.wav audio/OBRA-027_final.wav --fondo fuego --nivel-capa 0 --nivel-obra -20 --capa audio/OBRA-027_capa.wav</t>
         </is>
       </c>
-      <c r="V28" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W28" s="4" t="inlineStr"/>
+      <c r="W28" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X28" s="4" t="inlineStr"/>
       <c r="Y28" s="4" t="inlineStr"/>
-      <c r="Z28" s="5">
-        <f>IFERROR(Y28/X28*1000,"")</f>
+      <c r="Z28" s="4" t="inlineStr"/>
+      <c r="AA28" s="5">
+        <f>IFERROR(Z28/Y28*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -3937,26 +4078,31 @@
       <c r="S29" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T29" s="3" t="inlineStr">
+      <c r="T29" s="2" t="inlineStr">
+        <is>
+          <t>What are you letting go of today? 🌿 Write one word.</t>
+        </is>
+      </c>
+      <c r="U29" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 45 --raiz 417 --modo hirajoshi --semilla 409966 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U29" s="2" t="inlineStr">
+      <c r="V29" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-028_capa.wav --semilla 409966 --raiz 417 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-028_417_hirajoshi.wav audio/OBRA-028_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-028_capa.wav</t>
         </is>
       </c>
-      <c r="V29" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W29" s="4" t="inlineStr"/>
+      <c r="W29" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X29" s="4" t="inlineStr"/>
       <c r="Y29" s="4" t="inlineStr"/>
-      <c r="Z29" s="5">
-        <f>IFERROR(Y29/X29*1000,"")</f>
+      <c r="Z29" s="4" t="inlineStr"/>
+      <c r="AA29" s="5">
+        <f>IFERROR(Z29/Y29*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4054,26 +4200,31 @@
       <c r="S30" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T30" s="3" t="inlineStr">
+      <c r="T30" s="2" t="inlineStr">
+        <is>
+          <t>What are you letting go of today? 🌿 Write one word.</t>
+        </is>
+      </c>
+      <c r="U30" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 639 --modo yo --semilla 133046 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U30" s="2" t="inlineStr">
+      <c r="V30" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 3640 audio/OBRA-029_capa.wav --semilla 133046 --raiz 639 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-029_639_yo.wav audio/OBRA-029_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-029_capa.wav</t>
         </is>
       </c>
-      <c r="V30" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W30" s="4" t="inlineStr"/>
+      <c r="W30" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X30" s="4" t="inlineStr"/>
       <c r="Y30" s="4" t="inlineStr"/>
-      <c r="Z30" s="5">
-        <f>IFERROR(Y30/X30*1000,"")</f>
+      <c r="Z30" s="4" t="inlineStr"/>
+      <c r="AA30" s="5">
+        <f>IFERROR(Z30/Y30*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4171,26 +4322,31 @@
       <c r="S31" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T31" s="3" t="inlineStr">
+      <c r="T31" s="2" t="inlineStr">
+        <is>
+          <t>What are you letting go of today? 🌿 Write one word.</t>
+        </is>
+      </c>
+      <c r="U31" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 45 --raiz 741 --modo yo --semilla 244487 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U31" s="2" t="inlineStr">
+      <c r="V31" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 2740 audio/OBRA-030_capa.wav --semilla 244487 --raiz 741 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-030_741_yo.wav audio/OBRA-030_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-030_capa.wav</t>
         </is>
       </c>
-      <c r="V31" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W31" s="4" t="inlineStr"/>
+      <c r="W31" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X31" s="4" t="inlineStr"/>
       <c r="Y31" s="4" t="inlineStr"/>
-      <c r="Z31" s="5">
-        <f>IFERROR(Y31/X31*1000,"")</f>
+      <c r="Z31" s="4" t="inlineStr"/>
+      <c r="AA31" s="5">
+        <f>IFERROR(Z31/Y31*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4288,26 +4444,31 @@
       <c r="S32" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T32" s="3" t="inlineStr">
+      <c r="T32" s="2" t="inlineStr">
+        <is>
+          <t>What are you letting go of today? 🌿 Write one word.</t>
+        </is>
+      </c>
+      <c r="U32" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 45 --raiz 852 --modo hirajoshi --semilla 288169 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U32" s="2" t="inlineStr">
+      <c r="V32" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-031_capa.wav --semilla 288169 --raiz 852 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-031_852_hirajoshi.wav audio/OBRA-031_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-031_capa.wav</t>
         </is>
       </c>
-      <c r="V32" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W32" s="4" t="inlineStr"/>
+      <c r="W32" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X32" s="4" t="inlineStr"/>
       <c r="Y32" s="4" t="inlineStr"/>
-      <c r="Z32" s="5">
-        <f>IFERROR(Y32/X32*1000,"")</f>
+      <c r="Z32" s="4" t="inlineStr"/>
+      <c r="AA32" s="5">
+        <f>IFERROR(Z32/Y32*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4405,26 +4566,31 @@
       <c r="S33" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T33" s="3" t="inlineStr">
+      <c r="T33" s="2" t="inlineStr">
+        <is>
+          <t>What are you letting go of today? 🌿 Write one word.</t>
+        </is>
+      </c>
+      <c r="U33" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 528 --modo hirajoshi --semilla 638156 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U33" s="2" t="inlineStr">
+      <c r="V33" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 10840 audio/OBRA-032_capa.wav --semilla 638156 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-032_528_hirajoshi.wav audio/OBRA-032_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-032_capa.wav</t>
         </is>
       </c>
-      <c r="V33" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W33" s="4" t="inlineStr"/>
+      <c r="W33" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X33" s="4" t="inlineStr"/>
       <c r="Y33" s="4" t="inlineStr"/>
-      <c r="Z33" s="5">
-        <f>IFERROR(Y33/X33*1000,"")</f>
+      <c r="Z33" s="4" t="inlineStr"/>
+      <c r="AA33" s="5">
+        <f>IFERROR(Z33/Y33*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4522,26 +4688,31 @@
       <c r="S34" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T34" s="3" t="inlineStr">
+      <c r="T34" s="2" t="inlineStr">
+        <is>
+          <t>What are you working on? ✍️ Tell us, and we'll keep you company.</t>
+        </is>
+      </c>
+      <c r="U34" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 639 --modo yo --semilla 112334 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U34" s="2" t="inlineStr">
+      <c r="V34" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 7240 audio/OBRA-033_capa.wav --semilla 112334 --raiz 639 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-033_639_yo.wav audio/OBRA-033_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-033_capa.wav</t>
         </is>
       </c>
-      <c r="V34" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W34" s="4" t="inlineStr"/>
+      <c r="W34" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X34" s="4" t="inlineStr"/>
       <c r="Y34" s="4" t="inlineStr"/>
-      <c r="Z34" s="5">
-        <f>IFERROR(Y34/X34*1000,"")</f>
+      <c r="Z34" s="4" t="inlineStr"/>
+      <c r="AA34" s="5">
+        <f>IFERROR(Z34/Y34*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4639,26 +4810,31 @@
       <c r="S35" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T35" s="3" t="inlineStr">
+      <c r="T35" s="2" t="inlineStr">
+        <is>
+          <t>What are you working on? ✍️ Tell us, and we'll keep you company.</t>
+        </is>
+      </c>
+      <c r="U35" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 528 --modo yo --semilla 249239 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U35" s="2" t="inlineStr">
+      <c r="V35" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 10840 audio/OBRA-034_capa.wav --semilla 249239 --raiz 528 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-034_528_yo.wav audio/OBRA-034_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-034_capa.wav</t>
         </is>
       </c>
-      <c r="V35" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W35" s="4" t="inlineStr"/>
+      <c r="W35" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X35" s="4" t="inlineStr"/>
       <c r="Y35" s="4" t="inlineStr"/>
-      <c r="Z35" s="5">
-        <f>IFERROR(Y35/X35*1000,"")</f>
+      <c r="Z35" s="4" t="inlineStr"/>
+      <c r="AA35" s="5">
+        <f>IFERROR(Z35/Y35*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4756,26 +4932,31 @@
       <c r="S36" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T36" s="3" t="inlineStr">
+      <c r="T36" s="2" t="inlineStr">
+        <is>
+          <t>What are you working on? ✍️ Tell us, and we'll keep you company.</t>
+        </is>
+      </c>
+      <c r="U36" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 741 --modo yo --semilla 74636 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U36" s="2" t="inlineStr">
+      <c r="V36" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 7240 audio/OBRA-035_capa.wav --semilla 74636 --raiz 741 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-035_741_yo.wav audio/OBRA-035_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-035_capa.wav</t>
         </is>
       </c>
-      <c r="V36" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W36" s="4" t="inlineStr"/>
+      <c r="W36" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X36" s="4" t="inlineStr"/>
       <c r="Y36" s="4" t="inlineStr"/>
-      <c r="Z36" s="5">
-        <f>IFERROR(Y36/X36*1000,"")</f>
+      <c r="Z36" s="4" t="inlineStr"/>
+      <c r="AA36" s="5">
+        <f>IFERROR(Z36/Y36*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4873,26 +5054,31 @@
       <c r="S37" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T37" s="3" t="inlineStr">
+      <c r="T37" s="2" t="inlineStr">
+        <is>
+          <t>What are you working on? ✍️ Tell us, and we'll keep you company.</t>
+        </is>
+      </c>
+      <c r="U37" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 90 --raiz 852 --modo yo --semilla 903477 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U37" s="2" t="inlineStr">
+      <c r="V37" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 5440 audio/OBRA-036_capa.wav --semilla 903477 --raiz 852 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-036_852_yo.wav audio/OBRA-036_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-036_capa.wav</t>
         </is>
       </c>
-      <c r="V37" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W37" s="4" t="inlineStr"/>
+      <c r="W37" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X37" s="4" t="inlineStr"/>
       <c r="Y37" s="4" t="inlineStr"/>
-      <c r="Z37" s="5">
-        <f>IFERROR(Y37/X37*1000,"")</f>
+      <c r="Z37" s="4" t="inlineStr"/>
+      <c r="AA37" s="5">
+        <f>IFERROR(Z37/Y37*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -4990,26 +5176,31 @@
       <c r="S38" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T38" s="3" t="inlineStr">
+      <c r="T38" s="2" t="inlineStr">
+        <is>
+          <t>What are you working on? ✍️ Tell us, and we'll keep you company.</t>
+        </is>
+      </c>
+      <c r="U38" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 432 --modo yo --semilla 718809 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U38" s="2" t="inlineStr">
+      <c r="V38" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 7240 audio/OBRA-037_capa.wav --semilla 718809 --raiz 432 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-037_432_yo.wav audio/OBRA-037_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-037_capa.wav</t>
         </is>
       </c>
-      <c r="V38" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W38" s="4" t="inlineStr"/>
+      <c r="W38" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X38" s="4" t="inlineStr"/>
       <c r="Y38" s="4" t="inlineStr"/>
-      <c r="Z38" s="5">
-        <f>IFERROR(Y38/X38*1000,"")</f>
+      <c r="Z38" s="4" t="inlineStr"/>
+      <c r="AA38" s="5">
+        <f>IFERROR(Z38/Y38*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -5107,26 +5298,31 @@
       <c r="S39" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T39" s="3" t="inlineStr">
+      <c r="T39" s="2" t="inlineStr">
+        <is>
+          <t>What are you working on? ✍️ Tell us, and we'll keep you company.</t>
+        </is>
+      </c>
+      <c r="U39" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 120 --raiz 528 --modo shin --semilla 203246 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U39" s="2" t="inlineStr">
+      <c r="V39" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-038_528_shin.wav audio/OBRA-038_final.wav --fondo mar</t>
         </is>
       </c>
-      <c r="V39" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W39" s="4" t="inlineStr"/>
+      <c r="W39" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X39" s="4" t="inlineStr"/>
       <c r="Y39" s="4" t="inlineStr"/>
-      <c r="Z39" s="5">
-        <f>IFERROR(Y39/X39*1000,"")</f>
+      <c r="Z39" s="4" t="inlineStr"/>
+      <c r="AA39" s="5">
+        <f>IFERROR(Z39/Y39*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -5224,26 +5420,31 @@
       <c r="S40" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T40" s="3" t="inlineStr">
+      <c r="T40" s="2" t="inlineStr">
+        <is>
+          <t>What are you working on? ✍️ Tell us, and we'll keep you company.</t>
+        </is>
+      </c>
+      <c r="U40" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 90 --raiz 639 --modo yo --semilla 281608 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U40" s="2" t="inlineStr">
+      <c r="V40" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 5440 audio/OBRA-039_capa.wav --semilla 281608 --raiz 639 --densidad 2 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-039_639_yo.wav audio/OBRA-039_final.wav --fondo selva --nivel-capa -2 --capa audio/OBRA-039_capa.wav</t>
         </is>
       </c>
-      <c r="V40" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W40" s="4" t="inlineStr"/>
+      <c r="W40" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X40" s="4" t="inlineStr"/>
       <c r="Y40" s="4" t="inlineStr"/>
-      <c r="Z40" s="5">
-        <f>IFERROR(Y40/X40*1000,"")</f>
+      <c r="Z40" s="4" t="inlineStr"/>
+      <c r="AA40" s="5">
+        <f>IFERROR(Z40/Y40*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -5341,26 +5542,31 @@
       <c r="S41" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T41" s="3" t="inlineStr">
+      <c r="T41" s="2" t="inlineStr">
+        <is>
+          <t>What are you working on? ✍️ Tell us, and we'll keep you company.</t>
+        </is>
+      </c>
+      <c r="U41" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 741 --modo yo --semilla 883876 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U41" s="2" t="inlineStr">
+      <c r="V41" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py aves 10840 audio/OBRA-040_capa.wav --semilla 883876 --raiz 741 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-040_741_yo.wav audio/OBRA-040_final.wav --fondo mar --nivel-capa -4 --capa audio/OBRA-040_capa.wav</t>
         </is>
       </c>
-      <c r="V41" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W41" s="4" t="inlineStr"/>
+      <c r="W41" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X41" s="4" t="inlineStr"/>
       <c r="Y41" s="4" t="inlineStr"/>
-      <c r="Z41" s="5">
-        <f>IFERROR(Y41/X41*1000,"")</f>
+      <c r="Z41" s="4" t="inlineStr"/>
+      <c r="AA41" s="5">
+        <f>IFERROR(Z41/Y41*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -5459,30 +5665,35 @@
       <c r="S42" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T42" s="3" t="inlineStr">
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>What's on your mind right now? 🌿 Write it here and leave it with us. Sometimes saying it is enough to set it down.</t>
+        </is>
+      </c>
+      <c r="U42" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 60 --raiz 432 --modo hirajoshi --semilla 304617 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U42" s="2" t="inlineStr">
+      <c r="V42" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py jardin 3640 audio/OBRA-041_capa.wav --semilla 304617 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-041_432_hirajoshi.wav audio/OBRA-041_final.wav --fondo mar --nivel-fondo -8 --nivel-capa 0 --capa audio/OBRA-041_capa.wav</t>
         </is>
       </c>
-      <c r="V42" s="4" t="inlineStr">
+      <c r="W42" s="4" t="inlineStr">
         <is>
           <t>publicada</t>
         </is>
       </c>
-      <c r="W42" s="4" t="inlineStr">
+      <c r="X42" s="4" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="X42" s="4" t="inlineStr"/>
       <c r="Y42" s="4" t="inlineStr"/>
-      <c r="Z42" s="5">
-        <f>IFERROR(Y42/X42*1000,"")</f>
+      <c r="Z42" s="4" t="inlineStr"/>
+      <c r="AA42" s="5">
+        <f>IFERROR(Z42/Y42*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -5581,30 +5792,35 @@
       <c r="S43" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T43" s="3" t="inlineStr">
+      <c r="T43" s="2" t="inlineStr">
+        <is>
+          <t>What's on your mind right now? 🌿 Write it here and leave it with us. Sometimes saying it is enough to set it down.</t>
+        </is>
+      </c>
+      <c r="U43" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 528 --modo shin --semilla 266691 --caracter sin-cuenco</t>
         </is>
       </c>
-      <c r="U43" s="2" t="inlineStr">
+      <c r="V43" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py zen 10840 audio/OBRA-042_capa.wav --semilla 266691 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-042_528_shin.wav audio/OBRA-042_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-042_capa.wav</t>
         </is>
       </c>
-      <c r="V43" s="4" t="inlineStr">
+      <c r="W43" s="4" t="inlineStr">
         <is>
           <t>publicada</t>
         </is>
       </c>
-      <c r="W43" s="4" t="inlineStr">
+      <c r="X43" s="4" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="X43" s="4" t="inlineStr"/>
       <c r="Y43" s="4" t="inlineStr"/>
-      <c r="Z43" s="5">
-        <f>IFERROR(Y43/X43*1000,"")</f>
+      <c r="Z43" s="4" t="inlineStr"/>
+      <c r="AA43" s="5">
+        <f>IFERROR(Z43/Y43*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -5703,30 +5919,35 @@
       <c r="S44" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="T44" s="3" t="inlineStr">
+      <c r="T44" s="2" t="inlineStr">
+        <is>
+          <t>How long did the rain take to put you to sleep? 🌧️ Tell us in minutes. If you're reading this awake: lights off, phone face down, and press play again.</t>
+        </is>
+      </c>
+      <c r="U44" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 432 --modo kumoi --semilla 615127 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U44" s="2" t="inlineStr">
+      <c r="V44" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/ambiente.py audio/OBRA-043_432_kumoi.wav audio/OBRA-043_final.wav --fondo lluvia</t>
         </is>
       </c>
-      <c r="V44" s="4" t="inlineStr">
+      <c r="W44" s="4" t="inlineStr">
         <is>
           <t>publicada</t>
         </is>
       </c>
-      <c r="W44" s="4" t="inlineStr">
+      <c r="X44" s="4" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="X44" s="4" t="inlineStr"/>
       <c r="Y44" s="4" t="inlineStr"/>
-      <c r="Z44" s="5">
-        <f>IFERROR(Y44/X44*1000,"")</f>
+      <c r="Z44" s="4" t="inlineStr"/>
+      <c r="AA44" s="5">
+        <f>IFERROR(Z44/Y44*1000,"")</f>
         <v/>
       </c>
     </row>
@@ -5822,31 +6043,36 @@
       <c r="S45" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="T45" s="3" t="inlineStr">
+      <c r="T45" s="2" t="inlineStr">
+        <is>
+          <t>Headphones or speaker? 🎧 Tell us which, and how far into the theta waves you got before falling asleep.</t>
+        </is>
+      </c>
+      <c r="U45" s="3" t="inlineStr">
         <is>
           <t>python3 03-composicion/compositor.py --minutos 180 --raiz 432 --modo shin --semilla 810318 --caracter sin-cuenco --registro grave</t>
         </is>
       </c>
-      <c r="U45" s="2" t="inlineStr">
+      <c r="V45" s="2" t="inlineStr">
         <is>
           <t>python3 03-composicion/capas.py theta 10840 audio/OBRA-044_capa.wav --semilla 810318 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-044_432_shin.wav audio/OBRA-044_final.wav --fondo mar --nivel-fondo -4 --nivel-capa -11 --capa audio/OBRA-044_capa.wav</t>
         </is>
       </c>
-      <c r="V45" s="4" t="inlineStr">
-        <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W45" s="4" t="inlineStr"/>
+      <c r="W45" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
       <c r="X45" s="4" t="inlineStr"/>
       <c r="Y45" s="4" t="inlineStr"/>
-      <c r="Z45" s="5">
-        <f>IFERROR(Y45/X45*1000,"")</f>
+      <c r="Z45" s="4" t="inlineStr"/>
+      <c r="AA45" s="5">
+        <f>IFERROR(Z45/Y45*1000,"")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z45"/>
+  <autoFilter ref="A1:AA45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27850,7 +28076,7 @@
         </is>
       </c>
       <c r="B3" s="7">
-        <f>COUNTIF(Catálogo!V2:V45,"pendiente")</f>
+        <f>COUNTIF(Catálogo!W2:W45,"pendiente")</f>
         <v/>
       </c>
     </row>
@@ -27861,7 +28087,7 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>COUNTIF(Catálogo!V2:V45,"compuesta")</f>
+        <f>COUNTIF(Catálogo!W2:W45,"compuesta")</f>
         <v/>
       </c>
     </row>
@@ -27872,7 +28098,7 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF(Catálogo!V2:V45,"montada")</f>
+        <f>COUNTIF(Catálogo!W2:W45,"montada")</f>
         <v/>
       </c>
     </row>
@@ -27883,7 +28109,7 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF(Catálogo!V2:V45,"publicada")</f>
+        <f>COUNTIF(Catálogo!W2:W45,"publicada")</f>
         <v/>
       </c>
     </row>
@@ -27927,7 +28153,7 @@
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>COUNTIFS(Catálogo!D2:D45,A10,Catálogo!V2:V45,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D45,A10,Catálogo!W2:W45,"publicada")</f>
         <v/>
       </c>
       <c r="D10" s="7">
@@ -27946,7 +28172,7 @@
         <v/>
       </c>
       <c r="C11" s="7">
-        <f>COUNTIFS(Catálogo!D2:D45,A11,Catálogo!V2:V45,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D45,A11,Catálogo!W2:W45,"publicada")</f>
         <v/>
       </c>
       <c r="D11" s="7">
@@ -27965,7 +28191,7 @@
         <v/>
       </c>
       <c r="C12" s="7">
-        <f>COUNTIFS(Catálogo!D2:D45,A12,Catálogo!V2:V45,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D45,A12,Catálogo!W2:W45,"publicada")</f>
         <v/>
       </c>
       <c r="D12" s="7">
@@ -27984,7 +28210,7 @@
         <v/>
       </c>
       <c r="C13" s="7">
-        <f>COUNTIFS(Catálogo!D2:D45,A13,Catálogo!V2:V45,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D45,A13,Catálogo!W2:W45,"publicada")</f>
         <v/>
       </c>
       <c r="D13" s="7">
@@ -28003,7 +28229,7 @@
         <v/>
       </c>
       <c r="C14" s="7">
-        <f>COUNTIFS(Catálogo!D2:D45,A14,Catálogo!V2:V45,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D45,A14,Catálogo!W2:W45,"publicada")</f>
         <v/>
       </c>
       <c r="D14" s="7">
@@ -28044,7 +28270,7 @@
         </is>
       </c>
       <c r="B18" s="7">
-        <f>SUM(Catálogo!X2:X45)</f>
+        <f>SUM(Catálogo!Y2:Y45)</f>
         <v/>
       </c>
     </row>
@@ -28055,7 +28281,7 @@
         </is>
       </c>
       <c r="B19" s="7">
-        <f>SUM(Catálogo!Y2:Y45)</f>
+        <f>SUM(Catálogo!Z2:Z45)</f>
         <v/>
       </c>
     </row>
@@ -28086,7 +28312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -28217,220 +28443,232 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>pantalla_oscura_min</t>
+          <t>comentario_fijado</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Minutos de mandala antes de que la pantalla se funda a negro (videos para dormir). 0: el mandala dura todo el video.</t>
+          <t>Comentario para escribir y fijar apenas se publica: una pregunta fácil de contestar.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>descripcion_optimizada</t>
+          <t>pantalla_oscura_min</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Descripción bilingüe lista para pegar. Solo falta añadir los capítulos tras el montaje.</t>
+          <t>Minutos de mandala antes de que la pantalla se funda a negro (videos para dormir). 0: el mandala dura todo el video.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>titulo_miniatura</t>
+          <t>descripcion_optimizada</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Texto de la miniatura: 2-4 palabras que COMPLETAN el título, nunca lo repiten.</t>
+          <t>Descripción bilingüe lista para pegar. Solo falta añadir los capítulos tras el montaje.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>hashtags</t>
+          <t>titulo_miniatura</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Tres, al final de la descripción.</t>
+          <t>Texto de la miniatura: 2-4 palabras que COMPLETAN el título, nunca lo repiten.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>etiquetas</t>
+          <t>hashtags</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Etiquetas del video, separadas por coma.</t>
+          <t>Tres, al final de la descripción.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>imagen_miniatura</t>
+          <t>etiquetas</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>AMARILLA. Ruta o URL de la portada una vez generada.</t>
+          <t>Etiquetas del video, separadas por coma.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>url_video</t>
+          <t>imagen_miniatura</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>AMARILLA. URL de YouTube una vez publicado.</t>
+          <t>AMARILLA. Ruta o URL de la portada una vez generada.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>raiz_hz / modo / registro / semilla</t>
+          <t>url_video</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Parámetros de composición. El registro grave baja una octava (Dormir y Concentración). La semilla regenera la obra idéntica.</t>
+          <t>AMARILLA. URL de YouTube una vez publicado.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>comando_regeneracion</t>
+          <t>raiz_hz / modo / registro / semilla</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Comando exacto. Copiar, pegar y ejecutar: devuelve el mismo audio bit a bit.</t>
+          <t>Parámetros de composición. El registro grave baja una octava (Dormir y Concentración). La semilla regenera la obra idéntica.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>estado</t>
+          <t>comando_regeneracion</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>AMARILLA. pendiente / compuesta / montada / publicada</t>
+          <t>Comando exacto. Copiar, pegar y ejecutar: devuelve el mismo audio bit a bit.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>fecha_publicacion</t>
+          <t>estado</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>AMARILLA. Formato AAAA-MM-DD.</t>
+          <t>AMARILLA. pendiente / compuesta / montada / publicada</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>vistas / suscriptores</t>
+          <t>fecha_publicacion</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>AMARILLA. Copiar de YouTube Studio a los 14 días de publicar.</t>
+          <t>AMARILLA. Formato AAAA-MM-DD.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
+          <t>vistas / suscriptores</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>AMARILLA. Copiar de YouTube Studio a los 14 días de publicar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
           <t>subs_por_1000</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>Calculada. Es la métrica que decide el canal: por debajo de 1, el problema es la portada, no la música.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr"/>
-    </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>Hoja Shorts</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>5 por obra. Cada uno cambia de tramo de la obra, encuadre, instante del mandala y frase.</t>
-        </is>
-      </c>
+      <c r="A27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>tiktok_portada</t>
+          <t>Hoja Shorts</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>El título de la portada en TikTok (el que se ve en el perfil). Distinto de la descripción.</t>
+          <t>5 por obra. Cada uno cambia de tramo de la obra, encuadre, instante del mandala y frase.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>tiktok_descripcion</t>
+          <t>tiktok_portada</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>El texto que acompaña al video en TikTok, con hashtags. En Metricool, nunca en el campo título.</t>
+          <t>El título de la portada en TikTok (el que se ve en el perfil). Distinto de la descripción.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
+          <t>tiktok_descripcion</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>El texto que acompaña al video en TikTok, con hashtags. En Metricool, nunca en el campo título.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
           <t>yt_video_relacionado</t>
         </is>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>El video largo. En YouTube Studio va en «Video relacionado» del Short.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr"/>
-    </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>Ejemplo de fila rellenada</t>
         </is>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>imagen_miniatura: portadas/obra-001.png | url_video: https://youtu.be/XXXXXXXXXXX | estado: publicada | fecha_publicacion: 2026-10-07 | vistas: 4820 | suscriptores: 11</t>
         </is>

</xml_diff>

<commit_message>
OBRA-045: Woke Up at 3 AM? Guqin y lluvia, 3 h, la versión larga del TikTok
- tao_largo.py: el guqin de tao.py en tramos de 4 min con semilla propia,
  un solo ciclo respiratorio (4.5 -> 3.5) y las colas de la sala que pasan de
  un tramo al otro: tres horas sin repetir ni costuras, en memoria acotada.
  La música se retira con las horas (frases, xiao, −4 dB) y queda la lluvia.
- montar.py: el script de composición sale del catálogo
- ambiente «guqin»: lluvia a −6 dB bajo la obra (~8 dB; en el TikTok 12,7)
- mismo jade que el TikTok, miniatura «WOKE UP AT 3 AM? · FALL BACK ASLEEP»
- Shorts de la primera media hora, cuando todavía suenan guqin y xiao

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$AA$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$301</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$AA$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$304</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA45"/>
+  <dimension ref="A1:AA46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6071,8 +6071,127 @@
         <v/>
       </c>
     </row>
+    <row r="46" ht="58" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-045</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Woke Up at 3 AM? 🌙 Chinese Guqin &amp; Rain to Fall Back Asleep · Dark Screen · 3 Hours</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Música para dormir · Guqin y lluvia · 432 Hz · Las tres de la mañana · 3 horas</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Dormir</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>guqin</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Woke up at 3 AM again? Three hours of guqin, xiao flute and gentle rain to fall back asleep.
+In the Chinese body clock, 1 to 3 AM is the liver's hour: the hour of what you couldn't let go of. Don't check the time. Breathe out slowly through your lips, "shhh" (xū), six times, and let the strings take it from there. The screen fades to black after 3 minutes.
+🌙 Phone face down, volume low. The music thins out over the hours, until only the rain is left.
+🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+Original composition by Rin, synthesized from scratch in just intonation around 432 Hz, yu mode. No samples. The yu scale is the one Chinese five-element music keeps for the night. A 2,000-year-old tradition, not medical advice.
+#sleepmusic #guqin #chinesemusic</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Las tres de la mañana · 3 horas
+Para acompañar el sueño.
+Ambiente: guqin y lluvia.
+Compuesta con raíz en 432 Hz, en entonación justa, modo yu.
+Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
+Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#sleepmusic #meditation #432hz</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>3 HOURS</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>#sleepmusic #guqin #chinesemusic</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>woke up at 3am, fall back asleep, music to fall back asleep, chinese sleep music, guqin, guqin music, chinese meditation music, chinese music for sleep, rain sounds for sleeping, dark screen sleep music, black screen sleep music, deep sleep music, sleep music, traditional chinese medicine, chinamaxxing, 3 hours, rin, música para dormir</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr"/>
+      <c r="L46" s="4" t="inlineStr"/>
+      <c r="M46" s="2" t="n">
+        <v>432</v>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>yu</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>grave</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="n">
+        <v>270978</v>
+      </c>
+      <c r="Q46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R46" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="S46" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="T46" s="2" t="inlineStr">
+        <is>
+          <t>What time did you wake up tonight? 🌙 Tell us, then press play and breathe out slowly: shhh.</t>
+        </is>
+      </c>
+      <c r="U46" s="3" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/tao_largo.py --minutos 180 --raiz 432 --modo yu --semilla 270978</t>
+        </is>
+      </c>
+      <c r="V46" s="2" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/ambiente.py audio/OBRA-045_432_yu.wav audio/OBRA-045_final.wav --fondo lluvia --nivel-obra 0 --nivel-fondo -6 --entrada-obra 6</t>
+        </is>
+      </c>
+      <c r="W46" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="X46" s="4" t="inlineStr"/>
+      <c r="Y46" s="4" t="inlineStr"/>
+      <c r="Z46" s="4" t="inlineStr"/>
+      <c r="AA46" s="5">
+        <f>IFERROR(Z46/Y46*1000,"")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA45"/>
+  <autoFilter ref="A1:AA46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6083,7 +6202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S301"/>
+  <dimension ref="A1:S304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -28029,8 +28148,224 @@
       <c r="R301" s="4" t="inlineStr"/>
       <c r="S301" s="4" t="inlineStr"/>
     </row>
+    <row r="302" ht="58" customHeight="1">
+      <c r="A302" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-045-S1</t>
+        </is>
+      </c>
+      <c r="B302" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-045</t>
+        </is>
+      </c>
+      <c r="C302" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D302" s="2" t="inlineStr">
+        <is>
+          <t>short-1.mp4</t>
+        </is>
+      </c>
+      <c r="E302" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="F302" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G302" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H302" s="2" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in</t>
+        </is>
+      </c>
+      <c r="I302" s="3" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in · 432 Hz · Guqin and Rain</t>
+        </is>
+      </c>
+      <c r="J302" s="3" t="inlineStr">
+        <is>
+          <t>Save this for tonight.
+Full piece (3 h): Woke Up at 3 AM? 🌙 Chinese Guqin &amp; Rain to Fall Back Asleep · Dark Screen · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K302" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, guqin and rain, Rin</t>
+        </is>
+      </c>
+      <c r="L302" s="2" t="inlineStr"/>
+      <c r="M302" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · sleep</t>
+        </is>
+      </c>
+      <c r="N302" s="3" t="inlineStr">
+        <is>
+          <t>Save this for tonight. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O302" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P302" s="4" t="inlineStr"/>
+      <c r="Q302" s="4" t="inlineStr"/>
+      <c r="R302" s="4" t="inlineStr"/>
+      <c r="S302" s="4" t="inlineStr"/>
+    </row>
+    <row r="303" ht="58" customHeight="1">
+      <c r="A303" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-045-S2</t>
+        </is>
+      </c>
+      <c r="B303" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-045</t>
+        </is>
+      </c>
+      <c r="C303" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D303" s="2" t="inlineStr">
+        <is>
+          <t>short-2.mp4</t>
+        </is>
+      </c>
+      <c r="E303" s="2" t="n">
+        <v>960</v>
+      </c>
+      <c r="F303" s="2" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G303" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H303" s="2" t="inlineStr">
+        <is>
+          <t>Unclench your jaw. Let the pillow hold you</t>
+        </is>
+      </c>
+      <c r="I303" s="3" t="inlineStr">
+        <is>
+          <t>Unclench your jaw. Let the pillow hold you · 432 Hz · Guqin and Rain</t>
+        </is>
+      </c>
+      <c r="J303" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, volume low.
+Full piece (3 h): Woke Up at 3 AM? 🌙 Chinese Guqin &amp; Rain to Fall Back Asleep · Dark Screen · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K303" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, guqin and rain, Rin</t>
+        </is>
+      </c>
+      <c r="L303" s="2" t="inlineStr"/>
+      <c r="M303" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · night</t>
+        </is>
+      </c>
+      <c r="N303" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, volume low. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O303" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P303" s="4" t="inlineStr"/>
+      <c r="Q303" s="4" t="inlineStr"/>
+      <c r="R303" s="4" t="inlineStr"/>
+      <c r="S303" s="4" t="inlineStr"/>
+    </row>
+    <row r="304" ht="58" customHeight="1">
+      <c r="A304" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-045-S3</t>
+        </is>
+      </c>
+      <c r="B304" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-045</t>
+        </is>
+      </c>
+      <c r="C304" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D304" s="2" t="inlineStr">
+        <is>
+          <t>short-3.mp4</t>
+        </is>
+      </c>
+      <c r="E304" s="2" t="n">
+        <v>1980</v>
+      </c>
+      <c r="F304" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G304" s="2" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H304" s="2" t="inlineStr">
+        <is>
+          <t>Close your eyes. Just listen</t>
+        </is>
+      </c>
+      <c r="I304" s="3" t="inlineStr">
+        <is>
+          <t>Close your eyes. Just listen · 432 Hz · Guqin and Rain</t>
+        </is>
+      </c>
+      <c r="J304" s="3" t="inlineStr">
+        <is>
+          <t>Stay until your breathing slows.
+Full piece (3 h): Woke Up at 3 AM? 🌙 Chinese Guqin &amp; Rain to Fall Back Asleep · Dark Screen · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K304" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, guqin and rain, Rin</t>
+        </is>
+      </c>
+      <c r="L304" s="2" t="inlineStr"/>
+      <c r="M304" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · rest</t>
+        </is>
+      </c>
+      <c r="N304" s="3" t="inlineStr">
+        <is>
+          <t>Stay until your breathing slows. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O304" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P304" s="4" t="inlineStr"/>
+      <c r="Q304" s="4" t="inlineStr"/>
+      <c r="R304" s="4" t="inlineStr"/>
+      <c r="S304" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S301"/>
+  <autoFilter ref="A1:S304"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -28065,7 +28400,7 @@
         </is>
       </c>
       <c r="B2" s="7">
-        <f>COUNTA(Catálogo!A2:A45)</f>
+        <f>COUNTA(Catálogo!A2:A46)</f>
         <v/>
       </c>
     </row>
@@ -28076,7 +28411,7 @@
         </is>
       </c>
       <c r="B3" s="7">
-        <f>COUNTIF(Catálogo!W2:W45,"pendiente")</f>
+        <f>COUNTIF(Catálogo!W2:W46,"pendiente")</f>
         <v/>
       </c>
     </row>
@@ -28087,7 +28422,7 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>COUNTIF(Catálogo!W2:W45,"compuesta")</f>
+        <f>COUNTIF(Catálogo!W2:W46,"compuesta")</f>
         <v/>
       </c>
     </row>
@@ -28098,7 +28433,7 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF(Catálogo!W2:W45,"montada")</f>
+        <f>COUNTIF(Catálogo!W2:W46,"montada")</f>
         <v/>
       </c>
     </row>
@@ -28109,7 +28444,7 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF(Catálogo!W2:W45,"publicada")</f>
+        <f>COUNTIF(Catálogo!W2:W46,"publicada")</f>
         <v/>
       </c>
     </row>
@@ -28149,15 +28484,15 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Catálogo!D2:D45,A10)</f>
+        <f>COUNTIF(Catálogo!D2:D46,A10)</f>
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>COUNTIFS(Catálogo!D2:D45,A10,Catálogo!W2:W45,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D46,A10,Catálogo!W2:W46,"publicada")</f>
         <v/>
       </c>
       <c r="D10" s="7">
-        <f>SUMIF(Catálogo!D2:D45,A10,Catálogo!R2:R45)</f>
+        <f>SUMIF(Catálogo!D2:D46,A10,Catálogo!R2:R46)</f>
         <v/>
       </c>
     </row>
@@ -28168,15 +28503,15 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Catálogo!D2:D45,A11)</f>
+        <f>COUNTIF(Catálogo!D2:D46,A11)</f>
         <v/>
       </c>
       <c r="C11" s="7">
-        <f>COUNTIFS(Catálogo!D2:D45,A11,Catálogo!W2:W45,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D46,A11,Catálogo!W2:W46,"publicada")</f>
         <v/>
       </c>
       <c r="D11" s="7">
-        <f>SUMIF(Catálogo!D2:D45,A11,Catálogo!R2:R45)</f>
+        <f>SUMIF(Catálogo!D2:D46,A11,Catálogo!R2:R46)</f>
         <v/>
       </c>
     </row>
@@ -28187,15 +28522,15 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Catálogo!D2:D45,A12)</f>
+        <f>COUNTIF(Catálogo!D2:D46,A12)</f>
         <v/>
       </c>
       <c r="C12" s="7">
-        <f>COUNTIFS(Catálogo!D2:D45,A12,Catálogo!W2:W45,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D46,A12,Catálogo!W2:W46,"publicada")</f>
         <v/>
       </c>
       <c r="D12" s="7">
-        <f>SUMIF(Catálogo!D2:D45,A12,Catálogo!R2:R45)</f>
+        <f>SUMIF(Catálogo!D2:D46,A12,Catálogo!R2:R46)</f>
         <v/>
       </c>
     </row>
@@ -28206,15 +28541,15 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Catálogo!D2:D45,A13)</f>
+        <f>COUNTIF(Catálogo!D2:D46,A13)</f>
         <v/>
       </c>
       <c r="C13" s="7">
-        <f>COUNTIFS(Catálogo!D2:D45,A13,Catálogo!W2:W45,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D46,A13,Catálogo!W2:W46,"publicada")</f>
         <v/>
       </c>
       <c r="D13" s="7">
-        <f>SUMIF(Catálogo!D2:D45,A13,Catálogo!R2:R45)</f>
+        <f>SUMIF(Catálogo!D2:D46,A13,Catálogo!R2:R46)</f>
         <v/>
       </c>
     </row>
@@ -28225,15 +28560,15 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Catálogo!D2:D45,A14)</f>
+        <f>COUNTIF(Catálogo!D2:D46,A14)</f>
         <v/>
       </c>
       <c r="C14" s="7">
-        <f>COUNTIFS(Catálogo!D2:D45,A14,Catálogo!W2:W45,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D46,A14,Catálogo!W2:W46,"publicada")</f>
         <v/>
       </c>
       <c r="D14" s="7">
-        <f>SUMIF(Catálogo!D2:D45,A14,Catálogo!R2:R45)</f>
+        <f>SUMIF(Catálogo!D2:D46,A14,Catálogo!R2:R46)</f>
         <v/>
       </c>
     </row>
@@ -28270,7 +28605,7 @@
         </is>
       </c>
       <c r="B18" s="7">
-        <f>SUM(Catálogo!Y2:Y45)</f>
+        <f>SUM(Catálogo!Y2:Y46)</f>
         <v/>
       </c>
     </row>
@@ -28281,7 +28616,7 @@
         </is>
       </c>
       <c r="B19" s="7">
-        <f>SUM(Catálogo!Z2:Z45)</f>
+        <f>SUM(Catálogo!Z2:Z46)</f>
         <v/>
       </c>
     </row>
@@ -28424,7 +28759,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Ambiente aprobado en escucha: mar, mar-aves, zen, selva, lluvia-tambor, jardin, lluvia o theta.</t>
+          <t>Ambiente aprobado en escucha: mar, mar-aves, zen, selva, lluvia-tambor, jardin, lluvia, theta o guqin.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Calendario de 15 días: obras 46–49 (3 AM Reset, 5-Minute Reset, Temple Bells 3 h, Stop Overthinking 10 min)
La música entra a los 8 s en vez de 15 (el de 10 minutos perdía a la gente a
los 40 s). Los Shorts del guqin solo usan los tramos fijos si la obra dura
40 minutos o más.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$AA$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$304</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$AA$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$316</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA46"/>
+  <dimension ref="A1:AA50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6190,8 +6190,484 @@
         <v/>
       </c>
     </row>
+    <row r="47" ht="58" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-046</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>3 AM Reset 🌙 10 Minutes of Guqin &amp; Rain to Fall Back Asleep · Chinese Sleep Music</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Música para dormir · Guqin y lluvia · 432 Hz · Volver a dormir · 10 minutos</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Dormir</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>guqin</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Woke up at 3 AM? Ten minutes of guqin, xiao flute and gentle rain to fall back asleep.
+Don't check the time. Breathe out slowly through your lips, "shhh", six times, and let the strings take it from there.
+🌙 Phone face down, volume low. If you're still awake at the end, the full 3 hours are on the channel.
+🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+Original composition by Rin, synthesized from scratch in just intonation around 432 Hz, yu mode. No samples. The yu scale is the one Chinese five-element music keeps for the night. A 2,000-year-old tradition, not medical advice.
+#sleepmusic #guqin #3am</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Volver a dormir · 10 minutos
+Para acompañar el sueño.
+Ambiente: guqin y lluvia.
+Compuesta con raíz en 432 Hz, en entonación justa, modo yu.
+Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
+Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#sleepmusic #meditation #432hz</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>10 MIN</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>#sleepmusic #guqin #3am</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>3am reset, fall back asleep, woke up at 3am, music to fall back asleep, guqin, chinese sleep music, 10 minute sleep music, rain sounds for sleeping, sleep music, chinese meditation music, rin, música para dormir</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr"/>
+      <c r="L47" s="4" t="inlineStr"/>
+      <c r="M47" s="2" t="n">
+        <v>432</v>
+      </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>yu</t>
+        </is>
+      </c>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>grave</t>
+        </is>
+      </c>
+      <c r="P47" s="2" t="n">
+        <v>926874</v>
+      </c>
+      <c r="Q47" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="R47" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="S47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T47" s="2" t="inlineStr">
+        <is>
+          <t>What time did you wake up tonight? 🌙 Tell us, then breathe out slowly: shhh.</t>
+        </is>
+      </c>
+      <c r="U47" s="3" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/tao_largo.py --minutos 10 --raiz 432 --modo yu --semilla 926874</t>
+        </is>
+      </c>
+      <c r="V47" s="2" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/ambiente.py audio/OBRA-046_432_yu.wav audio/OBRA-046_final.wav --fondo lluvia --nivel-obra 0 --nivel-fondo -6 --entrada-obra 6</t>
+        </is>
+      </c>
+      <c r="W47" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="X47" s="4" t="inlineStr"/>
+      <c r="Y47" s="4" t="inlineStr"/>
+      <c r="Z47" s="4" t="inlineStr"/>
+      <c r="AA47" s="5">
+        <f>IFERROR(Z47/Y47*1000,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="58" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-047</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>5-Minute Nervous System Reset 🔔 Zen Temple Bells to Calm Anxiety Fast · 528 Hz</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Música para momentos de ansiedad · Templo zen · 528 Hz · Reinicio de cinco minutos · 5 minutos</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Ansiedad</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>zen</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Five minutes to calm your nervous system: zen temple bells over a warm, slow drone.
+Drop your shoulders. Breathe out longer than you breathe in, and let the bells keep you company until the end.
+🎧 Use it between meetings, before a hard conversation, or whenever your chest feels tight.
+🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+Original composition by Rin, synthesized from scratch in just intonation around 528 Hz, shin mode. No samples.
+#nervoussystemreset #anxietyrelief #528hz</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Reinicio de cinco minutos · 5 minutos
+Para acompañar un momento de pausa cuando la cabeza no para.
+Ambiente: templo zen.
+Compuesta con raíz en 528 Hz, en entonación justa, modo shin.
+Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
+Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#relaxingmusic #meditation #528hz</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>5 MIN</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>#nervoussystemreset #anxietyrelief #528hz</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>nervous system reset, 5 minute nervous system reset, calm anxiety fast, anxiety relief, 5 minute meditation, zen temple bells, temple bells, calming music, 528 hz, nervous system regulation, quick calm, rin, música para la ansiedad</t>
+        </is>
+      </c>
+      <c r="K48" s="4" t="inlineStr"/>
+      <c r="L48" s="4" t="inlineStr"/>
+      <c r="M48" s="2" t="n">
+        <v>528</v>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>shin</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>medio</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="n">
+        <v>756077</v>
+      </c>
+      <c r="Q48" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="R48" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T48" s="2" t="inlineStr">
+        <is>
+          <t>Where are you listening from right now? 🔔 Work, bed, car? Tell us.</t>
+        </is>
+      </c>
+      <c r="U48" s="3" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/compositor.py --minutos 5 --raiz 528 --modo shin --semilla 756077 --caracter sin-cuenco</t>
+        </is>
+      </c>
+      <c r="V48" s="2" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/capas.py zen 340 audio/OBRA-047_capa.wav --semilla 756077 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-047_528_shin.wav audio/OBRA-047_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-047_capa.wav</t>
+        </is>
+      </c>
+      <c r="W48" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="X48" s="4" t="inlineStr"/>
+      <c r="Y48" s="4" t="inlineStr"/>
+      <c r="Z48" s="4" t="inlineStr"/>
+      <c r="AA48" s="5">
+        <f>IFERROR(Z48/Y48*1000,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="58" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-048</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Zen Temple Bells for Deep Sleep 🌙 Dark Screen · Calm Your Mind · 432 Hz · 3 Hours</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Música para dormir · Templo zen · 432 Hz · Campanas para dormir · 3 horas</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Dormir</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>zen</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Three hours of soft zen temple bells over a distant ocean, for deep sleep.
+The bells grow sparse as the night goes on. The screen fades to black after 3 minutes, so no light keeps you awake.
+🌙 Lights off, phone face down, volume low.
+🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+Original composition by Rin, synthesized from scratch in just intonation around 216 Hz, the low octave of 432 Hz, kumoi mode. No samples.
+#sleepmusic #templebells #darkscreen</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Campanas para dormir · 3 horas
+Para acompañar el sueño.
+Ambiente: templo zen.
+Compuesta con raíz en 216 Hz, la octava grave de 432 Hz, en entonación justa, modo kumoi.
+Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
+Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#sleepmusic #meditation #432hz</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>3 HOURS</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>#sleepmusic #templebells #darkscreen</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>zen temple bells, temple bells sleep, zen sleep music, dark screen sleep music, black screen sleep music, deep sleep music, sleep music, calm your mind, zen music, meditation music, 432 hz, 3 hours, rin, música para dormir</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr"/>
+      <c r="L49" s="4" t="inlineStr"/>
+      <c r="M49" s="2" t="n">
+        <v>432</v>
+      </c>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>kumoi</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>grave</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="n">
+        <v>762820</v>
+      </c>
+      <c r="Q49" s="2" t="n">
+        <v>-70</v>
+      </c>
+      <c r="R49" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="S49" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="T49" s="2" t="inlineStr">
+        <is>
+          <t>Do bells help you sleep, or do you prefer rain? 🔔🌧️ Tell us, it shapes the next piece.</t>
+        </is>
+      </c>
+      <c r="U49" s="3" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/compositor.py --minutos 180 --raiz 432 --modo kumoi --semilla 762820 --caracter sin-cuenco --registro grave</t>
+        </is>
+      </c>
+      <c r="V49" s="2" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/capas.py zen 10840 audio/OBRA-048_capa.wav --semilla 762820 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-048_432_kumoi.wav audio/OBRA-048_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-048_capa.wav</t>
+        </is>
+      </c>
+      <c r="W49" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="X49" s="4" t="inlineStr"/>
+      <c r="Y49" s="4" t="inlineStr"/>
+      <c r="Z49" s="4" t="inlineStr"/>
+      <c r="AA49" s="5">
+        <f>IFERROR(Z49/Y49*1000,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="58" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-049</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Stop Overthinking in 10 Minutes 🌿 Birdsong &amp; Temple Bells · Calming Music · 432 Hz</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Música para momentos de ansiedad · Pájaros y campanas del templo · 432 Hz · Dejar de pensar en diez · 10 minutos</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Ansiedad</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>jardin</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Ten minutes to stop overthinking: birdsong, soft temple bells and a slower breath.
+You don't have to solve it now. Breathe out longer than you breathe in, and just listen to the birds.
+🌿 Headphones on, eyes closed if you can.
+🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+Original composition by Rin, synthesized from scratch in just intonation around 432 Hz, hirajoshi mode. No samples.
+#stopoverthinking #calmingmusic #432hz</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Dejar de pensar en diez · 10 minutos
+Para acompañar un momento de pausa cuando la cabeza no para.
+Ambiente: pájaros y campanas del templo.
+Compuesta con raíz en 432 Hz, en entonación justa, modo hirajoshi.
+Ciclo respiratorio: de 6.0 a 4.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
+Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#relaxingmusic #meditation #432hz</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>10 MIN</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>#stopoverthinking #calmingmusic #432hz</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>stop overthinking, stop overthinking music, 10 minute meditation, calming music, music for anxiety, birdsong, temple bells, anxiety relief, calm your mind, 432 hz, rin, música para la ansiedad</t>
+        </is>
+      </c>
+      <c r="K50" s="4" t="inlineStr"/>
+      <c r="L50" s="4" t="inlineStr"/>
+      <c r="M50" s="2" t="n">
+        <v>432</v>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>hirajoshi</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>medio</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="n">
+        <v>341227</v>
+      </c>
+      <c r="Q50" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="R50" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="S50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T50" s="2" t="inlineStr">
+        <is>
+          <t>What's the thought that won't leave you alone today? 🌿 Write one word. Then let it go.</t>
+        </is>
+      </c>
+      <c r="U50" s="3" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/compositor.py --minutos 10 --raiz 432 --modo hirajoshi --semilla 341227 --caracter sin-cuenco</t>
+        </is>
+      </c>
+      <c r="V50" s="2" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/capas.py jardin 640 audio/OBRA-049_capa.wav --semilla 341227 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-049_432_hirajoshi.wav audio/OBRA-049_final.wav --fondo mar --nivel-fondo -8 --nivel-capa 0 --capa audio/OBRA-049_capa.wav</t>
+        </is>
+      </c>
+      <c r="W50" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="X50" s="4" t="inlineStr"/>
+      <c r="Y50" s="4" t="inlineStr"/>
+      <c r="Z50" s="4" t="inlineStr"/>
+      <c r="AA50" s="5">
+        <f>IFERROR(Z50/Y50*1000,"")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA46"/>
+  <autoFilter ref="A1:AA50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6202,7 +6678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S304"/>
+  <dimension ref="A1:S316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -28364,8 +28840,872 @@
       <c r="R304" s="4" t="inlineStr"/>
       <c r="S304" s="4" t="inlineStr"/>
     </row>
+    <row r="305" ht="58" customHeight="1">
+      <c r="A305" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-046-S1</t>
+        </is>
+      </c>
+      <c r="B305" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-046</t>
+        </is>
+      </c>
+      <c r="C305" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D305" s="2" t="inlineStr">
+        <is>
+          <t>short-1.mp4</t>
+        </is>
+      </c>
+      <c r="E305" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="F305" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G305" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H305" s="2" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in</t>
+        </is>
+      </c>
+      <c r="I305" s="3" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in · 432 Hz · Guqin and Rain</t>
+        </is>
+      </c>
+      <c r="J305" s="3" t="inlineStr">
+        <is>
+          <t>Save this for tonight.
+Full piece (10 min): 3 AM Reset 🌙 10 Minutes of Guqin &amp; Rain to Fall Back Asleep · Chinese Sleep Music
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K305" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, guqin and rain, Rin</t>
+        </is>
+      </c>
+      <c r="L305" s="2" t="inlineStr"/>
+      <c r="M305" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · sleep</t>
+        </is>
+      </c>
+      <c r="N305" s="3" t="inlineStr">
+        <is>
+          <t>Save this for tonight. Full 10 min piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O305" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P305" s="4" t="inlineStr"/>
+      <c r="Q305" s="4" t="inlineStr"/>
+      <c r="R305" s="4" t="inlineStr"/>
+      <c r="S305" s="4" t="inlineStr"/>
+    </row>
+    <row r="306" ht="58" customHeight="1">
+      <c r="A306" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-046-S2</t>
+        </is>
+      </c>
+      <c r="B306" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-046</t>
+        </is>
+      </c>
+      <c r="C306" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D306" s="2" t="inlineStr">
+        <is>
+          <t>short-2.mp4</t>
+        </is>
+      </c>
+      <c r="E306" s="2" t="n">
+        <v>332</v>
+      </c>
+      <c r="F306" s="2" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G306" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H306" s="2" t="inlineStr">
+        <is>
+          <t>Unclench your jaw. Let the pillow hold you</t>
+        </is>
+      </c>
+      <c r="I306" s="3" t="inlineStr">
+        <is>
+          <t>Unclench your jaw. Let the pillow hold you · 432 Hz · Guqin and Rain</t>
+        </is>
+      </c>
+      <c r="J306" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, volume low.
+Full piece (10 min): 3 AM Reset 🌙 10 Minutes of Guqin &amp; Rain to Fall Back Asleep · Chinese Sleep Music
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K306" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, guqin and rain, Rin</t>
+        </is>
+      </c>
+      <c r="L306" s="2" t="inlineStr"/>
+      <c r="M306" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · night</t>
+        </is>
+      </c>
+      <c r="N306" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, volume low. Full 10 min piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O306" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P306" s="4" t="inlineStr"/>
+      <c r="Q306" s="4" t="inlineStr"/>
+      <c r="R306" s="4" t="inlineStr"/>
+      <c r="S306" s="4" t="inlineStr"/>
+    </row>
+    <row r="307" ht="58" customHeight="1">
+      <c r="A307" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-046-S3</t>
+        </is>
+      </c>
+      <c r="B307" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-046</t>
+        </is>
+      </c>
+      <c r="C307" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D307" s="2" t="inlineStr">
+        <is>
+          <t>short-3.mp4</t>
+        </is>
+      </c>
+      <c r="E307" s="2" t="n">
+        <v>575</v>
+      </c>
+      <c r="F307" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G307" s="2" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H307" s="2" t="inlineStr">
+        <is>
+          <t>Close your eyes. Just listen</t>
+        </is>
+      </c>
+      <c r="I307" s="3" t="inlineStr">
+        <is>
+          <t>Close your eyes. Just listen · 432 Hz · Guqin and Rain</t>
+        </is>
+      </c>
+      <c r="J307" s="3" t="inlineStr">
+        <is>
+          <t>Stay until your breathing slows.
+Full piece (10 min): 3 AM Reset 🌙 10 Minutes of Guqin &amp; Rain to Fall Back Asleep · Chinese Sleep Music
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K307" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, guqin and rain, Rin</t>
+        </is>
+      </c>
+      <c r="L307" s="2" t="inlineStr"/>
+      <c r="M307" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · rest</t>
+        </is>
+      </c>
+      <c r="N307" s="3" t="inlineStr">
+        <is>
+          <t>Stay until your breathing slows. Full 10 min piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O307" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P307" s="4" t="inlineStr"/>
+      <c r="Q307" s="4" t="inlineStr"/>
+      <c r="R307" s="4" t="inlineStr"/>
+      <c r="S307" s="4" t="inlineStr"/>
+    </row>
+    <row r="308" ht="58" customHeight="1">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-047-S1</t>
+        </is>
+      </c>
+      <c r="B308" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-047</t>
+        </is>
+      </c>
+      <c r="C308" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D308" s="2" t="inlineStr">
+        <is>
+          <t>short-1.mp4</t>
+        </is>
+      </c>
+      <c r="E308" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="F308" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G308" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H308" s="2" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in</t>
+        </is>
+      </c>
+      <c r="I308" s="3" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in · 528 Hz · Zen Temple</t>
+        </is>
+      </c>
+      <c r="J308" s="3" t="inlineStr">
+        <is>
+          <t>Save this for the next hard moment.
+Full piece (5 min): 5-Minute Nervous System Reset 🔔 Zen Temple Bells to Calm Anxiety Fast · 528 Hz
+#anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
+        </is>
+      </c>
+      <c r="K308" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
+        </is>
+      </c>
+      <c r="L308" s="2" t="inlineStr"/>
+      <c r="M308" s="2" t="inlineStr">
+        <is>
+          <t>528 Hz · calm</t>
+        </is>
+      </c>
+      <c r="N308" s="3" t="inlineStr">
+        <is>
+          <t>Save this for the next hard moment. Full 5 min piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #528hz #meditation</t>
+        </is>
+      </c>
+      <c r="O308" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P308" s="4" t="inlineStr"/>
+      <c r="Q308" s="4" t="inlineStr"/>
+      <c r="R308" s="4" t="inlineStr"/>
+      <c r="S308" s="4" t="inlineStr"/>
+    </row>
+    <row r="309" ht="58" customHeight="1">
+      <c r="A309" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-047-S2</t>
+        </is>
+      </c>
+      <c r="B309" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-047</t>
+        </is>
+      </c>
+      <c r="C309" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D309" s="2" t="inlineStr">
+        <is>
+          <t>short-2.mp4</t>
+        </is>
+      </c>
+      <c r="E309" s="2" t="n">
+        <v>182</v>
+      </c>
+      <c r="F309" s="2" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G309" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H309" s="2" t="inlineStr">
+        <is>
+          <t>Drop your shoulders. Unclench your jaw</t>
+        </is>
+      </c>
+      <c r="I309" s="3" t="inlineStr">
+        <is>
+          <t>Drop your shoulders. Unclench your jaw · 528 Hz · Zen Temple</t>
+        </is>
+      </c>
+      <c r="J309" s="3" t="inlineStr">
+        <is>
+          <t>Headphones on. Exhale slowly.
+Full piece (5 min): 5-Minute Nervous System Reset 🔔 Zen Temple Bells to Calm Anxiety Fast · 528 Hz
+#anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
+        </is>
+      </c>
+      <c r="K309" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
+        </is>
+      </c>
+      <c r="L309" s="2" t="inlineStr"/>
+      <c r="M309" s="2" t="inlineStr">
+        <is>
+          <t>528 Hz · exhale</t>
+        </is>
+      </c>
+      <c r="N309" s="3" t="inlineStr">
+        <is>
+          <t>Headphones on. Exhale slowly. Full 5 min piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #528hz #meditation</t>
+        </is>
+      </c>
+      <c r="O309" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P309" s="4" t="inlineStr"/>
+      <c r="Q309" s="4" t="inlineStr"/>
+      <c r="R309" s="4" t="inlineStr"/>
+      <c r="S309" s="4" t="inlineStr"/>
+    </row>
+    <row r="310" ht="58" customHeight="1">
+      <c r="A310" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-047-S3</t>
+        </is>
+      </c>
+      <c r="B310" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-047</t>
+        </is>
+      </c>
+      <c r="C310" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D310" s="2" t="inlineStr">
+        <is>
+          <t>short-3.mp4</t>
+        </is>
+      </c>
+      <c r="E310" s="2" t="n">
+        <v>275</v>
+      </c>
+      <c r="F310" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G310" s="2" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H310" s="2" t="inlineStr">
+        <is>
+          <t>Hand on your chest. Breathe slower</t>
+        </is>
+      </c>
+      <c r="I310" s="3" t="inlineStr">
+        <is>
+          <t>Hand on your chest. Breathe slower · 528 Hz · Zen Temple</t>
+        </is>
+      </c>
+      <c r="J310" s="3" t="inlineStr">
+        <is>
+          <t>Stay for one full breath.
+Full piece (5 min): 5-Minute Nervous System Reset 🔔 Zen Temple Bells to Calm Anxiety Fast · 528 Hz
+#anxietyrelief #calm #relaxingmusic #528hz #shorts</t>
+        </is>
+      </c>
+      <c r="K310" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 528 hz, zen temple, Rin</t>
+        </is>
+      </c>
+      <c r="L310" s="2" t="inlineStr"/>
+      <c r="M310" s="2" t="inlineStr">
+        <is>
+          <t>528 Hz · pause</t>
+        </is>
+      </c>
+      <c r="N310" s="3" t="inlineStr">
+        <is>
+          <t>Stay for one full breath. Full 5 min piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #528hz #meditation</t>
+        </is>
+      </c>
+      <c r="O310" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P310" s="4" t="inlineStr"/>
+      <c r="Q310" s="4" t="inlineStr"/>
+      <c r="R310" s="4" t="inlineStr"/>
+      <c r="S310" s="4" t="inlineStr"/>
+    </row>
+    <row r="311" ht="58" customHeight="1">
+      <c r="A311" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-048-S1</t>
+        </is>
+      </c>
+      <c r="B311" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-048</t>
+        </is>
+      </c>
+      <c r="C311" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D311" s="2" t="inlineStr">
+        <is>
+          <t>short-1.mp4</t>
+        </is>
+      </c>
+      <c r="E311" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="F311" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G311" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H311" s="2" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in</t>
+        </is>
+      </c>
+      <c r="I311" s="3" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in · 432 Hz · Zen Temple</t>
+        </is>
+      </c>
+      <c r="J311" s="3" t="inlineStr">
+        <is>
+          <t>Save this for tonight.
+Full piece (3 h): Zen Temple Bells for Deep Sleep 🌙 Dark Screen · Calm Your Mind · 432 Hz · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K311" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, zen temple, Rin</t>
+        </is>
+      </c>
+      <c r="L311" s="2" t="inlineStr"/>
+      <c r="M311" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · sleep</t>
+        </is>
+      </c>
+      <c r="N311" s="3" t="inlineStr">
+        <is>
+          <t>Save this for tonight. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O311" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P311" s="4" t="inlineStr"/>
+      <c r="Q311" s="4" t="inlineStr"/>
+      <c r="R311" s="4" t="inlineStr"/>
+      <c r="S311" s="4" t="inlineStr"/>
+    </row>
+    <row r="312" ht="58" customHeight="1">
+      <c r="A312" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-048-S2</t>
+        </is>
+      </c>
+      <c r="B312" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-048</t>
+        </is>
+      </c>
+      <c r="C312" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D312" s="2" t="inlineStr">
+        <is>
+          <t>short-2.mp4</t>
+        </is>
+      </c>
+      <c r="E312" s="2" t="n">
+        <v>5432</v>
+      </c>
+      <c r="F312" s="2" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G312" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H312" s="2" t="inlineStr">
+        <is>
+          <t>Unclench your jaw. Let the pillow hold you</t>
+        </is>
+      </c>
+      <c r="I312" s="3" t="inlineStr">
+        <is>
+          <t>Unclench your jaw. Let the pillow hold you · 432 Hz · Zen Temple</t>
+        </is>
+      </c>
+      <c r="J312" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, volume low.
+Full piece (3 h): Zen Temple Bells for Deep Sleep 🌙 Dark Screen · Calm Your Mind · 432 Hz · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K312" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, zen temple, Rin</t>
+        </is>
+      </c>
+      <c r="L312" s="2" t="inlineStr"/>
+      <c r="M312" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · night</t>
+        </is>
+      </c>
+      <c r="N312" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, volume low. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O312" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P312" s="4" t="inlineStr"/>
+      <c r="Q312" s="4" t="inlineStr"/>
+      <c r="R312" s="4" t="inlineStr"/>
+      <c r="S312" s="4" t="inlineStr"/>
+    </row>
+    <row r="313" ht="58" customHeight="1">
+      <c r="A313" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-048-S3</t>
+        </is>
+      </c>
+      <c r="B313" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-048</t>
+        </is>
+      </c>
+      <c r="C313" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D313" s="2" t="inlineStr">
+        <is>
+          <t>short-3.mp4</t>
+        </is>
+      </c>
+      <c r="E313" s="2" t="n">
+        <v>10775</v>
+      </c>
+      <c r="F313" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G313" s="2" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H313" s="2" t="inlineStr">
+        <is>
+          <t>Close your eyes. Just listen</t>
+        </is>
+      </c>
+      <c r="I313" s="3" t="inlineStr">
+        <is>
+          <t>Close your eyes. Just listen · 432 Hz · Zen Temple</t>
+        </is>
+      </c>
+      <c r="J313" s="3" t="inlineStr">
+        <is>
+          <t>Stay until your breathing slows.
+Full piece (3 h): Zen Temple Bells for Deep Sleep 🌙 Dark Screen · Calm Your Mind · 432 Hz · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K313" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, zen temple, Rin</t>
+        </is>
+      </c>
+      <c r="L313" s="2" t="inlineStr"/>
+      <c r="M313" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · rest</t>
+        </is>
+      </c>
+      <c r="N313" s="3" t="inlineStr">
+        <is>
+          <t>Stay until your breathing slows. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O313" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P313" s="4" t="inlineStr"/>
+      <c r="Q313" s="4" t="inlineStr"/>
+      <c r="R313" s="4" t="inlineStr"/>
+      <c r="S313" s="4" t="inlineStr"/>
+    </row>
+    <row r="314" ht="58" customHeight="1">
+      <c r="A314" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-049-S1</t>
+        </is>
+      </c>
+      <c r="B314" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-049</t>
+        </is>
+      </c>
+      <c r="C314" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D314" s="2" t="inlineStr">
+        <is>
+          <t>short-1.mp4</t>
+        </is>
+      </c>
+      <c r="E314" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="F314" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G314" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H314" s="2" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in</t>
+        </is>
+      </c>
+      <c r="I314" s="3" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in · 432 Hz · Birds and Temple Bells</t>
+        </is>
+      </c>
+      <c r="J314" s="3" t="inlineStr">
+        <is>
+          <t>Save this for the next hard moment.
+Full piece (10 min): Stop Overthinking in 10 Minutes 🌿 Birdsong &amp; Temple Bells · Calming Music · 432 Hz
+#anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K314" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
+        </is>
+      </c>
+      <c r="L314" s="2" t="inlineStr"/>
+      <c r="M314" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · calm</t>
+        </is>
+      </c>
+      <c r="N314" s="3" t="inlineStr">
+        <is>
+          <t>Save this for the next hard moment. Full 10 min piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O314" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P314" s="4" t="inlineStr"/>
+      <c r="Q314" s="4" t="inlineStr"/>
+      <c r="R314" s="4" t="inlineStr"/>
+      <c r="S314" s="4" t="inlineStr"/>
+    </row>
+    <row r="315" ht="58" customHeight="1">
+      <c r="A315" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-049-S2</t>
+        </is>
+      </c>
+      <c r="B315" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-049</t>
+        </is>
+      </c>
+      <c r="C315" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D315" s="2" t="inlineStr">
+        <is>
+          <t>short-2.mp4</t>
+        </is>
+      </c>
+      <c r="E315" s="2" t="n">
+        <v>332</v>
+      </c>
+      <c r="F315" s="2" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G315" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H315" s="2" t="inlineStr">
+        <is>
+          <t>Drop your shoulders. Unclench your jaw</t>
+        </is>
+      </c>
+      <c r="I315" s="3" t="inlineStr">
+        <is>
+          <t>Drop your shoulders. Unclench your jaw · 432 Hz · Birds and Temple Bells</t>
+        </is>
+      </c>
+      <c r="J315" s="3" t="inlineStr">
+        <is>
+          <t>Headphones on. Exhale slowly.
+Full piece (10 min): Stop Overthinking in 10 Minutes 🌿 Birdsong &amp; Temple Bells · Calming Music · 432 Hz
+#anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K315" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
+        </is>
+      </c>
+      <c r="L315" s="2" t="inlineStr"/>
+      <c r="M315" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · exhale</t>
+        </is>
+      </c>
+      <c r="N315" s="3" t="inlineStr">
+        <is>
+          <t>Headphones on. Exhale slowly. Full 10 min piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O315" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P315" s="4" t="inlineStr"/>
+      <c r="Q315" s="4" t="inlineStr"/>
+      <c r="R315" s="4" t="inlineStr"/>
+      <c r="S315" s="4" t="inlineStr"/>
+    </row>
+    <row r="316" ht="58" customHeight="1">
+      <c r="A316" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-049-S3</t>
+        </is>
+      </c>
+      <c r="B316" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-049</t>
+        </is>
+      </c>
+      <c r="C316" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D316" s="2" t="inlineStr">
+        <is>
+          <t>short-3.mp4</t>
+        </is>
+      </c>
+      <c r="E316" s="2" t="n">
+        <v>575</v>
+      </c>
+      <c r="F316" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G316" s="2" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H316" s="2" t="inlineStr">
+        <is>
+          <t>Hand on your chest. Breathe slower</t>
+        </is>
+      </c>
+      <c r="I316" s="3" t="inlineStr">
+        <is>
+          <t>Hand on your chest. Breathe slower · 432 Hz · Birds and Temple Bells</t>
+        </is>
+      </c>
+      <c r="J316" s="3" t="inlineStr">
+        <is>
+          <t>Stay for one full breath.
+Full piece (10 min): Stop Overthinking in 10 Minutes 🌿 Birdsong &amp; Temple Bells · Calming Music · 432 Hz
+#anxietyrelief #calm #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K316" s="2" t="inlineStr">
+        <is>
+          <t>anxiety relief, calming music, 432 hz, birds and temple bells, Rin</t>
+        </is>
+      </c>
+      <c r="L316" s="2" t="inlineStr"/>
+      <c r="M316" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · pause</t>
+        </is>
+      </c>
+      <c r="N316" s="3" t="inlineStr">
+        <is>
+          <t>Stay for one full breath. Full 10 min piece on YouTube: Rin.
+#anxietyrelief #calm #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O316" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P316" s="4" t="inlineStr"/>
+      <c r="Q316" s="4" t="inlineStr"/>
+      <c r="R316" s="4" t="inlineStr"/>
+      <c r="S316" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S304"/>
+  <autoFilter ref="A1:S316"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -28400,7 +29740,7 @@
         </is>
       </c>
       <c r="B2" s="7">
-        <f>COUNTA(Catálogo!A2:A46)</f>
+        <f>COUNTA(Catálogo!A2:A50)</f>
         <v/>
       </c>
     </row>
@@ -28411,7 +29751,7 @@
         </is>
       </c>
       <c r="B3" s="7">
-        <f>COUNTIF(Catálogo!W2:W46,"pendiente")</f>
+        <f>COUNTIF(Catálogo!W2:W50,"pendiente")</f>
         <v/>
       </c>
     </row>
@@ -28422,7 +29762,7 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>COUNTIF(Catálogo!W2:W46,"compuesta")</f>
+        <f>COUNTIF(Catálogo!W2:W50,"compuesta")</f>
         <v/>
       </c>
     </row>
@@ -28433,7 +29773,7 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF(Catálogo!W2:W46,"montada")</f>
+        <f>COUNTIF(Catálogo!W2:W50,"montada")</f>
         <v/>
       </c>
     </row>
@@ -28444,7 +29784,7 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF(Catálogo!W2:W46,"publicada")</f>
+        <f>COUNTIF(Catálogo!W2:W50,"publicada")</f>
         <v/>
       </c>
     </row>
@@ -28484,15 +29824,15 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Catálogo!D2:D46,A10)</f>
+        <f>COUNTIF(Catálogo!D2:D50,A10)</f>
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>COUNTIFS(Catálogo!D2:D46,A10,Catálogo!W2:W46,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D50,A10,Catálogo!W2:W50,"publicada")</f>
         <v/>
       </c>
       <c r="D10" s="7">
-        <f>SUMIF(Catálogo!D2:D46,A10,Catálogo!R2:R46)</f>
+        <f>SUMIF(Catálogo!D2:D50,A10,Catálogo!R2:R50)</f>
         <v/>
       </c>
     </row>
@@ -28503,15 +29843,15 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Catálogo!D2:D46,A11)</f>
+        <f>COUNTIF(Catálogo!D2:D50,A11)</f>
         <v/>
       </c>
       <c r="C11" s="7">
-        <f>COUNTIFS(Catálogo!D2:D46,A11,Catálogo!W2:W46,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D50,A11,Catálogo!W2:W50,"publicada")</f>
         <v/>
       </c>
       <c r="D11" s="7">
-        <f>SUMIF(Catálogo!D2:D46,A11,Catálogo!R2:R46)</f>
+        <f>SUMIF(Catálogo!D2:D50,A11,Catálogo!R2:R50)</f>
         <v/>
       </c>
     </row>
@@ -28522,15 +29862,15 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Catálogo!D2:D46,A12)</f>
+        <f>COUNTIF(Catálogo!D2:D50,A12)</f>
         <v/>
       </c>
       <c r="C12" s="7">
-        <f>COUNTIFS(Catálogo!D2:D46,A12,Catálogo!W2:W46,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D50,A12,Catálogo!W2:W50,"publicada")</f>
         <v/>
       </c>
       <c r="D12" s="7">
-        <f>SUMIF(Catálogo!D2:D46,A12,Catálogo!R2:R46)</f>
+        <f>SUMIF(Catálogo!D2:D50,A12,Catálogo!R2:R50)</f>
         <v/>
       </c>
     </row>
@@ -28541,15 +29881,15 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Catálogo!D2:D46,A13)</f>
+        <f>COUNTIF(Catálogo!D2:D50,A13)</f>
         <v/>
       </c>
       <c r="C13" s="7">
-        <f>COUNTIFS(Catálogo!D2:D46,A13,Catálogo!W2:W46,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D50,A13,Catálogo!W2:W50,"publicada")</f>
         <v/>
       </c>
       <c r="D13" s="7">
-        <f>SUMIF(Catálogo!D2:D46,A13,Catálogo!R2:R46)</f>
+        <f>SUMIF(Catálogo!D2:D50,A13,Catálogo!R2:R50)</f>
         <v/>
       </c>
     </row>
@@ -28560,15 +29900,15 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Catálogo!D2:D46,A14)</f>
+        <f>COUNTIF(Catálogo!D2:D50,A14)</f>
         <v/>
       </c>
       <c r="C14" s="7">
-        <f>COUNTIFS(Catálogo!D2:D46,A14,Catálogo!W2:W46,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D50,A14,Catálogo!W2:W50,"publicada")</f>
         <v/>
       </c>
       <c r="D14" s="7">
-        <f>SUMIF(Catálogo!D2:D46,A14,Catálogo!R2:R46)</f>
+        <f>SUMIF(Catálogo!D2:D50,A14,Catálogo!R2:R50)</f>
         <v/>
       </c>
     </row>
@@ -28605,7 +29945,7 @@
         </is>
       </c>
       <c r="B18" s="7">
-        <f>SUM(Catálogo!Y2:Y46)</f>
+        <f>SUM(Catálogo!Y2:Y50)</f>
         <v/>
       </c>
     </row>
@@ -28616,7 +29956,7 @@
         </is>
       </c>
       <c r="B19" s="7">
-        <f>SUM(Catálogo!Z2:Z46)</f>
+        <f>SUM(Catálogo!Z2:Z50)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Ruidos de color: ruido marrón con campanas lejanas y ruido rosa con ondas delta
Nuevos fondos (marron, rosa) en ambiente.py y capa delta en capas.py (de 3 a
1,5 Hz). Obras 50 y 51 de 3 h con pantalla negra, sus paletas y miniaturas, y
los TikToks: ruido marrón, ruido rosa + delta y el 3 AM Reset entero en 10 min.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$AA$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$316</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$AA$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shorts'!$A$1:$S$322</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA50"/>
+  <dimension ref="A1:AA52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6017,7 +6017,11 @@
         </is>
       </c>
       <c r="K45" s="4" t="inlineStr"/>
-      <c r="L45" s="4" t="inlineStr"/>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>https://youtu.be/BeFuK1CnmII</t>
+        </is>
+      </c>
       <c r="M45" s="2" t="n">
         <v>432</v>
       </c>
@@ -6060,10 +6064,14 @@
       </c>
       <c r="W45" s="4" t="inlineStr">
         <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="X45" s="4" t="inlineStr"/>
+          <t>publicada</t>
+        </is>
+      </c>
+      <c r="X45" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
       <c r="Y45" s="4" t="inlineStr"/>
       <c r="Z45" s="4" t="inlineStr"/>
       <c r="AA45" s="5">
@@ -6666,8 +6674,246 @@
         <v/>
       </c>
     </row>
+    <row r="51" ht="58" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-050</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Brown Noise for Deep Sleep 🌙 Distant Temple Bells · Black Screen · Fall Asleep Fast · 3 Hours</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Música para dormir · Ruido marrón y campanas lejanas · 432 Hz · Ruido marrón · 3 horas</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Dormir</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>marron</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Brown noise and pink noise are the most searched sounds for sleep. This is brown noise: low, warm and steady, with distant temple bells.
+Like heavy rain on a faraway roof. No beat, no melody to follow, nothing to listen for. The screen fades to black after 3 minutes.
+🌙 Lights off, phone face down, volume low. Let it cover the noise.
+🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+Original composition by Rin, synthesized from scratch in just intonation around 216 Hz, the low octave of 432 Hz, kumoi mode. No samples.
+#brownnoise #sleepsounds #darkscreen</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Ruido marrón · 3 horas
+Para acompañar el sueño.
+Ambiente: ruido marrón y campanas lejanas.
+Compuesta con raíz en 216 Hz, la octava grave de 432 Hz, en entonación justa, modo kumoi.
+Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
+Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#sleepmusic #meditation #432hz</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>3 HOURS</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>#brownnoise #sleepsounds #darkscreen</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>brown noise, brown noise for sleeping, brown noise sleep, brown noise black screen, brown noise 3 hours, deep sleep, sleep sounds, black screen sleep, dark screen sleep music, fall asleep fast, temple bells, noise for sleeping, rin, ruido marrón para dormir</t>
+        </is>
+      </c>
+      <c r="K51" s="4" t="inlineStr"/>
+      <c r="L51" s="4" t="inlineStr"/>
+      <c r="M51" s="2" t="n">
+        <v>432</v>
+      </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>kumoi</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>grave</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="n">
+        <v>36529</v>
+      </c>
+      <c r="Q51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R51" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="S51" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="T51" s="2" t="inlineStr">
+        <is>
+          <t>Brown noise or rain: which one puts you to sleep faster? 🌙 Tell us.</t>
+        </is>
+      </c>
+      <c r="U51" s="3" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/compositor.py --minutos 180 --raiz 432 --modo kumoi --semilla 36529 --caracter sin-cuenco --registro grave</t>
+        </is>
+      </c>
+      <c r="V51" s="2" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/capas.py zen 10840 audio/OBRA-050_capa.wav --semilla 36529 --raiz 432 --densidad 0.6 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-050_432_kumoi.wav audio/OBRA-050_final.wav --fondo marron --nivel-obra -24 --nivel-capa -9 --entrada-obra 4 --capa audio/OBRA-050_capa.wav</t>
+        </is>
+      </c>
+      <c r="W51" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="X51" s="4" t="inlineStr"/>
+      <c r="Y51" s="4" t="inlineStr"/>
+      <c r="Z51" s="4" t="inlineStr"/>
+      <c r="AA51" s="5">
+        <f>IFERROR(Z51/Y51*1000,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="58" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-051</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Pink Noise + Delta Waves for Deep Sleep 🌙 Binaural Beats · Black Screen · 3 Hours</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Música para dormir · Ruido rosa y ondas delta · 432 Hz · Ruido rosa y delta · 3 horas</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Dormir</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>delta</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Pink noise and brown noise are the most searched sounds for sleep, and pink noise with delta waves is the pairing sleep apps use in their sleep category. 🎧 Use headphones for the best experience.
+Pink noise is soft and even, like steady rain. Underneath, each ear hears a slightly different tone: the difference starts at 3 Hz and slows to 1.5 Hz, the rhythm of deep sleep. The screen fades to black after 3 minutes.
+🌙 Headphones on, lights off, volume low.
+🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+Original composition by Rin, synthesized from scratch in just intonation around 216 Hz, the low octave of 432 Hz, shin mode. No samples. Delta waves are the brain's slowest rhythm, the one of deep sleep. Not medical advice.
+#pinknoise #deltawaves #deepsleep</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Ruido rosa y delta · 3 horas
+Para acompañar el sueño.
+Ambiente: ruido rosa y ondas delta.
+Compuesta con raíz en 216 Hz, la octava grave de 432 Hz, en entonación justa, modo shin.
+Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
+Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
+Mejor a volumen bajo.
+Suscríbete para las próximas obras: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
+#sleepmusic #meditation #432hz</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>3 HOURS</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>#pinknoise #deltawaves #deepsleep</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>pink noise, pink noise for sleeping, delta waves, delta waves sleep, pink noise delta waves, binaural beats, binaural beats for sleep, deep sleep, black screen sleep, sleep sounds, fall asleep fast, 3 hours, rin, ruido rosa para dormir</t>
+        </is>
+      </c>
+      <c r="K52" s="4" t="inlineStr"/>
+      <c r="L52" s="4" t="inlineStr"/>
+      <c r="M52" s="2" t="n">
+        <v>432</v>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>shin</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>grave</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="n">
+        <v>127804</v>
+      </c>
+      <c r="Q52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R52" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="S52" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="T52" s="2" t="inlineStr">
+        <is>
+          <t>Headphones or speaker? 🎧 Tell us how far you got before falling asleep.</t>
+        </is>
+      </c>
+      <c r="U52" s="3" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/compositor.py --minutos 180 --raiz 432 --modo shin --semilla 127804 --caracter sin-cuenco --registro grave</t>
+        </is>
+      </c>
+      <c r="V52" s="2" t="inlineStr">
+        <is>
+          <t>python3 03-composicion/capas.py delta 10840 audio/OBRA-051_capa.wav --semilla 127804 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-051_432_shin.wav audio/OBRA-051_final.wav --fondo rosa --nivel-fondo -1 --nivel-obra -22 --nivel-capa -13 --entrada-obra 4 --capa audio/OBRA-051_capa.wav</t>
+        </is>
+      </c>
+      <c r="W52" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="X52" s="4" t="inlineStr"/>
+      <c r="Y52" s="4" t="inlineStr"/>
+      <c r="Z52" s="4" t="inlineStr"/>
+      <c r="AA52" s="5">
+        <f>IFERROR(Z52/Y52*1000,"")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA50"/>
+  <autoFilter ref="A1:AA52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6678,7 +6924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S316"/>
+  <dimension ref="A1:S322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -28450,6 +28696,7 @@
         <is>
           <t>🎧 Use headphones for the best experience. Save this for tonight.
 Full piece (3 h): Deep Sleep Theta Waves 🌙 Turn Off Your Thoughts · Dark Screen · Fall Asleep Fast · 3 Hours
+https://youtu.be/BeFuK1CnmII
 #sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
@@ -28458,7 +28705,11 @@
           <t>sleep music, deep sleep, 432 hz, theta waves, Rin</t>
         </is>
       </c>
-      <c r="L299" s="2" t="inlineStr"/>
+      <c r="L299" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/BeFuK1CnmII</t>
+        </is>
+      </c>
       <c r="M299" s="2" t="inlineStr">
         <is>
           <t>432 Hz · sleep</t>
@@ -28522,6 +28773,7 @@
         <is>
           <t>🎧 Use headphones for the best experience. Lights off, volume low.
 Full piece (3 h): Deep Sleep Theta Waves 🌙 Turn Off Your Thoughts · Dark Screen · Fall Asleep Fast · 3 Hours
+https://youtu.be/BeFuK1CnmII
 #sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
@@ -28530,7 +28782,11 @@
           <t>sleep music, deep sleep, 432 hz, theta waves, Rin</t>
         </is>
       </c>
-      <c r="L300" s="2" t="inlineStr"/>
+      <c r="L300" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/BeFuK1CnmII</t>
+        </is>
+      </c>
       <c r="M300" s="2" t="inlineStr">
         <is>
           <t>432 Hz · night</t>
@@ -28594,6 +28850,7 @@
         <is>
           <t>🎧 Use headphones for the best experience. Stay until your breathing slows.
 Full piece (3 h): Deep Sleep Theta Waves 🌙 Turn Off Your Thoughts · Dark Screen · Fall Asleep Fast · 3 Hours
+https://youtu.be/BeFuK1CnmII
 #sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
@@ -28602,7 +28859,11 @@
           <t>sleep music, deep sleep, 432 hz, theta waves, Rin</t>
         </is>
       </c>
-      <c r="L301" s="2" t="inlineStr"/>
+      <c r="L301" s="2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/BeFuK1CnmII</t>
+        </is>
+      </c>
       <c r="M301" s="2" t="inlineStr">
         <is>
           <t>432 Hz · rest</t>
@@ -29704,8 +29965,440 @@
       <c r="R316" s="4" t="inlineStr"/>
       <c r="S316" s="4" t="inlineStr"/>
     </row>
+    <row r="317" ht="58" customHeight="1">
+      <c r="A317" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-050-S1</t>
+        </is>
+      </c>
+      <c r="B317" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-050</t>
+        </is>
+      </c>
+      <c r="C317" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D317" s="2" t="inlineStr">
+        <is>
+          <t>short-1.mp4</t>
+        </is>
+      </c>
+      <c r="E317" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="F317" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G317" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H317" s="2" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in</t>
+        </is>
+      </c>
+      <c r="I317" s="3" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in · 432 Hz · Brown Noise</t>
+        </is>
+      </c>
+      <c r="J317" s="3" t="inlineStr">
+        <is>
+          <t>Save this for tonight.
+Full piece (3 h): Brown Noise for Deep Sleep 🌙 Distant Temple Bells · Black Screen · Fall Asleep Fast · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K317" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, brown noise, Rin</t>
+        </is>
+      </c>
+      <c r="L317" s="2" t="inlineStr"/>
+      <c r="M317" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · sleep</t>
+        </is>
+      </c>
+      <c r="N317" s="3" t="inlineStr">
+        <is>
+          <t>Save this for tonight. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O317" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P317" s="4" t="inlineStr"/>
+      <c r="Q317" s="4" t="inlineStr"/>
+      <c r="R317" s="4" t="inlineStr"/>
+      <c r="S317" s="4" t="inlineStr"/>
+    </row>
+    <row r="318" ht="58" customHeight="1">
+      <c r="A318" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-050-S2</t>
+        </is>
+      </c>
+      <c r="B318" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-050</t>
+        </is>
+      </c>
+      <c r="C318" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D318" s="2" t="inlineStr">
+        <is>
+          <t>short-2.mp4</t>
+        </is>
+      </c>
+      <c r="E318" s="2" t="n">
+        <v>5432</v>
+      </c>
+      <c r="F318" s="2" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G318" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H318" s="2" t="inlineStr">
+        <is>
+          <t>Unclench your jaw. Let the pillow hold you</t>
+        </is>
+      </c>
+      <c r="I318" s="3" t="inlineStr">
+        <is>
+          <t>Unclench your jaw. Let the pillow hold you · 432 Hz · Brown Noise</t>
+        </is>
+      </c>
+      <c r="J318" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, volume low.
+Full piece (3 h): Brown Noise for Deep Sleep 🌙 Distant Temple Bells · Black Screen · Fall Asleep Fast · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K318" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, brown noise, Rin</t>
+        </is>
+      </c>
+      <c r="L318" s="2" t="inlineStr"/>
+      <c r="M318" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · night</t>
+        </is>
+      </c>
+      <c r="N318" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, volume low. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O318" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P318" s="4" t="inlineStr"/>
+      <c r="Q318" s="4" t="inlineStr"/>
+      <c r="R318" s="4" t="inlineStr"/>
+      <c r="S318" s="4" t="inlineStr"/>
+    </row>
+    <row r="319" ht="58" customHeight="1">
+      <c r="A319" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-050-S3</t>
+        </is>
+      </c>
+      <c r="B319" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-050</t>
+        </is>
+      </c>
+      <c r="C319" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D319" s="2" t="inlineStr">
+        <is>
+          <t>short-3.mp4</t>
+        </is>
+      </c>
+      <c r="E319" s="2" t="n">
+        <v>10775</v>
+      </c>
+      <c r="F319" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G319" s="2" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H319" s="2" t="inlineStr">
+        <is>
+          <t>Close your eyes. Just listen</t>
+        </is>
+      </c>
+      <c r="I319" s="3" t="inlineStr">
+        <is>
+          <t>Close your eyes. Just listen · 432 Hz · Brown Noise</t>
+        </is>
+      </c>
+      <c r="J319" s="3" t="inlineStr">
+        <is>
+          <t>Stay until your breathing slows.
+Full piece (3 h): Brown Noise for Deep Sleep 🌙 Distant Temple Bells · Black Screen · Fall Asleep Fast · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K319" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, brown noise, Rin</t>
+        </is>
+      </c>
+      <c r="L319" s="2" t="inlineStr"/>
+      <c r="M319" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · rest</t>
+        </is>
+      </c>
+      <c r="N319" s="3" t="inlineStr">
+        <is>
+          <t>Stay until your breathing slows. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O319" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P319" s="4" t="inlineStr"/>
+      <c r="Q319" s="4" t="inlineStr"/>
+      <c r="R319" s="4" t="inlineStr"/>
+      <c r="S319" s="4" t="inlineStr"/>
+    </row>
+    <row r="320" ht="58" customHeight="1">
+      <c r="A320" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-051-S1</t>
+        </is>
+      </c>
+      <c r="B320" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-051</t>
+        </is>
+      </c>
+      <c r="C320" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D320" s="2" t="inlineStr">
+        <is>
+          <t>short-1.mp4</t>
+        </is>
+      </c>
+      <c r="E320" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="F320" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G320" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H320" s="2" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in</t>
+        </is>
+      </c>
+      <c r="I320" s="3" t="inlineStr">
+        <is>
+          <t>Breathe out longer than you breathe in · 432 Hz · Pink Noise and Delta Waves</t>
+        </is>
+      </c>
+      <c r="J320" s="3" t="inlineStr">
+        <is>
+          <t>Save this for tonight.
+Full piece (3 h): Pink Noise + Delta Waves for Deep Sleep 🌙 Binaural Beats · Black Screen · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K320" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, pink noise and delta waves, Rin</t>
+        </is>
+      </c>
+      <c r="L320" s="2" t="inlineStr"/>
+      <c r="M320" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · sleep</t>
+        </is>
+      </c>
+      <c r="N320" s="3" t="inlineStr">
+        <is>
+          <t>Save this for tonight. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O320" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P320" s="4" t="inlineStr"/>
+      <c r="Q320" s="4" t="inlineStr"/>
+      <c r="R320" s="4" t="inlineStr"/>
+      <c r="S320" s="4" t="inlineStr"/>
+    </row>
+    <row r="321" ht="58" customHeight="1">
+      <c r="A321" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-051-S2</t>
+        </is>
+      </c>
+      <c r="B321" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-051</t>
+        </is>
+      </c>
+      <c r="C321" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D321" s="2" t="inlineStr">
+        <is>
+          <t>short-2.mp4</t>
+        </is>
+      </c>
+      <c r="E321" s="2" t="n">
+        <v>5432</v>
+      </c>
+      <c r="F321" s="2" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G321" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H321" s="2" t="inlineStr">
+        <is>
+          <t>Unclench your jaw. Let the pillow hold you</t>
+        </is>
+      </c>
+      <c r="I321" s="3" t="inlineStr">
+        <is>
+          <t>Unclench your jaw. Let the pillow hold you · 432 Hz · Pink Noise and Delta Waves</t>
+        </is>
+      </c>
+      <c r="J321" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, volume low.
+Full piece (3 h): Pink Noise + Delta Waves for Deep Sleep 🌙 Binaural Beats · Black Screen · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K321" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, pink noise and delta waves, Rin</t>
+        </is>
+      </c>
+      <c r="L321" s="2" t="inlineStr"/>
+      <c r="M321" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · night</t>
+        </is>
+      </c>
+      <c r="N321" s="3" t="inlineStr">
+        <is>
+          <t>Lights off, volume low. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O321" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P321" s="4" t="inlineStr"/>
+      <c r="Q321" s="4" t="inlineStr"/>
+      <c r="R321" s="4" t="inlineStr"/>
+      <c r="S321" s="4" t="inlineStr"/>
+    </row>
+    <row r="322" ht="58" customHeight="1">
+      <c r="A322" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-051-S3</t>
+        </is>
+      </c>
+      <c r="B322" s="2" t="inlineStr">
+        <is>
+          <t>OBRA-051</t>
+        </is>
+      </c>
+      <c r="C322" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D322" s="2" t="inlineStr">
+        <is>
+          <t>short-3.mp4</t>
+        </is>
+      </c>
+      <c r="E322" s="2" t="n">
+        <v>10775</v>
+      </c>
+      <c r="F322" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G322" s="2" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H322" s="2" t="inlineStr">
+        <is>
+          <t>Close your eyes. Just listen</t>
+        </is>
+      </c>
+      <c r="I322" s="3" t="inlineStr">
+        <is>
+          <t>Close your eyes. Just listen · 432 Hz · Pink Noise and Delta Waves</t>
+        </is>
+      </c>
+      <c r="J322" s="3" t="inlineStr">
+        <is>
+          <t>Stay until your breathing slows.
+Full piece (3 h): Pink Noise + Delta Waves for Deep Sleep 🌙 Binaural Beats · Black Screen · 3 Hours
+#sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
+        </is>
+      </c>
+      <c r="K322" s="2" t="inlineStr">
+        <is>
+          <t>sleep music, deep sleep, 432 hz, pink noise and delta waves, Rin</t>
+        </is>
+      </c>
+      <c r="L322" s="2" t="inlineStr"/>
+      <c r="M322" s="2" t="inlineStr">
+        <is>
+          <t>432 Hz · rest</t>
+        </is>
+      </c>
+      <c r="N322" s="3" t="inlineStr">
+        <is>
+          <t>Stay until your breathing slows. Full 3 h piece on YouTube: Rin.
+#sleepmusic #sleep #relaxingmusic #432hz #meditation</t>
+        </is>
+      </c>
+      <c r="O322" s="4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="P322" s="4" t="inlineStr"/>
+      <c r="Q322" s="4" t="inlineStr"/>
+      <c r="R322" s="4" t="inlineStr"/>
+      <c r="S322" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S316"/>
+  <autoFilter ref="A1:S322"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -29740,7 +30433,7 @@
         </is>
       </c>
       <c r="B2" s="7">
-        <f>COUNTA(Catálogo!A2:A50)</f>
+        <f>COUNTA(Catálogo!A2:A52)</f>
         <v/>
       </c>
     </row>
@@ -29751,7 +30444,7 @@
         </is>
       </c>
       <c r="B3" s="7">
-        <f>COUNTIF(Catálogo!W2:W50,"pendiente")</f>
+        <f>COUNTIF(Catálogo!W2:W52,"pendiente")</f>
         <v/>
       </c>
     </row>
@@ -29762,7 +30455,7 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>COUNTIF(Catálogo!W2:W50,"compuesta")</f>
+        <f>COUNTIF(Catálogo!W2:W52,"compuesta")</f>
         <v/>
       </c>
     </row>
@@ -29773,7 +30466,7 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF(Catálogo!W2:W50,"montada")</f>
+        <f>COUNTIF(Catálogo!W2:W52,"montada")</f>
         <v/>
       </c>
     </row>
@@ -29784,7 +30477,7 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF(Catálogo!W2:W50,"publicada")</f>
+        <f>COUNTIF(Catálogo!W2:W52,"publicada")</f>
         <v/>
       </c>
     </row>
@@ -29824,15 +30517,15 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Catálogo!D2:D50,A10)</f>
+        <f>COUNTIF(Catálogo!D2:D52,A10)</f>
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>COUNTIFS(Catálogo!D2:D50,A10,Catálogo!W2:W50,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D52,A10,Catálogo!W2:W52,"publicada")</f>
         <v/>
       </c>
       <c r="D10" s="7">
-        <f>SUMIF(Catálogo!D2:D50,A10,Catálogo!R2:R50)</f>
+        <f>SUMIF(Catálogo!D2:D52,A10,Catálogo!R2:R52)</f>
         <v/>
       </c>
     </row>
@@ -29843,15 +30536,15 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Catálogo!D2:D50,A11)</f>
+        <f>COUNTIF(Catálogo!D2:D52,A11)</f>
         <v/>
       </c>
       <c r="C11" s="7">
-        <f>COUNTIFS(Catálogo!D2:D50,A11,Catálogo!W2:W50,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D52,A11,Catálogo!W2:W52,"publicada")</f>
         <v/>
       </c>
       <c r="D11" s="7">
-        <f>SUMIF(Catálogo!D2:D50,A11,Catálogo!R2:R50)</f>
+        <f>SUMIF(Catálogo!D2:D52,A11,Catálogo!R2:R52)</f>
         <v/>
       </c>
     </row>
@@ -29862,15 +30555,15 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Catálogo!D2:D50,A12)</f>
+        <f>COUNTIF(Catálogo!D2:D52,A12)</f>
         <v/>
       </c>
       <c r="C12" s="7">
-        <f>COUNTIFS(Catálogo!D2:D50,A12,Catálogo!W2:W50,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D52,A12,Catálogo!W2:W52,"publicada")</f>
         <v/>
       </c>
       <c r="D12" s="7">
-        <f>SUMIF(Catálogo!D2:D50,A12,Catálogo!R2:R50)</f>
+        <f>SUMIF(Catálogo!D2:D52,A12,Catálogo!R2:R52)</f>
         <v/>
       </c>
     </row>
@@ -29881,15 +30574,15 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Catálogo!D2:D50,A13)</f>
+        <f>COUNTIF(Catálogo!D2:D52,A13)</f>
         <v/>
       </c>
       <c r="C13" s="7">
-        <f>COUNTIFS(Catálogo!D2:D50,A13,Catálogo!W2:W50,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D52,A13,Catálogo!W2:W52,"publicada")</f>
         <v/>
       </c>
       <c r="D13" s="7">
-        <f>SUMIF(Catálogo!D2:D50,A13,Catálogo!R2:R50)</f>
+        <f>SUMIF(Catálogo!D2:D52,A13,Catálogo!R2:R52)</f>
         <v/>
       </c>
     </row>
@@ -29900,15 +30593,15 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Catálogo!D2:D50,A14)</f>
+        <f>COUNTIF(Catálogo!D2:D52,A14)</f>
         <v/>
       </c>
       <c r="C14" s="7">
-        <f>COUNTIFS(Catálogo!D2:D50,A14,Catálogo!W2:W50,"publicada")</f>
+        <f>COUNTIFS(Catálogo!D2:D52,A14,Catálogo!W2:W52,"publicada")</f>
         <v/>
       </c>
       <c r="D14" s="7">
-        <f>SUMIF(Catálogo!D2:D50,A14,Catálogo!R2:R50)</f>
+        <f>SUMIF(Catálogo!D2:D52,A14,Catálogo!R2:R52)</f>
         <v/>
       </c>
     </row>
@@ -29945,7 +30638,7 @@
         </is>
       </c>
       <c r="B18" s="7">
-        <f>SUM(Catálogo!Y2:Y50)</f>
+        <f>SUM(Catálogo!Y2:Y52)</f>
         <v/>
       </c>
     </row>
@@ -29956,7 +30649,7 @@
         </is>
       </c>
       <c r="B19" s="7">
-        <f>SUM(Catálogo!Z2:Z50)</f>
+        <f>SUM(Catálogo!Z2:Z52)</f>
         <v/>
       </c>
     </row>
@@ -30099,7 +30792,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Ambiente aprobado en escucha: mar, mar-aves, zen, selva, lluvia-tambor, jardin, lluvia, theta o guqin.</t>
+          <t>Ambiente aprobado en escucha: mar, mar-aves, zen, selva, lluvia-tambor, jardin, lluvia, theta, guqin, marron o delta.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ruidos de color: sin mencionar apps; el título y la descripción dicen qué suena
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -6702,7 +6702,7 @@
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>Brown noise and pink noise are the most searched sounds for sleep. This is brown noise: low, warm and steady, with distant temple bells.
+          <t>Brown noise for deep sleep: low, warm and steady, with distant temple bells.
 Like heavy rain on a faraway roof. No beat, no melody to follow, nothing to listen for. The screen fades to black after 3 minutes.
 🌙 Lights off, phone face down, volume low. Let it cover the noise.
 🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
@@ -6821,7 +6821,7 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Pink noise and brown noise are the most searched sounds for sleep, and pink noise with delta waves is the pairing sleep apps use in their sleep category. 🎧 Use headphones for the best experience.
+          <t>Pink noise with delta waves for deep sleep. 🎧 Use headphones for the best experience.
 Pink noise is soft and even, like steady rain. Underneath, each ear hears a slightly different tone: the difference starts at 3 Hz and slows to 1.5 Hz, the rhythm of deep sleep. The screen fades to black after 3 minutes.
 🌙 Headphones on, lights off, volume low.
 🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1

</xml_diff>

<commit_message>
Nada de bocina ni retumbe en el código
- ambiente.py: la obra pasa por un corte de graves en 150 Hz (--corte-obra; el
  guqin usa 70). El fondo de fogata pierde el zumbido tipo didgeridoo.
- tao.py y tao_largo.py: el bordón sin la quinta grave ni el 108 Hz al frente,
  más bajo y con una respiración que casi no se nota.
- El drone del compositor ya no tiene timbre de clarinete (commit anterior).

Escucha del 05/10: la muestra C (diapasones con el fondo nuevo y este corte)
fue la única sin «bocina».

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -6182,7 +6182,7 @@
       </c>
       <c r="V46" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/ambiente.py audio/OBRA-045_432_yu.wav audio/OBRA-045_final.wav --fondo lluvia --nivel-obra 0 --nivel-fondo -6 --entrada-obra 6</t>
+          <t>python3 03-composicion/ambiente.py audio/OBRA-045_432_yu.wav audio/OBRA-045_final.wav --fondo lluvia --nivel-obra 0 --nivel-fondo -6 --entrada-obra 6 --corte-obra 70</t>
         </is>
       </c>
       <c r="W46" s="4" t="inlineStr">
@@ -6301,7 +6301,7 @@
       </c>
       <c r="V47" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/ambiente.py audio/OBRA-046_432_yu.wav audio/OBRA-046_final.wav --fondo lluvia --nivel-obra 0 --nivel-fondo -6 --entrada-obra 6</t>
+          <t>python3 03-composicion/ambiente.py audio/OBRA-046_432_yu.wav audio/OBRA-046_final.wav --fondo lluvia --nivel-obra 0 --nivel-fondo -6 --entrada-obra 6 --corte-obra 70</t>
         </is>
       </c>
       <c r="W47" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Videos 45 a 49 sin estática: guqin sin lluvia, mar más bajo en zen y jardín
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -1870,7 +1870,7 @@
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 1840 audio/OBRA-010_capa.wav --semilla 739461 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-010_432_hirajoshi.wav audio/OBRA-010_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-010_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 1840 audio/OBRA-010_capa.wav --semilla 739461 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-010_432_hirajoshi.wav audio/OBRA-010_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-010_capa.wav</t>
         </is>
       </c>
       <c r="W11" s="4" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="V13" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 640 audio/OBRA-012_capa.wav --semilla 43734 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-012_528_shin.wav audio/OBRA-012_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-012_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 640 audio/OBRA-012_capa.wav --semilla 43734 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-012_528_shin.wav audio/OBRA-012_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-012_capa.wav</t>
         </is>
       </c>
       <c r="W13" s="4" t="inlineStr">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="V15" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-014_capa.wav --semilla 310137 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-014_528_yo.wav audio/OBRA-014_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-014_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-014_capa.wav --semilla 310137 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-014_528_yo.wav audio/OBRA-014_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-014_capa.wav</t>
         </is>
       </c>
       <c r="W15" s="4" t="inlineStr">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="V18" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-017_capa.wav --semilla 714152 --raiz 417 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-017_417_hirajoshi.wav audio/OBRA-017_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-017_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-017_capa.wav --semilla 714152 --raiz 417 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-017_417_hirajoshi.wav audio/OBRA-017_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-017_capa.wav</t>
         </is>
       </c>
       <c r="W18" s="4" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="V19" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-018_capa.wav --semilla 735455 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-018_528_hirajoshi.wav audio/OBRA-018_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-018_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-018_capa.wav --semilla 735455 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-018_528_hirajoshi.wav audio/OBRA-018_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-018_capa.wav</t>
         </is>
       </c>
       <c r="W19" s="4" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="V20" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-019_capa.wav --semilla 627577 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-019_432_shin.wav audio/OBRA-019_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-019_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-019_capa.wav --semilla 627577 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-019_432_shin.wav audio/OBRA-019_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-019_capa.wav</t>
         </is>
       </c>
       <c r="W20" s="4" t="inlineStr">
@@ -3236,7 +3236,7 @@
       </c>
       <c r="V22" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-021_capa.wav --semilla 864630 --raiz 396 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-021_396_kumoi.wav audio/OBRA-021_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-021_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-021_capa.wav --semilla 864630 --raiz 396 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-021_396_kumoi.wav audio/OBRA-021_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-021_capa.wav</t>
         </is>
       </c>
       <c r="W22" s="4" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="V23" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-022_capa.wav --semilla 335798 --raiz 639 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-022_639_yo.wav audio/OBRA-022_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-022_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-022_capa.wav --semilla 335798 --raiz 639 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-022_639_yo.wav audio/OBRA-022_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-022_capa.wav</t>
         </is>
       </c>
       <c r="W23" s="4" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="V24" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-023_capa.wav --semilla 299306 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-023_528_shin.wav audio/OBRA-023_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-023_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-023_capa.wav --semilla 299306 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-023_528_shin.wav audio/OBRA-023_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-023_capa.wav</t>
         </is>
       </c>
       <c r="W24" s="4" t="inlineStr">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="V29" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-028_capa.wav --semilla 409966 --raiz 417 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-028_417_hirajoshi.wav audio/OBRA-028_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-028_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-028_capa.wav --semilla 409966 --raiz 417 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-028_417_hirajoshi.wav audio/OBRA-028_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-028_capa.wav</t>
         </is>
       </c>
       <c r="W29" s="4" t="inlineStr">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="V32" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-031_capa.wav --semilla 288169 --raiz 852 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-031_852_hirajoshi.wav audio/OBRA-031_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-031_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-031_capa.wav --semilla 288169 --raiz 852 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-031_852_hirajoshi.wav audio/OBRA-031_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-031_capa.wav</t>
         </is>
       </c>
       <c r="W32" s="4" t="inlineStr">
@@ -5677,7 +5677,7 @@
       </c>
       <c r="V42" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py jardin 3640 audio/OBRA-041_capa.wav --semilla 304617 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-041_432_hirajoshi.wav audio/OBRA-041_final.wav --fondo mar --nivel-fondo -8 --nivel-capa 0 --capa audio/OBRA-041_capa.wav</t>
+          <t>python3 03-composicion/capas.py jardin 3640 audio/OBRA-041_capa.wav --semilla 304617 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-041_432_hirajoshi.wav audio/OBRA-041_final.wav --fondo mar --nivel-fondo -13 --nivel-capa 0 --capa audio/OBRA-041_capa.wav</t>
         </is>
       </c>
       <c r="W42" s="4" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="V43" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 10840 audio/OBRA-042_capa.wav --semilla 266691 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-042_528_shin.wav audio/OBRA-042_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-042_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 10840 audio/OBRA-042_capa.wav --semilla 266691 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-042_528_shin.wav audio/OBRA-042_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-042_capa.wav</t>
         </is>
       </c>
       <c r="W43" s="4" t="inlineStr">
@@ -6087,12 +6087,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Woke Up at 3 AM? 🌙 Chinese Guqin &amp; Rain to Fall Back Asleep · Dark Screen · 3 Hours</t>
+          <t>Woke Up at 3 AM? 🌙 Chinese Guqin &amp; Xiao Flute to Fall Back Asleep · Dark Screen · 3 Hours</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Música para dormir · Guqin y lluvia · 432 Hz · Las tres de la mañana · 3 horas</t>
+          <t>Música para dormir · Guqin y flauta xiao · 432 Hz · Las tres de la mañana · 3 horas</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -6107,9 +6107,9 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Woke up at 3 AM again? Three hours of guqin, xiao flute and gentle rain to fall back asleep.
+          <t>Woke up at 3 AM again? Three hours of Chinese guqin and xiao flute to fall back asleep.
 In the Chinese body clock, 1 to 3 AM is the liver's hour: the hour of what you couldn't let go of. Don't check the time. Breathe out slowly through your lips, "shhh" (xū), six times, and let the strings take it from there. The screen fades to black after 3 minutes.
-🌙 Phone face down, volume low. The music thins out over the hours, until only the rain is left.
+🌙 Phone face down, volume low. The music thins out over the hours, until only soft harmonics are left.
 🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
 Original composition by Rin, synthesized from scratch in just intonation around 432 Hz, yu mode. No samples. The yu scale is the one Chinese five-element music keeps for the night. A 2,000-year-old tradition, not medical advice.
 #sleepmusic #guqin #chinesemusic</t>
@@ -6119,7 +6119,7 @@
         <is>
           <t>Las tres de la mañana · 3 horas
 Para acompañar el sueño.
-Ambiente: guqin y lluvia.
+Ambiente: guqin y flauta xiao.
 Compuesta con raíz en 432 Hz, en entonación justa, modo yu.
 Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
@@ -6140,7 +6140,7 @@
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>woke up at 3am, fall back asleep, music to fall back asleep, chinese sleep music, guqin, guqin music, chinese meditation music, chinese music for sleep, rain sounds for sleeping, dark screen sleep music, black screen sleep music, deep sleep music, sleep music, traditional chinese medicine, chinamaxxing, 3 hours, rin, música para dormir</t>
+          <t>woke up at 3am, fall back asleep, music to fall back asleep, chinese sleep music, guqin, guqin music, chinese meditation music, chinese music for sleep, chinese flute music, dark screen sleep music, black screen sleep music, deep sleep music, sleep music, traditional chinese medicine, chinamaxxing, 3 hours, rin, música para dormir</t>
         </is>
       </c>
       <c r="K46" s="4" t="inlineStr"/>
@@ -6182,7 +6182,7 @@
       </c>
       <c r="V46" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/ambiente.py audio/OBRA-045_432_yu.wav audio/OBRA-045_final.wav --fondo lluvia --nivel-obra 0 --nivel-fondo -6 --entrada-obra 6 --corte-obra 70</t>
+          <t>python3 03-composicion/ambiente.py audio/OBRA-045_432_yu.wav audio/OBRA-045_final.wav --fondo nada --nivel-obra 0 --entrada-obra 6 --corte-obra 70</t>
         </is>
       </c>
       <c r="W46" s="4" t="inlineStr">
@@ -6206,12 +6206,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>3 AM Reset 🌙 10 Minutes of Guqin &amp; Rain to Fall Back Asleep · Chinese Sleep Music</t>
+          <t>3 AM Reset 🌙 10 Minutes of Chinese Guqin to Fall Back Asleep · Sleep Music</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Música para dormir · Guqin y lluvia · 432 Hz · Volver a dormir · 10 minutos</t>
+          <t>Música para dormir · Guqin y flauta xiao · 432 Hz · Volver a dormir · 10 minutos</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -6226,7 +6226,7 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Woke up at 3 AM? Ten minutes of guqin, xiao flute and gentle rain to fall back asleep.
+          <t>Woke up at 3 AM? Ten minutes of Chinese guqin and xiao flute to fall back asleep.
 Don't check the time. Breathe out slowly through your lips, "shhh", six times, and let the strings take it from there.
 🌙 Phone face down, volume low. If you're still awake at the end, the full 3 hours are on the channel.
 🌿 Subscribe for a new calm piece every week: https://www.youtube.com/@rinchanneloficial?sub_confirmation=1
@@ -6238,7 +6238,7 @@
         <is>
           <t>Volver a dormir · 10 minutos
 Para acompañar el sueño.
-Ambiente: guqin y lluvia.
+Ambiente: guqin y flauta xiao.
 Compuesta con raíz en 432 Hz, en entonación justa, modo yu.
 Ciclo respiratorio: de 4.5 a 3.5 respiraciones por minuto, inhalar 40 % / exhalar 60 %.
 Composición original, sintetizada desde cero: el ambiente también. Ninguna muestra procede de terceros.
@@ -6259,7 +6259,7 @@
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>3am reset, fall back asleep, woke up at 3am, music to fall back asleep, guqin, chinese sleep music, 10 minute sleep music, rain sounds for sleeping, sleep music, chinese meditation music, rin, música para dormir</t>
+          <t>3am reset, fall back asleep, woke up at 3am, music to fall back asleep, guqin, chinese sleep music, 10 minute sleep music, chinese flute music, sleep music, chinese meditation music, rin, música para dormir</t>
         </is>
       </c>
       <c r="K47" s="4" t="inlineStr"/>
@@ -6301,7 +6301,7 @@
       </c>
       <c r="V47" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/ambiente.py audio/OBRA-046_432_yu.wav audio/OBRA-046_final.wav --fondo lluvia --nivel-obra 0 --nivel-fondo -6 --entrada-obra 6 --corte-obra 70</t>
+          <t>python3 03-composicion/ambiente.py audio/OBRA-046_432_yu.wav audio/OBRA-046_final.wav --fondo nada --nivel-obra 0 --entrada-obra 6 --corte-obra 70</t>
         </is>
       </c>
       <c r="W47" s="4" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="V48" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 340 audio/OBRA-047_capa.wav --semilla 756077 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-047_528_shin.wav audio/OBRA-047_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-047_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 340 audio/OBRA-047_capa.wav --semilla 756077 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-047_528_shin.wav audio/OBRA-047_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-047_capa.wav</t>
         </is>
       </c>
       <c r="W48" s="4" t="inlineStr">
@@ -6529,7 +6529,7 @@
       </c>
       <c r="T49" s="2" t="inlineStr">
         <is>
-          <t>Do bells help you sleep, or do you prefer rain? 🔔🌧️ Tell us, it shapes the next piece.</t>
+          <t>Do bells help you sleep? 🔔 Tell us what sound you want next, it shapes the next piece.</t>
         </is>
       </c>
       <c r="U49" s="3" t="inlineStr">
@@ -6539,7 +6539,7 @@
       </c>
       <c r="V49" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 10840 audio/OBRA-048_capa.wav --semilla 762820 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-048_432_kumoi.wav audio/OBRA-048_final.wav --fondo mar --nivel-fondo -7 --nivel-capa 2 --capa audio/OBRA-048_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 10840 audio/OBRA-048_capa.wav --semilla 762820 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-048_432_kumoi.wav audio/OBRA-048_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-048_capa.wav</t>
         </is>
       </c>
       <c r="W49" s="4" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="V50" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py jardin 640 audio/OBRA-049_capa.wav --semilla 341227 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-049_432_hirajoshi.wav audio/OBRA-049_final.wav --fondo mar --nivel-fondo -8 --nivel-capa 0 --capa audio/OBRA-049_capa.wav</t>
+          <t>python3 03-composicion/capas.py jardin 640 audio/OBRA-049_capa.wav --semilla 341227 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-049_432_hirajoshi.wav audio/OBRA-049_final.wav --fondo mar --nivel-fondo -13 --nivel-capa 0 --capa audio/OBRA-049_capa.wav</t>
         </is>
       </c>
       <c r="W50" s="4" t="inlineStr">
@@ -28920,19 +28920,19 @@
       </c>
       <c r="I302" s="3" t="inlineStr">
         <is>
-          <t>Breathe out longer than you breathe in · 432 Hz · Guqin and Rain</t>
+          <t>Breathe out longer than you breathe in · 432 Hz · Guqin and Xiao Flute</t>
         </is>
       </c>
       <c r="J302" s="3" t="inlineStr">
         <is>
           <t>Save this for tonight.
-Full piece (3 h): Woke Up at 3 AM? 🌙 Chinese Guqin &amp; Rain to Fall Back Asleep · Dark Screen · 3 Hours
+Full piece (3 h): Woke Up at 3 AM? 🌙 Chinese Guqin &amp; Xiao Flute to Fall Back Asleep · Dark Screen · 3 Hours
 #sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
       <c r="K302" s="2" t="inlineStr">
         <is>
-          <t>sleep music, deep sleep, 432 hz, guqin and rain, Rin</t>
+          <t>sleep music, deep sleep, 432 hz, guqin and xiao flute, Rin</t>
         </is>
       </c>
       <c r="L302" s="2" t="inlineStr"/>
@@ -28992,19 +28992,19 @@
       </c>
       <c r="I303" s="3" t="inlineStr">
         <is>
-          <t>Unclench your jaw. Let the pillow hold you · 432 Hz · Guqin and Rain</t>
+          <t>Unclench your jaw. Let the pillow hold you · 432 Hz · Guqin and Xiao Flute</t>
         </is>
       </c>
       <c r="J303" s="3" t="inlineStr">
         <is>
           <t>Lights off, volume low.
-Full piece (3 h): Woke Up at 3 AM? 🌙 Chinese Guqin &amp; Rain to Fall Back Asleep · Dark Screen · 3 Hours
+Full piece (3 h): Woke Up at 3 AM? 🌙 Chinese Guqin &amp; Xiao Flute to Fall Back Asleep · Dark Screen · 3 Hours
 #sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
       <c r="K303" s="2" t="inlineStr">
         <is>
-          <t>sleep music, deep sleep, 432 hz, guqin and rain, Rin</t>
+          <t>sleep music, deep sleep, 432 hz, guqin and xiao flute, Rin</t>
         </is>
       </c>
       <c r="L303" s="2" t="inlineStr"/>
@@ -29064,19 +29064,19 @@
       </c>
       <c r="I304" s="3" t="inlineStr">
         <is>
-          <t>Close your eyes. Just listen · 432 Hz · Guqin and Rain</t>
+          <t>Close your eyes. Just listen · 432 Hz · Guqin and Xiao Flute</t>
         </is>
       </c>
       <c r="J304" s="3" t="inlineStr">
         <is>
           <t>Stay until your breathing slows.
-Full piece (3 h): Woke Up at 3 AM? 🌙 Chinese Guqin &amp; Rain to Fall Back Asleep · Dark Screen · 3 Hours
+Full piece (3 h): Woke Up at 3 AM? 🌙 Chinese Guqin &amp; Xiao Flute to Fall Back Asleep · Dark Screen · 3 Hours
 #sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
       <c r="K304" s="2" t="inlineStr">
         <is>
-          <t>sleep music, deep sleep, 432 hz, guqin and rain, Rin</t>
+          <t>sleep music, deep sleep, 432 hz, guqin and xiao flute, Rin</t>
         </is>
       </c>
       <c r="L304" s="2" t="inlineStr"/>
@@ -29136,19 +29136,19 @@
       </c>
       <c r="I305" s="3" t="inlineStr">
         <is>
-          <t>Breathe out longer than you breathe in · 432 Hz · Guqin and Rain</t>
+          <t>Breathe out longer than you breathe in · 432 Hz · Guqin and Xiao Flute</t>
         </is>
       </c>
       <c r="J305" s="3" t="inlineStr">
         <is>
           <t>Save this for tonight.
-Full piece (10 min): 3 AM Reset 🌙 10 Minutes of Guqin &amp; Rain to Fall Back Asleep · Chinese Sleep Music
+Full piece (10 min): 3 AM Reset 🌙 10 Minutes of Chinese Guqin to Fall Back Asleep · Sleep Music
 #sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
       <c r="K305" s="2" t="inlineStr">
         <is>
-          <t>sleep music, deep sleep, 432 hz, guqin and rain, Rin</t>
+          <t>sleep music, deep sleep, 432 hz, guqin and xiao flute, Rin</t>
         </is>
       </c>
       <c r="L305" s="2" t="inlineStr"/>
@@ -29208,19 +29208,19 @@
       </c>
       <c r="I306" s="3" t="inlineStr">
         <is>
-          <t>Unclench your jaw. Let the pillow hold you · 432 Hz · Guqin and Rain</t>
+          <t>Unclench your jaw. Let the pillow hold you · 432 Hz · Guqin and Xiao Flute</t>
         </is>
       </c>
       <c r="J306" s="3" t="inlineStr">
         <is>
           <t>Lights off, volume low.
-Full piece (10 min): 3 AM Reset 🌙 10 Minutes of Guqin &amp; Rain to Fall Back Asleep · Chinese Sleep Music
+Full piece (10 min): 3 AM Reset 🌙 10 Minutes of Chinese Guqin to Fall Back Asleep · Sleep Music
 #sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
       <c r="K306" s="2" t="inlineStr">
         <is>
-          <t>sleep music, deep sleep, 432 hz, guqin and rain, Rin</t>
+          <t>sleep music, deep sleep, 432 hz, guqin and xiao flute, Rin</t>
         </is>
       </c>
       <c r="L306" s="2" t="inlineStr"/>
@@ -29280,19 +29280,19 @@
       </c>
       <c r="I307" s="3" t="inlineStr">
         <is>
-          <t>Close your eyes. Just listen · 432 Hz · Guqin and Rain</t>
+          <t>Close your eyes. Just listen · 432 Hz · Guqin and Xiao Flute</t>
         </is>
       </c>
       <c r="J307" s="3" t="inlineStr">
         <is>
           <t>Stay until your breathing slows.
-Full piece (10 min): 3 AM Reset 🌙 10 Minutes of Guqin &amp; Rain to Fall Back Asleep · Chinese Sleep Music
+Full piece (10 min): 3 AM Reset 🌙 10 Minutes of Chinese Guqin to Fall Back Asleep · Sleep Music
 #sleepmusic #sleep #relaxingmusic #432hz #shorts</t>
         </is>
       </c>
       <c r="K307" s="2" t="inlineStr">
         <is>
-          <t>sleep music, deep sleep, 432 hz, guqin and rain, Rin</t>
+          <t>sleep music, deep sleep, 432 hz, guqin and xiao flute, Rin</t>
         </is>
       </c>
       <c r="L307" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Guqin sin lluvia: la música entra en 1,5 s (los primeros segundos quedaban en silencio)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -6182,7 +6182,7 @@
       </c>
       <c r="V46" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/ambiente.py audio/OBRA-045_432_yu.wav audio/OBRA-045_final.wav --fondo nada --nivel-obra 0 --entrada-obra 6 --corte-obra 70</t>
+          <t>python3 03-composicion/ambiente.py audio/OBRA-045_432_yu.wav audio/OBRA-045_final.wav --fondo nada --nivel-obra 0 --entrada-obra 1.5 --corte-obra 70</t>
         </is>
       </c>
       <c r="W46" s="4" t="inlineStr">
@@ -6301,7 +6301,7 @@
       </c>
       <c r="V47" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/ambiente.py audio/OBRA-046_432_yu.wav audio/OBRA-046_final.wav --fondo nada --nivel-obra 0 --entrada-obra 6 --corte-obra 70</t>
+          <t>python3 03-composicion/ambiente.py audio/OBRA-046_432_yu.wav audio/OBRA-046_final.wav --fondo nada --nivel-obra 0 --entrada-obra 1.5 --corte-obra 70</t>
         </is>
       </c>
       <c r="W47" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Botón de SUBSCRIBE con campana en todos los videos, guqin sin silencio al final, drone más bajo
- suscribir.html: botón rojo SUBSCRIBE, campana y RIN (antes, texto crema
  que no se notaba), entre el 0:45 y el 2:30.
- montar.py: los videos de hasta 30 min sin pantalla negra también lo llevan.
- Guqin: --intro 0.3 --cola 3 (sin lluvia, la cola de 20 s quedaba muda).
- Zen y jardín: el drone a -23 dB (todavía se sentía la bocina).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -1870,7 +1870,7 @@
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 1840 audio/OBRA-010_capa.wav --semilla 739461 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-010_432_hirajoshi.wav audio/OBRA-010_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-010_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 1840 audio/OBRA-010_capa.wav --semilla 739461 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-010_432_hirajoshi.wav audio/OBRA-010_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --nivel-obra -23 --capa audio/OBRA-010_capa.wav</t>
         </is>
       </c>
       <c r="W11" s="4" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="V13" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 640 audio/OBRA-012_capa.wav --semilla 43734 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-012_528_shin.wav audio/OBRA-012_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-012_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 640 audio/OBRA-012_capa.wav --semilla 43734 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-012_528_shin.wav audio/OBRA-012_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --nivel-obra -23 --capa audio/OBRA-012_capa.wav</t>
         </is>
       </c>
       <c r="W13" s="4" t="inlineStr">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="V15" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-014_capa.wav --semilla 310137 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-014_528_yo.wav audio/OBRA-014_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-014_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-014_capa.wav --semilla 310137 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-014_528_yo.wav audio/OBRA-014_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --nivel-obra -23 --capa audio/OBRA-014_capa.wav</t>
         </is>
       </c>
       <c r="W15" s="4" t="inlineStr">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="V18" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-017_capa.wav --semilla 714152 --raiz 417 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-017_417_hirajoshi.wav audio/OBRA-017_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-017_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-017_capa.wav --semilla 714152 --raiz 417 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-017_417_hirajoshi.wav audio/OBRA-017_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --nivel-obra -23 --capa audio/OBRA-017_capa.wav</t>
         </is>
       </c>
       <c r="W18" s="4" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="V19" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-018_capa.wav --semilla 735455 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-018_528_hirajoshi.wav audio/OBRA-018_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-018_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-018_capa.wav --semilla 735455 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-018_528_hirajoshi.wav audio/OBRA-018_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --nivel-obra -23 --capa audio/OBRA-018_capa.wav</t>
         </is>
       </c>
       <c r="W19" s="4" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="V20" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-019_capa.wav --semilla 627577 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-019_432_shin.wav audio/OBRA-019_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-019_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-019_capa.wav --semilla 627577 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-019_432_shin.wav audio/OBRA-019_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --nivel-obra -23 --capa audio/OBRA-019_capa.wav</t>
         </is>
       </c>
       <c r="W20" s="4" t="inlineStr">
@@ -3236,7 +3236,7 @@
       </c>
       <c r="V22" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-021_capa.wav --semilla 864630 --raiz 396 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-021_396_kumoi.wav audio/OBRA-021_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-021_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-021_capa.wav --semilla 864630 --raiz 396 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-021_396_kumoi.wav audio/OBRA-021_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --nivel-obra -23 --capa audio/OBRA-021_capa.wav</t>
         </is>
       </c>
       <c r="W22" s="4" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="V23" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-022_capa.wav --semilla 335798 --raiz 639 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-022_639_yo.wav audio/OBRA-022_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-022_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 3640 audio/OBRA-022_capa.wav --semilla 335798 --raiz 639 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-022_639_yo.wav audio/OBRA-022_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --nivel-obra -23 --capa audio/OBRA-022_capa.wav</t>
         </is>
       </c>
       <c r="W23" s="4" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="V24" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-023_capa.wav --semilla 299306 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-023_528_shin.wav audio/OBRA-023_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-023_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 1240 audio/OBRA-023_capa.wav --semilla 299306 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-023_528_shin.wav audio/OBRA-023_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --nivel-obra -23 --capa audio/OBRA-023_capa.wav</t>
         </is>
       </c>
       <c r="W24" s="4" t="inlineStr">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="V29" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-028_capa.wav --semilla 409966 --raiz 417 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-028_417_hirajoshi.wav audio/OBRA-028_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-028_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-028_capa.wav --semilla 409966 --raiz 417 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-028_417_hirajoshi.wav audio/OBRA-028_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --nivel-obra -23 --capa audio/OBRA-028_capa.wav</t>
         </is>
       </c>
       <c r="W29" s="4" t="inlineStr">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="V32" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-031_capa.wav --semilla 288169 --raiz 852 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-031_852_hirajoshi.wav audio/OBRA-031_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-031_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 2740 audio/OBRA-031_capa.wav --semilla 288169 --raiz 852 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-031_852_hirajoshi.wav audio/OBRA-031_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --nivel-obra -23 --capa audio/OBRA-031_capa.wav</t>
         </is>
       </c>
       <c r="W32" s="4" t="inlineStr">
@@ -5677,7 +5677,7 @@
       </c>
       <c r="V42" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py jardin 3640 audio/OBRA-041_capa.wav --semilla 304617 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-041_432_hirajoshi.wav audio/OBRA-041_final.wav --fondo mar --nivel-fondo -13 --nivel-capa 0 --capa audio/OBRA-041_capa.wav</t>
+          <t>python3 03-composicion/capas.py jardin 3640 audio/OBRA-041_capa.wav --semilla 304617 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-041_432_hirajoshi.wav audio/OBRA-041_final.wav --fondo mar --nivel-fondo -13 --nivel-capa 0 --nivel-obra -23 --capa audio/OBRA-041_capa.wav</t>
         </is>
       </c>
       <c r="W42" s="4" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="V43" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 10840 audio/OBRA-042_capa.wav --semilla 266691 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-042_528_shin.wav audio/OBRA-042_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-042_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 10840 audio/OBRA-042_capa.wav --semilla 266691 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-042_528_shin.wav audio/OBRA-042_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --nivel-obra -23 --capa audio/OBRA-042_capa.wav</t>
         </is>
       </c>
       <c r="W43" s="4" t="inlineStr">
@@ -6182,7 +6182,7 @@
       </c>
       <c r="V46" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/ambiente.py audio/OBRA-045_432_yu.wav audio/OBRA-045_final.wav --fondo nada --nivel-obra 0 --entrada-obra 1.5 --corte-obra 70</t>
+          <t>python3 03-composicion/ambiente.py audio/OBRA-045_432_yu.wav audio/OBRA-045_final.wav --fondo nada --nivel-obra 0 --entrada-obra 1.5 --corte-obra 70 --intro 0.3 --cola 3</t>
         </is>
       </c>
       <c r="W46" s="4" t="inlineStr">
@@ -6301,7 +6301,7 @@
       </c>
       <c r="V47" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/ambiente.py audio/OBRA-046_432_yu.wav audio/OBRA-046_final.wav --fondo nada --nivel-obra 0 --entrada-obra 1.5 --corte-obra 70</t>
+          <t>python3 03-composicion/ambiente.py audio/OBRA-046_432_yu.wav audio/OBRA-046_final.wav --fondo nada --nivel-obra 0 --entrada-obra 1.5 --corte-obra 70 --intro 0.3 --cola 3</t>
         </is>
       </c>
       <c r="W47" s="4" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="V48" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 340 audio/OBRA-047_capa.wav --semilla 756077 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-047_528_shin.wav audio/OBRA-047_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-047_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 340 audio/OBRA-047_capa.wav --semilla 756077 --raiz 528 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-047_528_shin.wav audio/OBRA-047_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --nivel-obra -23 --capa audio/OBRA-047_capa.wav</t>
         </is>
       </c>
       <c r="W48" s="4" t="inlineStr">
@@ -6539,7 +6539,7 @@
       </c>
       <c r="V49" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py zen 10840 audio/OBRA-048_capa.wav --semilla 762820 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-048_432_kumoi.wav audio/OBRA-048_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --capa audio/OBRA-048_capa.wav</t>
+          <t>python3 03-composicion/capas.py zen 10840 audio/OBRA-048_capa.wav --semilla 762820 --raiz 432 --densidad 1.4 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-048_432_kumoi.wav audio/OBRA-048_final.wav --fondo mar --nivel-fondo -12 --nivel-capa 2 --nivel-obra -23 --capa audio/OBRA-048_capa.wav</t>
         </is>
       </c>
       <c r="W49" s="4" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="V50" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/capas.py jardin 640 audio/OBRA-049_capa.wav --semilla 341227 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-049_432_hirajoshi.wav audio/OBRA-049_final.wav --fondo mar --nivel-fondo -13 --nivel-capa 0 --capa audio/OBRA-049_capa.wav</t>
+          <t>python3 03-composicion/capas.py jardin 640 audio/OBRA-049_capa.wav --semilla 341227 --raiz 432 &amp;&amp; python3 03-composicion/ambiente.py audio/OBRA-049_432_hirajoshi.wav audio/OBRA-049_final.wav --fondo mar --nivel-fondo -13 --nivel-capa 0 --nivel-obra -23 --capa audio/OBRA-049_capa.wav</t>
         </is>
       </c>
       <c r="W50" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Guqin: el cierre a 11 s del final y la cola de 1 s, para que el video no termine mudo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRbYEsHA26rrbcL1hPQoJR
</commit_message>
<xml_diff>
--- a/08-catalogo/catalogo_canal.xlsx
+++ b/08-catalogo/catalogo_canal.xlsx
@@ -6182,7 +6182,7 @@
       </c>
       <c r="V46" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/ambiente.py audio/OBRA-045_432_yu.wav audio/OBRA-045_final.wav --fondo nada --nivel-obra 0 --entrada-obra 1.5 --corte-obra 70 --intro 0.3 --cola 3</t>
+          <t>python3 03-composicion/ambiente.py audio/OBRA-045_432_yu.wav audio/OBRA-045_final.wav --fondo nada --nivel-obra 0 --entrada-obra 1.5 --corte-obra 70 --intro 0.3 --cola 1</t>
         </is>
       </c>
       <c r="W46" s="4" t="inlineStr">
@@ -6301,7 +6301,7 @@
       </c>
       <c r="V47" s="2" t="inlineStr">
         <is>
-          <t>python3 03-composicion/ambiente.py audio/OBRA-046_432_yu.wav audio/OBRA-046_final.wav --fondo nada --nivel-obra 0 --entrada-obra 1.5 --corte-obra 70 --intro 0.3 --cola 3</t>
+          <t>python3 03-composicion/ambiente.py audio/OBRA-046_432_yu.wav audio/OBRA-046_final.wav --fondo nada --nivel-obra 0 --entrada-obra 1.5 --corte-obra 70 --intro 0.3 --cola 1</t>
         </is>
       </c>
       <c r="W47" s="4" t="inlineStr">

</xml_diff>